<commit_message>
Say plainly that six is how long one call rings, not how many calls
The assistant read "wait six rings" as "make six calls" — a fair reading, since
the sheet next to it has six numbered call columns. The rule now names what it
measures: seven calls per clinic spread over a week, and within any one of them
six rings before hanging up.

Brings the markdown instructions back in line with the two documents that are
actually handed over — it still lacked the daytime window and still forbade
calling during working hours, which the daytime baseline requires.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/obzvon-stomatologii-almaty.xlsx
+++ b/docs/obzvon-stomatologii-almaty.xlsx
@@ -205,7 +205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -219,6 +219,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -710,7 +713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -742,63 +745,63 @@
       <c r="A4" s="3" t="inlineStr"/>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>КОГДА ЗВОНИТЬ</t>
+          <t>СЕМЬ ЗВОНКОВ НА КЛИНИКУ, РАСТЯНУТЫХ НА НЕДЕЛЮ</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Раб.</t>
-        </is>
-      </c>
+      <c r="A5" s="5" t="inlineStr"/>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Вторник или среда, около 11:00. Один звонок. Это точка отсчёта: без неё вечерние цифры не с чем сравнить.</t>
+          <t>Каждая колонка в таблице — это один звонок. «1» и «2» означают два звонка в один и тот же день с интервалом десять минут.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Веч.1 / Веч.2</t>
+          <t>Раб.</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Будний вечер: 20:30 и повтор в 20:40.</t>
+          <t>Вторник или среда, около 11:00 — один звонок.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Сб.1 / Сб.2</t>
+          <t>Веч.1 / Веч.2</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Суббота: 13:00 и повтор в 13:10.</t>
+          <t>Будний вечер: первый в 20:30, второй в 20:40.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
+          <t>Сб.1 / Сб.2</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Суббота: первый в 13:00, второй в 13:10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
           <t>Вс.1 / Вс.2</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Воскресенье: 12:00 и повтор в 12:10.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="5" t="inlineStr"/>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Ждать шесть гудков. Повтор через десять минут обязателен — один неотвеченный звонок ничего не доказывает.</t>
+          <t>Воскресенье: первый в 12:00, второй в 12:10.</t>
         </is>
       </c>
     </row>
@@ -806,303 +809,319 @@
       <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="6" t="inlineStr">
         <is>
+          <t>Повтор через десять минут обязателен: один неотвеченный звонок ничего не доказывает, телефон могли просто не услышать.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>СКОЛЬКО ЖДАТЬ В ОДНОМ ЗВОНКЕ: шесть гудков, потом класть трубку. Это про длительность звонка, а не про их количество.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="5" t="inlineStr"/>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
           <t>Порядок: сначала приоритет A, потом B. Группа C — если останется время, у них вечернего окна почти нет.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="3" t="inlineStr"/>
-      <c r="B12" s="4" t="inlineStr">
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>КОДЫ</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Ч</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>ответил живой человек</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>А</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>автоответчик или голосовое сообщение</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Г</t>
+          <t>Ч</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>гудки, никто не взял трубку</t>
+          <t>ответил живой человек</t>
         </is>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>З</t>
+          <t>А</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>занято</t>
+          <t>автоответчик или голосовое сообщение</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Н</t>
+          <t>Г</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>номер недоступен или не существует</t>
+          <t>гудки, никто не взял трубку</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
+          <t>З</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>занято</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Н</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>номер недоступен или не существует</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
           <t>С</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>сбросили звонок</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="5" t="inlineStr"/>
-      <c r="B19" s="6" t="inlineStr">
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="5" t="inlineStr"/>
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Клетка подсвечивается сама: зелёным если ответили, красным если гудки.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="3" t="inlineStr"/>
-      <c r="B21" s="4" t="inlineStr">
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>ПРИМЕР ЗАПОЛНЕНИЯ</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Клиника</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Раб.</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>Веч.1</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>Веч.2</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>Сб.1</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>Сб.2</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G24" s="8" t="inlineStr">
         <is>
           <t>Вс.1</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H24" s="8" t="inlineStr">
         <is>
           <t>Вс.2</t>
         </is>
       </c>
-      <c r="I22" s="7" t="inlineStr">
+      <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Заметки</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="46" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+    <row r="25" ht="46" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>Ажар Дент</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>Ч</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
         <is>
           <t>Г</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t>Г</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>Г</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="F25" s="10" t="inlineStr">
         <is>
           <t>А</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr">
+      <c r="G25" s="10" t="inlineStr">
         <is>
           <t>Г</t>
         </is>
       </c>
-      <c r="H23" s="9" t="inlineStr">
+      <c r="H25" s="10" t="inlineStr">
         <is>
           <t>Г</t>
         </is>
       </c>
-      <c r="I23" s="8" t="inlineStr">
+      <c r="I25" s="9" t="inlineStr">
         <is>
           <t>Днём ответил администратор. Сказала, что вечером никого нет. Автоответчик в субботу: «клиника работает с 9 до 19». Перезвонили в пн 09:14.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="3" t="inlineStr"/>
-      <c r="B26" s="4" t="inlineStr">
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="3" t="inlineStr"/>
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>ЕСЛИ СНЯЛИ ТРУБКУ</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="5" t="inlineStr"/>
-      <c r="B27" s="6" t="inlineStr">
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="5" t="inlineStr"/>
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Представиться и сказать правду, без легенд: «Здравствуйте. Я провожу небольшое исследование по клиникам Алматы, буквально два вопроса, если у вас есть полминуты».</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>У вас можно записаться по телефону вечером, после закрытия?</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Кто отвечает на звонки в выходные — администратор или кто-то дежурит?</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>Сколько примерно записавшихся до вас не доходит? — самый ценный вопрос, ответ записывать целиком и своими словами.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="10" t="inlineStr"/>
-      <c r="B32" s="11" t="inlineStr">
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="11" t="inlineStr"/>
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>ЧЕГО ДЕЛАТЬ НЕЛЬЗЯ</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="12" t="inlineStr"/>
-      <c r="B33" s="13" t="inlineStr">
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="13" t="inlineStr"/>
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>Не притворяться пациентом. Ни при каких условиях.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="12" t="inlineStr"/>
-      <c r="B34" s="13" t="inlineStr">
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="13" t="inlineStr"/>
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>Не молчать в трубку. Ответили — сразу говорим.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="12" t="inlineStr"/>
-      <c r="B35" s="13" t="inlineStr">
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="13" t="inlineStr"/>
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>Ничего не предлагать и не продавать. Сейчас мы только считаем.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="12" t="inlineStr"/>
-      <c r="B36" s="13" t="inlineStr">
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="13" t="inlineStr"/>
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>Не спорить и не уговаривать. Отказались — спасибо, до свидания.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="5" t="inlineStr"/>
-      <c r="B38" s="6" t="inlineStr">
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="5" t="inlineStr"/>
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>Звонить с одного номера все дни, и с того, на который готовы ответить утром. Часть клиник перезвонит на пропущенный — записывайте дату и время в колонку «Перезвонили».</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="28" customHeight="1">
-      <c r="A40" s="14" t="inlineStr"/>
-      <c r="B40" s="15" t="inlineStr">
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="15" t="inlineStr"/>
+      <c r="B42" s="16" t="inlineStr">
         <is>
           <t>Телефоны, часы и районы взяты из 2ГИС 22 августа 2026 года. Если клиника называет другой график — впишите в заметки.</t>
         </is>
@@ -1145,2300 +1164,2300 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>Клиника</t>
         </is>
       </c>
-      <c r="C1" s="16" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>Телефон</t>
         </is>
       </c>
-      <c r="D1" s="16" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>Район</t>
         </is>
       </c>
-      <c r="E1" s="16" t="inlineStr">
+      <c r="E1" s="17" t="inlineStr">
         <is>
           <t>Часы по 2ГИС</t>
         </is>
       </c>
-      <c r="F1" s="16" t="inlineStr">
+      <c r="F1" s="17" t="inlineStr">
         <is>
           <t>Приор.</t>
         </is>
       </c>
-      <c r="G1" s="16" t="inlineStr">
+      <c r="G1" s="17" t="inlineStr">
         <is>
           <t>Раб.</t>
         </is>
       </c>
-      <c r="H1" s="16" t="inlineStr">
+      <c r="H1" s="17" t="inlineStr">
         <is>
           <t>Веч.1</t>
         </is>
       </c>
-      <c r="I1" s="16" t="inlineStr">
+      <c r="I1" s="17" t="inlineStr">
         <is>
           <t>Веч.2</t>
         </is>
       </c>
-      <c r="J1" s="16" t="inlineStr">
+      <c r="J1" s="17" t="inlineStr">
         <is>
           <t>Сб.1</t>
         </is>
       </c>
-      <c r="K1" s="16" t="inlineStr">
+      <c r="K1" s="17" t="inlineStr">
         <is>
           <t>Сб.2</t>
         </is>
       </c>
-      <c r="L1" s="16" t="inlineStr">
+      <c r="L1" s="17" t="inlineStr">
         <is>
           <t>Вс.1</t>
         </is>
       </c>
-      <c r="M1" s="16" t="inlineStr">
+      <c r="M1" s="17" t="inlineStr">
         <is>
           <t>Вс.2</t>
         </is>
       </c>
-      <c r="N1" s="16" t="inlineStr">
+      <c r="N1" s="17" t="inlineStr">
         <is>
           <t>Гудков</t>
         </is>
       </c>
-      <c r="O1" s="16" t="inlineStr">
+      <c r="O1" s="17" t="inlineStr">
         <is>
           <t>Ответов</t>
         </is>
       </c>
-      <c r="P1" s="16" t="inlineStr">
+      <c r="P1" s="17" t="inlineStr">
         <is>
           <t>Перезвонили</t>
         </is>
       </c>
-      <c r="Q1" s="16" t="inlineStr">
+      <c r="Q1" s="17" t="inlineStr">
         <is>
           <t>Заметки</t>
         </is>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="17" t="n">
+      <c r="A2" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="B2" s="19" t="inlineStr">
         <is>
           <t>Ажар Дент</t>
         </is>
       </c>
-      <c r="C2" s="19" t="inlineStr">
+      <c r="C2" s="20" t="inlineStr">
         <is>
           <t>+7 705 222 99 22</t>
         </is>
       </c>
-      <c r="D2" s="20" t="inlineStr">
+      <c r="D2" s="21" t="inlineStr">
         <is>
           <t>Жетысуский</t>
         </is>
       </c>
-      <c r="E2" s="20" t="inlineStr">
+      <c r="E2" s="21" t="inlineStr">
         <is>
           <t>09:00-19:00</t>
         </is>
       </c>
-      <c r="F2" s="21" t="inlineStr">
+      <c r="F2" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G2" s="22" t="n"/>
-      <c r="H2" s="22" t="n"/>
-      <c r="I2" s="22" t="n"/>
-      <c r="J2" s="22" t="n"/>
-      <c r="K2" s="22" t="n"/>
-      <c r="L2" s="22" t="n"/>
-      <c r="M2" s="22" t="n"/>
-      <c r="N2" s="23">
+      <c r="G2" s="23" t="n"/>
+      <c r="H2" s="23" t="n"/>
+      <c r="I2" s="23" t="n"/>
+      <c r="J2" s="23" t="n"/>
+      <c r="K2" s="23" t="n"/>
+      <c r="L2" s="23" t="n"/>
+      <c r="M2" s="23" t="n"/>
+      <c r="N2" s="24">
         <f>COUNTIF(H2:M2,"Г")</f>
         <v/>
       </c>
-      <c r="O2" s="23">
+      <c r="O2" s="24">
         <f>COUNTIF(H2:M2,"Ч")</f>
         <v/>
       </c>
-      <c r="P2" s="24" t="n"/>
-      <c r="Q2" s="25" t="n"/>
+      <c r="P2" s="25" t="n"/>
+      <c r="Q2" s="26" t="n"/>
     </row>
     <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="17" t="n">
+      <c r="A3" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>Empire dental clinic</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
         <is>
           <t>+7 778 114 76 94</t>
         </is>
       </c>
-      <c r="D3" s="20" t="inlineStr">
+      <c r="D3" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E3" s="20" t="inlineStr">
+      <c r="E3" s="21" t="inlineStr">
         <is>
           <t>10:00-20:00</t>
         </is>
       </c>
-      <c r="F3" s="21" t="inlineStr">
+      <c r="F3" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G3" s="22" t="n"/>
-      <c r="H3" s="22" t="n"/>
-      <c r="I3" s="22" t="n"/>
-      <c r="J3" s="22" t="n"/>
-      <c r="K3" s="22" t="n"/>
-      <c r="L3" s="22" t="n"/>
-      <c r="M3" s="22" t="n"/>
-      <c r="N3" s="23">
+      <c r="G3" s="23" t="n"/>
+      <c r="H3" s="23" t="n"/>
+      <c r="I3" s="23" t="n"/>
+      <c r="J3" s="23" t="n"/>
+      <c r="K3" s="23" t="n"/>
+      <c r="L3" s="23" t="n"/>
+      <c r="M3" s="23" t="n"/>
+      <c r="N3" s="24">
         <f>COUNTIF(H3:M3,"Г")</f>
         <v/>
       </c>
-      <c r="O3" s="23">
+      <c r="O3" s="24">
         <f>COUNTIF(H3:M3,"Ч")</f>
         <v/>
       </c>
-      <c r="P3" s="24" t="n"/>
-      <c r="Q3" s="25" t="n"/>
+      <c r="P3" s="25" t="n"/>
+      <c r="Q3" s="26" t="n"/>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="17" t="n">
+      <c r="A4" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>AylinDent</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>+7 707 963 30 44</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Ауэзовский</t>
         </is>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>09:00-21:00 ежедневно</t>
         </is>
       </c>
-      <c r="F4" s="21" t="inlineStr">
+      <c r="F4" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G4" s="22" t="n"/>
-      <c r="H4" s="22" t="n"/>
-      <c r="I4" s="22" t="n"/>
-      <c r="J4" s="22" t="n"/>
-      <c r="K4" s="22" t="n"/>
-      <c r="L4" s="22" t="n"/>
-      <c r="M4" s="22" t="n"/>
-      <c r="N4" s="23">
+      <c r="G4" s="23" t="n"/>
+      <c r="H4" s="23" t="n"/>
+      <c r="I4" s="23" t="n"/>
+      <c r="J4" s="23" t="n"/>
+      <c r="K4" s="23" t="n"/>
+      <c r="L4" s="23" t="n"/>
+      <c r="M4" s="23" t="n"/>
+      <c r="N4" s="24">
         <f>COUNTIF(H4:M4,"Г")</f>
         <v/>
       </c>
-      <c r="O4" s="23">
+      <c r="O4" s="24">
         <f>COUNTIF(H4:M4,"Ч")</f>
         <v/>
       </c>
-      <c r="P4" s="24" t="n"/>
-      <c r="Q4" s="25" t="n"/>
+      <c r="P4" s="25" t="n"/>
+      <c r="Q4" s="26" t="n"/>
     </row>
     <row r="5" ht="26" customHeight="1">
-      <c r="A5" s="17" t="n">
+      <c r="A5" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Light Dental Clinic</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>+7 705 333 19 99</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>Ауэзовский</t>
         </is>
       </c>
-      <c r="E5" s="20" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>09:00-21:00</t>
         </is>
       </c>
-      <c r="F5" s="21" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G5" s="22" t="n"/>
-      <c r="H5" s="22" t="n"/>
-      <c r="I5" s="22" t="n"/>
-      <c r="J5" s="22" t="n"/>
-      <c r="K5" s="22" t="n"/>
-      <c r="L5" s="22" t="n"/>
-      <c r="M5" s="22" t="n"/>
-      <c r="N5" s="23">
+      <c r="G5" s="23" t="n"/>
+      <c r="H5" s="23" t="n"/>
+      <c r="I5" s="23" t="n"/>
+      <c r="J5" s="23" t="n"/>
+      <c r="K5" s="23" t="n"/>
+      <c r="L5" s="23" t="n"/>
+      <c r="M5" s="23" t="n"/>
+      <c r="N5" s="24">
         <f>COUNTIF(H5:M5,"Г")</f>
         <v/>
       </c>
-      <c r="O5" s="23">
+      <c r="O5" s="24">
         <f>COUNTIF(H5:M5,"Ч")</f>
         <v/>
       </c>
-      <c r="P5" s="24" t="n"/>
-      <c r="Q5" s="25" t="n"/>
+      <c r="P5" s="25" t="n"/>
+      <c r="Q5" s="26" t="n"/>
     </row>
     <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="17" t="n">
+      <c r="A6" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="19" t="inlineStr">
         <is>
           <t>Kids Stom</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>+7 707 220 80 00</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>09:00-21:00 ежедневно</t>
         </is>
       </c>
-      <c r="F6" s="21" t="inlineStr">
+      <c r="F6" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G6" s="22" t="n"/>
-      <c r="H6" s="22" t="n"/>
-      <c r="I6" s="22" t="n"/>
-      <c r="J6" s="22" t="n"/>
-      <c r="K6" s="22" t="n"/>
-      <c r="L6" s="22" t="n"/>
-      <c r="M6" s="22" t="n"/>
-      <c r="N6" s="23">
+      <c r="G6" s="23" t="n"/>
+      <c r="H6" s="23" t="n"/>
+      <c r="I6" s="23" t="n"/>
+      <c r="J6" s="23" t="n"/>
+      <c r="K6" s="23" t="n"/>
+      <c r="L6" s="23" t="n"/>
+      <c r="M6" s="23" t="n"/>
+      <c r="N6" s="24">
         <f>COUNTIF(H6:M6,"Г")</f>
         <v/>
       </c>
-      <c r="O6" s="23">
+      <c r="O6" s="24">
         <f>COUNTIF(H6:M6,"Ч")</f>
         <v/>
       </c>
-      <c r="P6" s="24" t="n"/>
-      <c r="Q6" s="25" t="n"/>
+      <c r="P6" s="25" t="n"/>
+      <c r="Q6" s="26" t="n"/>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="17" t="n">
+      <c r="A7" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Sara clinic</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>+7 707 675 70 00</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>Ауэзовский</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>09:00-21:00 ежедневно</t>
         </is>
       </c>
-      <c r="F7" s="21" t="inlineStr">
+      <c r="F7" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G7" s="22" t="n"/>
-      <c r="H7" s="22" t="n"/>
-      <c r="I7" s="22" t="n"/>
-      <c r="J7" s="22" t="n"/>
-      <c r="K7" s="22" t="n"/>
-      <c r="L7" s="22" t="n"/>
-      <c r="M7" s="22" t="n"/>
-      <c r="N7" s="23">
+      <c r="G7" s="23" t="n"/>
+      <c r="H7" s="23" t="n"/>
+      <c r="I7" s="23" t="n"/>
+      <c r="J7" s="23" t="n"/>
+      <c r="K7" s="23" t="n"/>
+      <c r="L7" s="23" t="n"/>
+      <c r="M7" s="23" t="n"/>
+      <c r="N7" s="24">
         <f>COUNTIF(H7:M7,"Г")</f>
         <v/>
       </c>
-      <c r="O7" s="23">
+      <c r="O7" s="24">
         <f>COUNTIF(H7:M7,"Ч")</f>
         <v/>
       </c>
-      <c r="P7" s="24" t="n"/>
-      <c r="Q7" s="25" t="n"/>
+      <c r="P7" s="25" t="n"/>
+      <c r="Q7" s="26" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="17" t="n">
+      <c r="A8" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="19" t="inlineStr">
         <is>
           <t>DS Stomatology</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>+7 771 267 61 27</t>
         </is>
       </c>
-      <c r="D8" s="20" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>Талгарский</t>
         </is>
       </c>
-      <c r="E8" s="20" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>09:00-21:00 ежедневно</t>
         </is>
       </c>
-      <c r="F8" s="21" t="inlineStr">
+      <c r="F8" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G8" s="22" t="n"/>
-      <c r="H8" s="22" t="n"/>
-      <c r="I8" s="22" t="n"/>
-      <c r="J8" s="22" t="n"/>
-      <c r="K8" s="22" t="n"/>
-      <c r="L8" s="22" t="n"/>
-      <c r="M8" s="22" t="n"/>
-      <c r="N8" s="23">
+      <c r="G8" s="23" t="n"/>
+      <c r="H8" s="23" t="n"/>
+      <c r="I8" s="23" t="n"/>
+      <c r="J8" s="23" t="n"/>
+      <c r="K8" s="23" t="n"/>
+      <c r="L8" s="23" t="n"/>
+      <c r="M8" s="23" t="n"/>
+      <c r="N8" s="24">
         <f>COUNTIF(H8:M8,"Г")</f>
         <v/>
       </c>
-      <c r="O8" s="23">
+      <c r="O8" s="24">
         <f>COUNTIF(H8:M8,"Ч")</f>
         <v/>
       </c>
-      <c r="P8" s="24" t="n"/>
-      <c r="Q8" s="25" t="n"/>
+      <c r="P8" s="25" t="n"/>
+      <c r="Q8" s="26" t="n"/>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="17" t="n">
+      <c r="A9" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Ever Smile</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>+7 747 900 30 09</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>Алмалинский</t>
         </is>
       </c>
-      <c r="E9" s="20" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>10:00-22:00 обед 12:00-14:30</t>
         </is>
       </c>
-      <c r="F9" s="21" t="inlineStr">
+      <c r="F9" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G9" s="22" t="n"/>
-      <c r="H9" s="22" t="n"/>
-      <c r="I9" s="22" t="n"/>
-      <c r="J9" s="22" t="n"/>
-      <c r="K9" s="22" t="n"/>
-      <c r="L9" s="22" t="n"/>
-      <c r="M9" s="22" t="n"/>
-      <c r="N9" s="23">
+      <c r="G9" s="23" t="n"/>
+      <c r="H9" s="23" t="n"/>
+      <c r="I9" s="23" t="n"/>
+      <c r="J9" s="23" t="n"/>
+      <c r="K9" s="23" t="n"/>
+      <c r="L9" s="23" t="n"/>
+      <c r="M9" s="23" t="n"/>
+      <c r="N9" s="24">
         <f>COUNTIF(H9:M9,"Г")</f>
         <v/>
       </c>
-      <c r="O9" s="23">
+      <c r="O9" s="24">
         <f>COUNTIF(H9:M9,"Ч")</f>
         <v/>
       </c>
-      <c r="P9" s="24" t="n"/>
-      <c r="Q9" s="25" t="n"/>
+      <c r="P9" s="25" t="n"/>
+      <c r="Q9" s="26" t="n"/>
     </row>
     <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="17" t="n">
+      <c r="A10" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>Top Smile</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>+7 747 085 70 71</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E10" s="20" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>10:00-22:00 ежедневно по записи</t>
         </is>
       </c>
-      <c r="F10" s="21" t="inlineStr">
+      <c r="F10" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G10" s="22" t="n"/>
-      <c r="H10" s="22" t="n"/>
-      <c r="I10" s="22" t="n"/>
-      <c r="J10" s="22" t="n"/>
-      <c r="K10" s="22" t="n"/>
-      <c r="L10" s="22" t="n"/>
-      <c r="M10" s="22" t="n"/>
-      <c r="N10" s="23">
+      <c r="G10" s="23" t="n"/>
+      <c r="H10" s="23" t="n"/>
+      <c r="I10" s="23" t="n"/>
+      <c r="J10" s="23" t="n"/>
+      <c r="K10" s="23" t="n"/>
+      <c r="L10" s="23" t="n"/>
+      <c r="M10" s="23" t="n"/>
+      <c r="N10" s="24">
         <f>COUNTIF(H10:M10,"Г")</f>
         <v/>
       </c>
-      <c r="O10" s="23">
+      <c r="O10" s="24">
         <f>COUNTIF(H10:M10,"Ч")</f>
         <v/>
       </c>
-      <c r="P10" s="24" t="n"/>
-      <c r="Q10" s="25" t="n"/>
+      <c r="P10" s="25" t="n"/>
+      <c r="Q10" s="26" t="n"/>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="17" t="n">
+      <c r="A11" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="18" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>Dobro Dent</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>+7 775 030 09 99</t>
         </is>
       </c>
-      <c r="D11" s="20" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E11" s="20" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>09:00-22:00 ежедневно</t>
         </is>
       </c>
-      <c r="F11" s="21" t="inlineStr">
+      <c r="F11" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G11" s="22" t="n"/>
-      <c r="H11" s="22" t="n"/>
-      <c r="I11" s="22" t="n"/>
-      <c r="J11" s="22" t="n"/>
-      <c r="K11" s="22" t="n"/>
-      <c r="L11" s="22" t="n"/>
-      <c r="M11" s="22" t="n"/>
-      <c r="N11" s="23">
+      <c r="G11" s="23" t="n"/>
+      <c r="H11" s="23" t="n"/>
+      <c r="I11" s="23" t="n"/>
+      <c r="J11" s="23" t="n"/>
+      <c r="K11" s="23" t="n"/>
+      <c r="L11" s="23" t="n"/>
+      <c r="M11" s="23" t="n"/>
+      <c r="N11" s="24">
         <f>COUNTIF(H11:M11,"Г")</f>
         <v/>
       </c>
-      <c r="O11" s="23">
+      <c r="O11" s="24">
         <f>COUNTIF(H11:M11,"Ч")</f>
         <v/>
       </c>
-      <c r="P11" s="24" t="n"/>
-      <c r="Q11" s="25" t="n"/>
+      <c r="P11" s="25" t="n"/>
+      <c r="Q11" s="26" t="n"/>
     </row>
     <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="17" t="n">
+      <c r="A12" s="18" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>Doctor Dent</t>
         </is>
       </c>
-      <c r="C12" s="19" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>+7 705 170 78 59</t>
         </is>
       </c>
-      <c r="D12" s="20" t="inlineStr">
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E12" s="20" t="inlineStr">
+      <c r="E12" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F12" s="17" t="inlineStr">
+      <c r="F12" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G12" s="22" t="n"/>
-      <c r="H12" s="22" t="n"/>
-      <c r="I12" s="22" t="n"/>
-      <c r="J12" s="22" t="n"/>
-      <c r="K12" s="22" t="n"/>
-      <c r="L12" s="22" t="n"/>
-      <c r="M12" s="22" t="n"/>
-      <c r="N12" s="23">
+      <c r="G12" s="23" t="n"/>
+      <c r="H12" s="23" t="n"/>
+      <c r="I12" s="23" t="n"/>
+      <c r="J12" s="23" t="n"/>
+      <c r="K12" s="23" t="n"/>
+      <c r="L12" s="23" t="n"/>
+      <c r="M12" s="23" t="n"/>
+      <c r="N12" s="24">
         <f>COUNTIF(H12:M12,"Г")</f>
         <v/>
       </c>
-      <c r="O12" s="23">
+      <c r="O12" s="24">
         <f>COUNTIF(H12:M12,"Ч")</f>
         <v/>
       </c>
-      <c r="P12" s="24" t="n"/>
-      <c r="Q12" s="25" t="n"/>
+      <c r="P12" s="25" t="n"/>
+      <c r="Q12" s="26" t="n"/>
     </row>
     <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="17" t="n">
+      <c r="A13" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="18" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>Dr. Baratov</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>+7 707 189 36 45</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
+      <c r="D13" s="21" t="inlineStr">
         <is>
           <t>Алмалинский</t>
         </is>
       </c>
-      <c r="E13" s="20" t="inlineStr">
+      <c r="E13" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F13" s="17" t="inlineStr">
+      <c r="F13" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G13" s="22" t="n"/>
-      <c r="H13" s="22" t="n"/>
-      <c r="I13" s="22" t="n"/>
-      <c r="J13" s="22" t="n"/>
-      <c r="K13" s="22" t="n"/>
-      <c r="L13" s="22" t="n"/>
-      <c r="M13" s="22" t="n"/>
-      <c r="N13" s="23">
+      <c r="G13" s="23" t="n"/>
+      <c r="H13" s="23" t="n"/>
+      <c r="I13" s="23" t="n"/>
+      <c r="J13" s="23" t="n"/>
+      <c r="K13" s="23" t="n"/>
+      <c r="L13" s="23" t="n"/>
+      <c r="M13" s="23" t="n"/>
+      <c r="N13" s="24">
         <f>COUNTIF(H13:M13,"Г")</f>
         <v/>
       </c>
-      <c r="O13" s="23">
+      <c r="O13" s="24">
         <f>COUNTIF(H13:M13,"Ч")</f>
         <v/>
       </c>
-      <c r="P13" s="24" t="n"/>
-      <c r="Q13" s="25" t="n"/>
+      <c r="P13" s="25" t="n"/>
+      <c r="Q13" s="26" t="n"/>
     </row>
     <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="17" t="n">
+      <c r="A14" s="18" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>Dr. Park</t>
         </is>
       </c>
-      <c r="C14" s="19" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>+7 707 909 78 76</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
+      <c r="D14" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E14" s="20" t="inlineStr">
+      <c r="E14" s="21" t="inlineStr">
         <is>
           <t>открывается в 09:00</t>
         </is>
       </c>
-      <c r="F14" s="17" t="inlineStr">
+      <c r="F14" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G14" s="22" t="n"/>
-      <c r="H14" s="22" t="n"/>
-      <c r="I14" s="22" t="n"/>
-      <c r="J14" s="22" t="n"/>
-      <c r="K14" s="22" t="n"/>
-      <c r="L14" s="22" t="n"/>
-      <c r="M14" s="22" t="n"/>
-      <c r="N14" s="23">
+      <c r="G14" s="23" t="n"/>
+      <c r="H14" s="23" t="n"/>
+      <c r="I14" s="23" t="n"/>
+      <c r="J14" s="23" t="n"/>
+      <c r="K14" s="23" t="n"/>
+      <c r="L14" s="23" t="n"/>
+      <c r="M14" s="23" t="n"/>
+      <c r="N14" s="24">
         <f>COUNTIF(H14:M14,"Г")</f>
         <v/>
       </c>
-      <c r="O14" s="23">
+      <c r="O14" s="24">
         <f>COUNTIF(H14:M14,"Ч")</f>
         <v/>
       </c>
-      <c r="P14" s="24" t="n"/>
-      <c r="Q14" s="25" t="n"/>
+      <c r="P14" s="25" t="n"/>
+      <c r="Q14" s="26" t="n"/>
     </row>
     <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="17" t="n">
+      <c r="A15" s="18" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="18" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>Никамед</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
         <is>
           <t>+7 727 973 55 53</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
+      <c r="D15" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E15" s="20" t="inlineStr">
+      <c r="E15" s="21" t="inlineStr">
         <is>
           <t>открывается в 08:00</t>
         </is>
       </c>
-      <c r="F15" s="17" t="inlineStr">
+      <c r="F15" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G15" s="22" t="n"/>
-      <c r="H15" s="22" t="n"/>
-      <c r="I15" s="22" t="n"/>
-      <c r="J15" s="22" t="n"/>
-      <c r="K15" s="22" t="n"/>
-      <c r="L15" s="22" t="n"/>
-      <c r="M15" s="22" t="n"/>
-      <c r="N15" s="23">
+      <c r="G15" s="23" t="n"/>
+      <c r="H15" s="23" t="n"/>
+      <c r="I15" s="23" t="n"/>
+      <c r="J15" s="23" t="n"/>
+      <c r="K15" s="23" t="n"/>
+      <c r="L15" s="23" t="n"/>
+      <c r="M15" s="23" t="n"/>
+      <c r="N15" s="24">
         <f>COUNTIF(H15:M15,"Г")</f>
         <v/>
       </c>
-      <c r="O15" s="23">
+      <c r="O15" s="24">
         <f>COUNTIF(H15:M15,"Ч")</f>
         <v/>
       </c>
-      <c r="P15" s="24" t="n"/>
-      <c r="Q15" s="25" t="n"/>
+      <c r="P15" s="25" t="n"/>
+      <c r="Q15" s="26" t="n"/>
     </row>
     <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="17" t="n">
+      <c r="A16" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="18" t="inlineStr">
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>Diamond Dent</t>
         </is>
       </c>
-      <c r="C16" s="19" t="inlineStr">
+      <c r="C16" s="20" t="inlineStr">
         <is>
           <t>+7 771 275 39 49</t>
         </is>
       </c>
-      <c r="D16" s="20" t="inlineStr">
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>Ауэзовский</t>
         </is>
       </c>
-      <c r="E16" s="20" t="inlineStr">
+      <c r="E16" s="21" t="inlineStr">
         <is>
           <t>открывается в 09:00</t>
         </is>
       </c>
-      <c r="F16" s="17" t="inlineStr">
+      <c r="F16" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G16" s="22" t="n"/>
-      <c r="H16" s="22" t="n"/>
-      <c r="I16" s="22" t="n"/>
-      <c r="J16" s="22" t="n"/>
-      <c r="K16" s="22" t="n"/>
-      <c r="L16" s="22" t="n"/>
-      <c r="M16" s="22" t="n"/>
-      <c r="N16" s="23">
+      <c r="G16" s="23" t="n"/>
+      <c r="H16" s="23" t="n"/>
+      <c r="I16" s="23" t="n"/>
+      <c r="J16" s="23" t="n"/>
+      <c r="K16" s="23" t="n"/>
+      <c r="L16" s="23" t="n"/>
+      <c r="M16" s="23" t="n"/>
+      <c r="N16" s="24">
         <f>COUNTIF(H16:M16,"Г")</f>
         <v/>
       </c>
-      <c r="O16" s="23">
+      <c r="O16" s="24">
         <f>COUNTIF(H16:M16,"Ч")</f>
         <v/>
       </c>
-      <c r="P16" s="24" t="n"/>
-      <c r="Q16" s="25" t="n"/>
+      <c r="P16" s="25" t="n"/>
+      <c r="Q16" s="26" t="n"/>
     </row>
     <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="17" t="n">
+      <c r="A17" s="18" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="18" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>Mirai Dental Clinic</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
         <is>
           <t>+7 700 302 22 30</t>
         </is>
       </c>
-      <c r="D17" s="20" t="inlineStr">
+      <c r="D17" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E17" s="20" t="inlineStr">
+      <c r="E17" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F17" s="17" t="inlineStr">
+      <c r="F17" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G17" s="22" t="n"/>
-      <c r="H17" s="22" t="n"/>
-      <c r="I17" s="22" t="n"/>
-      <c r="J17" s="22" t="n"/>
-      <c r="K17" s="22" t="n"/>
-      <c r="L17" s="22" t="n"/>
-      <c r="M17" s="22" t="n"/>
-      <c r="N17" s="23">
+      <c r="G17" s="23" t="n"/>
+      <c r="H17" s="23" t="n"/>
+      <c r="I17" s="23" t="n"/>
+      <c r="J17" s="23" t="n"/>
+      <c r="K17" s="23" t="n"/>
+      <c r="L17" s="23" t="n"/>
+      <c r="M17" s="23" t="n"/>
+      <c r="N17" s="24">
         <f>COUNTIF(H17:M17,"Г")</f>
         <v/>
       </c>
-      <c r="O17" s="23">
+      <c r="O17" s="24">
         <f>COUNTIF(H17:M17,"Ч")</f>
         <v/>
       </c>
-      <c r="P17" s="24" t="n"/>
-      <c r="Q17" s="25" t="n"/>
+      <c r="P17" s="25" t="n"/>
+      <c r="Q17" s="26" t="n"/>
     </row>
     <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="17" t="n">
+      <c r="A18" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="18" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>Senim Dental Clinic</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>+7 701 408 84 44</t>
         </is>
       </c>
-      <c r="D18" s="20" t="inlineStr">
+      <c r="D18" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E18" s="20" t="inlineStr">
+      <c r="E18" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F18" s="17" t="inlineStr">
+      <c r="F18" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G18" s="22" t="n"/>
-      <c r="H18" s="22" t="n"/>
-      <c r="I18" s="22" t="n"/>
-      <c r="J18" s="22" t="n"/>
-      <c r="K18" s="22" t="n"/>
-      <c r="L18" s="22" t="n"/>
-      <c r="M18" s="22" t="n"/>
-      <c r="N18" s="23">
+      <c r="G18" s="23" t="n"/>
+      <c r="H18" s="23" t="n"/>
+      <c r="I18" s="23" t="n"/>
+      <c r="J18" s="23" t="n"/>
+      <c r="K18" s="23" t="n"/>
+      <c r="L18" s="23" t="n"/>
+      <c r="M18" s="23" t="n"/>
+      <c r="N18" s="24">
         <f>COUNTIF(H18:M18,"Г")</f>
         <v/>
       </c>
-      <c r="O18" s="23">
+      <c r="O18" s="24">
         <f>COUNTIF(H18:M18,"Ч")</f>
         <v/>
       </c>
-      <c r="P18" s="24" t="n"/>
-      <c r="Q18" s="25" t="n"/>
+      <c r="P18" s="25" t="n"/>
+      <c r="Q18" s="26" t="n"/>
     </row>
     <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="17" t="n">
+      <c r="A19" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="18" t="inlineStr">
+      <c r="B19" s="19" t="inlineStr">
         <is>
           <t>Клиника доктора Мирзоева</t>
         </is>
       </c>
-      <c r="C19" s="19" t="inlineStr">
+      <c r="C19" s="20" t="inlineStr">
         <is>
           <t>+7 701 758 55 21</t>
         </is>
       </c>
-      <c r="D19" s="20" t="inlineStr">
+      <c r="D19" s="21" t="inlineStr">
         <is>
           <t>Алмалинский</t>
         </is>
       </c>
-      <c r="E19" s="20" t="inlineStr">
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>открывается в 10:00 по записи</t>
         </is>
       </c>
-      <c r="F19" s="17" t="inlineStr">
+      <c r="F19" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G19" s="22" t="n"/>
-      <c r="H19" s="22" t="n"/>
-      <c r="I19" s="22" t="n"/>
-      <c r="J19" s="22" t="n"/>
-      <c r="K19" s="22" t="n"/>
-      <c r="L19" s="22" t="n"/>
-      <c r="M19" s="22" t="n"/>
-      <c r="N19" s="23">
+      <c r="G19" s="23" t="n"/>
+      <c r="H19" s="23" t="n"/>
+      <c r="I19" s="23" t="n"/>
+      <c r="J19" s="23" t="n"/>
+      <c r="K19" s="23" t="n"/>
+      <c r="L19" s="23" t="n"/>
+      <c r="M19" s="23" t="n"/>
+      <c r="N19" s="24">
         <f>COUNTIF(H19:M19,"Г")</f>
         <v/>
       </c>
-      <c r="O19" s="23">
+      <c r="O19" s="24">
         <f>COUNTIF(H19:M19,"Ч")</f>
         <v/>
       </c>
-      <c r="P19" s="24" t="n"/>
-      <c r="Q19" s="25" t="n"/>
+      <c r="P19" s="25" t="n"/>
+      <c r="Q19" s="26" t="n"/>
     </row>
     <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="17" t="n">
+      <c r="A20" s="18" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>MC Dent</t>
         </is>
       </c>
-      <c r="C20" s="19" t="inlineStr">
+      <c r="C20" s="20" t="inlineStr">
         <is>
           <t>+7 702 366 59 74</t>
         </is>
       </c>
-      <c r="D20" s="20" t="inlineStr">
+      <c r="D20" s="21" t="inlineStr">
         <is>
           <t>Алмалинский</t>
         </is>
       </c>
-      <c r="E20" s="20" t="inlineStr">
+      <c r="E20" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F20" s="17" t="inlineStr">
+      <c r="F20" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G20" s="22" t="n"/>
-      <c r="H20" s="22" t="n"/>
-      <c r="I20" s="22" t="n"/>
-      <c r="J20" s="22" t="n"/>
-      <c r="K20" s="22" t="n"/>
-      <c r="L20" s="22" t="n"/>
-      <c r="M20" s="22" t="n"/>
-      <c r="N20" s="23">
+      <c r="G20" s="23" t="n"/>
+      <c r="H20" s="23" t="n"/>
+      <c r="I20" s="23" t="n"/>
+      <c r="J20" s="23" t="n"/>
+      <c r="K20" s="23" t="n"/>
+      <c r="L20" s="23" t="n"/>
+      <c r="M20" s="23" t="n"/>
+      <c r="N20" s="24">
         <f>COUNTIF(H20:M20,"Г")</f>
         <v/>
       </c>
-      <c r="O20" s="23">
+      <c r="O20" s="24">
         <f>COUNTIF(H20:M20,"Ч")</f>
         <v/>
       </c>
-      <c r="P20" s="24" t="n"/>
-      <c r="Q20" s="25" t="n"/>
+      <c r="P20" s="25" t="n"/>
+      <c r="Q20" s="26" t="n"/>
     </row>
     <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="17" t="n">
+      <c r="A21" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>Elit Stom (Манаса 19)</t>
         </is>
       </c>
-      <c r="C21" s="19" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>+7 700 818 90 60</t>
         </is>
       </c>
-      <c r="D21" s="20" t="inlineStr">
+      <c r="D21" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E21" s="20" t="inlineStr">
+      <c r="E21" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F21" s="17" t="inlineStr">
+      <c r="F21" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G21" s="22" t="n"/>
-      <c r="H21" s="22" t="n"/>
-      <c r="I21" s="22" t="n"/>
-      <c r="J21" s="22" t="n"/>
-      <c r="K21" s="22" t="n"/>
-      <c r="L21" s="22" t="n"/>
-      <c r="M21" s="22" t="n"/>
-      <c r="N21" s="23">
+      <c r="G21" s="23" t="n"/>
+      <c r="H21" s="23" t="n"/>
+      <c r="I21" s="23" t="n"/>
+      <c r="J21" s="23" t="n"/>
+      <c r="K21" s="23" t="n"/>
+      <c r="L21" s="23" t="n"/>
+      <c r="M21" s="23" t="n"/>
+      <c r="N21" s="24">
         <f>COUNTIF(H21:M21,"Г")</f>
         <v/>
       </c>
-      <c r="O21" s="23">
+      <c r="O21" s="24">
         <f>COUNTIF(H21:M21,"Ч")</f>
         <v/>
       </c>
-      <c r="P21" s="24" t="n"/>
-      <c r="Q21" s="25" t="n"/>
+      <c r="P21" s="25" t="n"/>
+      <c r="Q21" s="26" t="n"/>
     </row>
     <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="17" t="n">
+      <c r="A22" s="18" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="18" t="inlineStr">
+      <c r="B22" s="19" t="inlineStr">
         <is>
           <t>Family Dent Dr. Kapanov</t>
         </is>
       </c>
-      <c r="C22" s="19" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
         <is>
           <t>+7 771 645 53 96</t>
         </is>
       </c>
-      <c r="D22" s="20" t="inlineStr">
+      <c r="D22" s="21" t="inlineStr">
         <is>
           <t>Ауэзовский</t>
         </is>
       </c>
-      <c r="E22" s="20" t="inlineStr">
+      <c r="E22" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F22" s="17" t="inlineStr">
+      <c r="F22" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G22" s="22" t="n"/>
-      <c r="H22" s="22" t="n"/>
-      <c r="I22" s="22" t="n"/>
-      <c r="J22" s="22" t="n"/>
-      <c r="K22" s="22" t="n"/>
-      <c r="L22" s="22" t="n"/>
-      <c r="M22" s="22" t="n"/>
-      <c r="N22" s="23">
+      <c r="G22" s="23" t="n"/>
+      <c r="H22" s="23" t="n"/>
+      <c r="I22" s="23" t="n"/>
+      <c r="J22" s="23" t="n"/>
+      <c r="K22" s="23" t="n"/>
+      <c r="L22" s="23" t="n"/>
+      <c r="M22" s="23" t="n"/>
+      <c r="N22" s="24">
         <f>COUNTIF(H22:M22,"Г")</f>
         <v/>
       </c>
-      <c r="O22" s="23">
+      <c r="O22" s="24">
         <f>COUNTIF(H22:M22,"Ч")</f>
         <v/>
       </c>
-      <c r="P22" s="24" t="n"/>
-      <c r="Q22" s="25" t="n"/>
+      <c r="P22" s="25" t="n"/>
+      <c r="Q22" s="26" t="n"/>
     </row>
     <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="17" t="n">
+      <c r="A23" s="18" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="18" t="inlineStr">
+      <c r="B23" s="19" t="inlineStr">
         <is>
           <t>Стоматология Аброра Исмаиловича</t>
         </is>
       </c>
-      <c r="C23" s="19" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
         <is>
           <t>+7 775 370 12 13</t>
         </is>
       </c>
-      <c r="D23" s="20" t="inlineStr">
+      <c r="D23" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E23" s="20" t="inlineStr">
+      <c r="E23" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F23" s="17" t="inlineStr">
+      <c r="F23" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G23" s="22" t="n"/>
-      <c r="H23" s="22" t="n"/>
-      <c r="I23" s="22" t="n"/>
-      <c r="J23" s="22" t="n"/>
-      <c r="K23" s="22" t="n"/>
-      <c r="L23" s="22" t="n"/>
-      <c r="M23" s="22" t="n"/>
-      <c r="N23" s="23">
+      <c r="G23" s="23" t="n"/>
+      <c r="H23" s="23" t="n"/>
+      <c r="I23" s="23" t="n"/>
+      <c r="J23" s="23" t="n"/>
+      <c r="K23" s="23" t="n"/>
+      <c r="L23" s="23" t="n"/>
+      <c r="M23" s="23" t="n"/>
+      <c r="N23" s="24">
         <f>COUNTIF(H23:M23,"Г")</f>
         <v/>
       </c>
-      <c r="O23" s="23">
+      <c r="O23" s="24">
         <f>COUNTIF(H23:M23,"Ч")</f>
         <v/>
       </c>
-      <c r="P23" s="24" t="n"/>
-      <c r="Q23" s="25" t="n"/>
+      <c r="P23" s="25" t="n"/>
+      <c r="Q23" s="26" t="n"/>
     </row>
     <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="17" t="n">
+      <c r="A24" s="18" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B24" s="19" t="inlineStr">
         <is>
           <t>Smilex Dental Center</t>
         </is>
       </c>
-      <c r="C24" s="19" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
         <is>
           <t>+7 747 897 32 07</t>
         </is>
       </c>
-      <c r="D24" s="20" t="inlineStr">
+      <c r="D24" s="21" t="inlineStr">
         <is>
           <t>Алмалинский</t>
         </is>
       </c>
-      <c r="E24" s="20" t="inlineStr">
+      <c r="E24" s="21" t="inlineStr">
         <is>
           <t>открывается в 09:30</t>
         </is>
       </c>
-      <c r="F24" s="17" t="inlineStr">
+      <c r="F24" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G24" s="22" t="n"/>
-      <c r="H24" s="22" t="n"/>
-      <c r="I24" s="22" t="n"/>
-      <c r="J24" s="22" t="n"/>
-      <c r="K24" s="22" t="n"/>
-      <c r="L24" s="22" t="n"/>
-      <c r="M24" s="22" t="n"/>
-      <c r="N24" s="23">
+      <c r="G24" s="23" t="n"/>
+      <c r="H24" s="23" t="n"/>
+      <c r="I24" s="23" t="n"/>
+      <c r="J24" s="23" t="n"/>
+      <c r="K24" s="23" t="n"/>
+      <c r="L24" s="23" t="n"/>
+      <c r="M24" s="23" t="n"/>
+      <c r="N24" s="24">
         <f>COUNTIF(H24:M24,"Г")</f>
         <v/>
       </c>
-      <c r="O24" s="23">
+      <c r="O24" s="24">
         <f>COUNTIF(H24:M24,"Ч")</f>
         <v/>
       </c>
-      <c r="P24" s="24" t="n"/>
-      <c r="Q24" s="25" t="n"/>
+      <c r="P24" s="25" t="n"/>
+      <c r="Q24" s="26" t="n"/>
     </row>
     <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="17" t="n">
+      <c r="A25" s="18" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="18" t="inlineStr">
+      <c r="B25" s="19" t="inlineStr">
         <is>
           <t>Altyn Dent</t>
         </is>
       </c>
-      <c r="C25" s="19" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
         <is>
           <t>+7 747 920 75 71</t>
         </is>
       </c>
-      <c r="D25" s="20" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>Алмалинский</t>
         </is>
       </c>
-      <c r="E25" s="20" t="inlineStr">
+      <c r="E25" s="21" t="inlineStr">
         <is>
           <t>открывается в 09:00</t>
         </is>
       </c>
-      <c r="F25" s="17" t="inlineStr">
+      <c r="F25" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G25" s="22" t="n"/>
-      <c r="H25" s="22" t="n"/>
-      <c r="I25" s="22" t="n"/>
-      <c r="J25" s="22" t="n"/>
-      <c r="K25" s="22" t="n"/>
-      <c r="L25" s="22" t="n"/>
-      <c r="M25" s="22" t="n"/>
-      <c r="N25" s="23">
+      <c r="G25" s="23" t="n"/>
+      <c r="H25" s="23" t="n"/>
+      <c r="I25" s="23" t="n"/>
+      <c r="J25" s="23" t="n"/>
+      <c r="K25" s="23" t="n"/>
+      <c r="L25" s="23" t="n"/>
+      <c r="M25" s="23" t="n"/>
+      <c r="N25" s="24">
         <f>COUNTIF(H25:M25,"Г")</f>
         <v/>
       </c>
-      <c r="O25" s="23">
+      <c r="O25" s="24">
         <f>COUNTIF(H25:M25,"Ч")</f>
         <v/>
       </c>
-      <c r="P25" s="24" t="n"/>
-      <c r="Q25" s="25" t="n"/>
+      <c r="P25" s="25" t="n"/>
+      <c r="Q25" s="26" t="n"/>
     </row>
     <row r="26" ht="26" customHeight="1">
-      <c r="A26" s="17" t="n">
+      <c r="A26" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="18" t="inlineStr">
+      <c r="B26" s="19" t="inlineStr">
         <is>
           <t>Azu Dental Clinic</t>
         </is>
       </c>
-      <c r="C26" s="19" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
         <is>
           <t>+7 708 002 22 02</t>
         </is>
       </c>
-      <c r="D26" s="20" t="inlineStr">
+      <c r="D26" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E26" s="20" t="inlineStr">
+      <c r="E26" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F26" s="17" t="inlineStr">
+      <c r="F26" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G26" s="22" t="n"/>
-      <c r="H26" s="22" t="n"/>
-      <c r="I26" s="22" t="n"/>
-      <c r="J26" s="22" t="n"/>
-      <c r="K26" s="22" t="n"/>
-      <c r="L26" s="22" t="n"/>
-      <c r="M26" s="22" t="n"/>
-      <c r="N26" s="23">
+      <c r="G26" s="23" t="n"/>
+      <c r="H26" s="23" t="n"/>
+      <c r="I26" s="23" t="n"/>
+      <c r="J26" s="23" t="n"/>
+      <c r="K26" s="23" t="n"/>
+      <c r="L26" s="23" t="n"/>
+      <c r="M26" s="23" t="n"/>
+      <c r="N26" s="24">
         <f>COUNTIF(H26:M26,"Г")</f>
         <v/>
       </c>
-      <c r="O26" s="23">
+      <c r="O26" s="24">
         <f>COUNTIF(H26:M26,"Ч")</f>
         <v/>
       </c>
-      <c r="P26" s="24" t="n"/>
-      <c r="Q26" s="25" t="n"/>
+      <c r="P26" s="25" t="n"/>
+      <c r="Q26" s="26" t="n"/>
     </row>
     <row r="27" ht="26" customHeight="1">
-      <c r="A27" s="17" t="n">
+      <c r="A27" s="18" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="18" t="inlineStr">
+      <c r="B27" s="19" t="inlineStr">
         <is>
           <t>Dental Planet</t>
         </is>
       </c>
-      <c r="C27" s="19" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
         <is>
           <t>+7 705 888 38 15</t>
         </is>
       </c>
-      <c r="D27" s="20" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>Алмалинский</t>
         </is>
       </c>
-      <c r="E27" s="20" t="inlineStr">
+      <c r="E27" s="21" t="inlineStr">
         <is>
           <t>открывается в 08:00</t>
         </is>
       </c>
-      <c r="F27" s="17" t="inlineStr">
+      <c r="F27" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G27" s="22" t="n"/>
-      <c r="H27" s="22" t="n"/>
-      <c r="I27" s="22" t="n"/>
-      <c r="J27" s="22" t="n"/>
-      <c r="K27" s="22" t="n"/>
-      <c r="L27" s="22" t="n"/>
-      <c r="M27" s="22" t="n"/>
-      <c r="N27" s="23">
+      <c r="G27" s="23" t="n"/>
+      <c r="H27" s="23" t="n"/>
+      <c r="I27" s="23" t="n"/>
+      <c r="J27" s="23" t="n"/>
+      <c r="K27" s="23" t="n"/>
+      <c r="L27" s="23" t="n"/>
+      <c r="M27" s="23" t="n"/>
+      <c r="N27" s="24">
         <f>COUNTIF(H27:M27,"Г")</f>
         <v/>
       </c>
-      <c r="O27" s="23">
+      <c r="O27" s="24">
         <f>COUNTIF(H27:M27,"Ч")</f>
         <v/>
       </c>
-      <c r="P27" s="24" t="n"/>
-      <c r="Q27" s="25" t="n"/>
+      <c r="P27" s="25" t="n"/>
+      <c r="Q27" s="26" t="n"/>
     </row>
     <row r="28" ht="26" customHeight="1">
-      <c r="A28" s="17" t="n">
+      <c r="A28" s="18" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="18" t="inlineStr">
+      <c r="B28" s="19" t="inlineStr">
         <is>
           <t>Estetik Dental Clinic</t>
         </is>
       </c>
-      <c r="C28" s="19" t="inlineStr">
+      <c r="C28" s="20" t="inlineStr">
         <is>
           <t>+7 707 530 00 54</t>
         </is>
       </c>
-      <c r="D28" s="20" t="inlineStr">
+      <c r="D28" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E28" s="20" t="inlineStr">
+      <c r="E28" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F28" s="17" t="inlineStr">
+      <c r="F28" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G28" s="22" t="n"/>
-      <c r="H28" s="22" t="n"/>
-      <c r="I28" s="22" t="n"/>
-      <c r="J28" s="22" t="n"/>
-      <c r="K28" s="22" t="n"/>
-      <c r="L28" s="22" t="n"/>
-      <c r="M28" s="22" t="n"/>
-      <c r="N28" s="23">
+      <c r="G28" s="23" t="n"/>
+      <c r="H28" s="23" t="n"/>
+      <c r="I28" s="23" t="n"/>
+      <c r="J28" s="23" t="n"/>
+      <c r="K28" s="23" t="n"/>
+      <c r="L28" s="23" t="n"/>
+      <c r="M28" s="23" t="n"/>
+      <c r="N28" s="24">
         <f>COUNTIF(H28:M28,"Г")</f>
         <v/>
       </c>
-      <c r="O28" s="23">
+      <c r="O28" s="24">
         <f>COUNTIF(H28:M28,"Ч")</f>
         <v/>
       </c>
-      <c r="P28" s="24" t="n"/>
-      <c r="Q28" s="25" t="n"/>
+      <c r="P28" s="25" t="n"/>
+      <c r="Q28" s="26" t="n"/>
     </row>
     <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="17" t="n">
+      <c r="A29" s="18" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="18" t="inlineStr">
+      <c r="B29" s="19" t="inlineStr">
         <is>
           <t>Infinity Dental Clinic</t>
         </is>
       </c>
-      <c r="C29" s="19" t="inlineStr">
+      <c r="C29" s="20" t="inlineStr">
         <is>
           <t>+7 707 515 64 85</t>
         </is>
       </c>
-      <c r="D29" s="20" t="inlineStr">
+      <c r="D29" s="21" t="inlineStr">
         <is>
           <t>Ауэзовский</t>
         </is>
       </c>
-      <c r="E29" s="20" t="inlineStr">
+      <c r="E29" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F29" s="17" t="inlineStr">
+      <c r="F29" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G29" s="22" t="n"/>
-      <c r="H29" s="22" t="n"/>
-      <c r="I29" s="22" t="n"/>
-      <c r="J29" s="22" t="n"/>
-      <c r="K29" s="22" t="n"/>
-      <c r="L29" s="22" t="n"/>
-      <c r="M29" s="22" t="n"/>
-      <c r="N29" s="23">
+      <c r="G29" s="23" t="n"/>
+      <c r="H29" s="23" t="n"/>
+      <c r="I29" s="23" t="n"/>
+      <c r="J29" s="23" t="n"/>
+      <c r="K29" s="23" t="n"/>
+      <c r="L29" s="23" t="n"/>
+      <c r="M29" s="23" t="n"/>
+      <c r="N29" s="24">
         <f>COUNTIF(H29:M29,"Г")</f>
         <v/>
       </c>
-      <c r="O29" s="23">
+      <c r="O29" s="24">
         <f>COUNTIF(H29:M29,"Ч")</f>
         <v/>
       </c>
-      <c r="P29" s="24" t="n"/>
-      <c r="Q29" s="25" t="n"/>
+      <c r="P29" s="25" t="n"/>
+      <c r="Q29" s="26" t="n"/>
     </row>
     <row r="30" ht="26" customHeight="1">
-      <c r="A30" s="17" t="n">
+      <c r="A30" s="18" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="18" t="inlineStr">
+      <c r="B30" s="19" t="inlineStr">
         <is>
           <t>Izi Clinic</t>
         </is>
       </c>
-      <c r="C30" s="19" t="inlineStr">
+      <c r="C30" s="20" t="inlineStr">
         <is>
           <t>+7 747 094 01 90</t>
         </is>
       </c>
-      <c r="D30" s="20" t="inlineStr">
+      <c r="D30" s="21" t="inlineStr">
         <is>
           <t>Алмалинский</t>
         </is>
       </c>
-      <c r="E30" s="20" t="inlineStr">
+      <c r="E30" s="21" t="inlineStr">
         <is>
           <t>по предварительной записи</t>
         </is>
       </c>
-      <c r="F30" s="17" t="inlineStr">
+      <c r="F30" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G30" s="22" t="n"/>
-      <c r="H30" s="22" t="n"/>
-      <c r="I30" s="22" t="n"/>
-      <c r="J30" s="22" t="n"/>
-      <c r="K30" s="22" t="n"/>
-      <c r="L30" s="22" t="n"/>
-      <c r="M30" s="22" t="n"/>
-      <c r="N30" s="23">
+      <c r="G30" s="23" t="n"/>
+      <c r="H30" s="23" t="n"/>
+      <c r="I30" s="23" t="n"/>
+      <c r="J30" s="23" t="n"/>
+      <c r="K30" s="23" t="n"/>
+      <c r="L30" s="23" t="n"/>
+      <c r="M30" s="23" t="n"/>
+      <c r="N30" s="24">
         <f>COUNTIF(H30:M30,"Г")</f>
         <v/>
       </c>
-      <c r="O30" s="23">
+      <c r="O30" s="24">
         <f>COUNTIF(H30:M30,"Ч")</f>
         <v/>
       </c>
-      <c r="P30" s="24" t="n"/>
-      <c r="Q30" s="25" t="n"/>
+      <c r="P30" s="25" t="n"/>
+      <c r="Q30" s="26" t="n"/>
     </row>
     <row r="31" ht="26" customHeight="1">
-      <c r="A31" s="17" t="n">
+      <c r="A31" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="18" t="inlineStr">
+      <c r="B31" s="19" t="inlineStr">
         <is>
           <t>Like-Clinic</t>
         </is>
       </c>
-      <c r="C31" s="19" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>+7 775 103 73 23</t>
         </is>
       </c>
-      <c r="D31" s="20" t="inlineStr">
+      <c r="D31" s="21" t="inlineStr">
         <is>
           <t>Ауэзовский</t>
         </is>
       </c>
-      <c r="E31" s="20" t="inlineStr">
+      <c r="E31" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F31" s="17" t="inlineStr">
+      <c r="F31" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G31" s="22" t="n"/>
-      <c r="H31" s="22" t="n"/>
-      <c r="I31" s="22" t="n"/>
-      <c r="J31" s="22" t="n"/>
-      <c r="K31" s="22" t="n"/>
-      <c r="L31" s="22" t="n"/>
-      <c r="M31" s="22" t="n"/>
-      <c r="N31" s="23">
+      <c r="G31" s="23" t="n"/>
+      <c r="H31" s="23" t="n"/>
+      <c r="I31" s="23" t="n"/>
+      <c r="J31" s="23" t="n"/>
+      <c r="K31" s="23" t="n"/>
+      <c r="L31" s="23" t="n"/>
+      <c r="M31" s="23" t="n"/>
+      <c r="N31" s="24">
         <f>COUNTIF(H31:M31,"Г")</f>
         <v/>
       </c>
-      <c r="O31" s="23">
+      <c r="O31" s="24">
         <f>COUNTIF(H31:M31,"Ч")</f>
         <v/>
       </c>
-      <c r="P31" s="24" t="n"/>
-      <c r="Q31" s="25" t="n"/>
+      <c r="P31" s="25" t="n"/>
+      <c r="Q31" s="26" t="n"/>
     </row>
     <row r="32" ht="26" customHeight="1">
-      <c r="A32" s="17" t="n">
+      <c r="A32" s="18" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="18" t="inlineStr">
+      <c r="B32" s="19" t="inlineStr">
         <is>
           <t>Dr. Yerzhana Musagalieva</t>
         </is>
       </c>
-      <c r="C32" s="19" t="inlineStr">
+      <c r="C32" s="20" t="inlineStr">
         <is>
           <t>+7 700 710 11 00</t>
         </is>
       </c>
-      <c r="D32" s="20" t="inlineStr">
+      <c r="D32" s="21" t="inlineStr">
         <is>
           <t>Алмалинский</t>
         </is>
       </c>
-      <c r="E32" s="20" t="inlineStr">
+      <c r="E32" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F32" s="17" t="inlineStr">
+      <c r="F32" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G32" s="22" t="n"/>
-      <c r="H32" s="22" t="n"/>
-      <c r="I32" s="22" t="n"/>
-      <c r="J32" s="22" t="n"/>
-      <c r="K32" s="22" t="n"/>
-      <c r="L32" s="22" t="n"/>
-      <c r="M32" s="22" t="n"/>
-      <c r="N32" s="23">
+      <c r="G32" s="23" t="n"/>
+      <c r="H32" s="23" t="n"/>
+      <c r="I32" s="23" t="n"/>
+      <c r="J32" s="23" t="n"/>
+      <c r="K32" s="23" t="n"/>
+      <c r="L32" s="23" t="n"/>
+      <c r="M32" s="23" t="n"/>
+      <c r="N32" s="24">
         <f>COUNTIF(H32:M32,"Г")</f>
         <v/>
       </c>
-      <c r="O32" s="23">
+      <c r="O32" s="24">
         <f>COUNTIF(H32:M32,"Ч")</f>
         <v/>
       </c>
-      <c r="P32" s="24" t="n"/>
-      <c r="Q32" s="25" t="n"/>
+      <c r="P32" s="25" t="n"/>
+      <c r="Q32" s="26" t="n"/>
     </row>
     <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="17" t="n">
+      <c r="A33" s="18" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="18" t="inlineStr">
+      <c r="B33" s="19" t="inlineStr">
         <is>
           <t>AQstom</t>
         </is>
       </c>
-      <c r="C33" s="19" t="inlineStr">
+      <c r="C33" s="20" t="inlineStr">
         <is>
           <t>+7 707 000 00 22</t>
         </is>
       </c>
-      <c r="D33" s="20" t="inlineStr">
+      <c r="D33" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E33" s="20" t="inlineStr">
+      <c r="E33" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F33" s="17" t="inlineStr">
+      <c r="F33" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G33" s="22" t="n"/>
-      <c r="H33" s="22" t="n"/>
-      <c r="I33" s="22" t="n"/>
-      <c r="J33" s="22" t="n"/>
-      <c r="K33" s="22" t="n"/>
-      <c r="L33" s="22" t="n"/>
-      <c r="M33" s="22" t="n"/>
-      <c r="N33" s="23">
+      <c r="G33" s="23" t="n"/>
+      <c r="H33" s="23" t="n"/>
+      <c r="I33" s="23" t="n"/>
+      <c r="J33" s="23" t="n"/>
+      <c r="K33" s="23" t="n"/>
+      <c r="L33" s="23" t="n"/>
+      <c r="M33" s="23" t="n"/>
+      <c r="N33" s="24">
         <f>COUNTIF(H33:M33,"Г")</f>
         <v/>
       </c>
-      <c r="O33" s="23">
+      <c r="O33" s="24">
         <f>COUNTIF(H33:M33,"Ч")</f>
         <v/>
       </c>
-      <c r="P33" s="24" t="n"/>
-      <c r="Q33" s="25" t="n"/>
+      <c r="P33" s="25" t="n"/>
+      <c r="Q33" s="26" t="n"/>
     </row>
     <row r="34" ht="26" customHeight="1">
-      <c r="A34" s="17" t="n">
+      <c r="A34" s="18" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="18" t="inlineStr">
+      <c r="B34" s="19" t="inlineStr">
         <is>
           <t>Global Dent</t>
         </is>
       </c>
-      <c r="C34" s="19" t="inlineStr">
+      <c r="C34" s="20" t="inlineStr">
         <is>
           <t>+7 707 470 90 88</t>
         </is>
       </c>
-      <c r="D34" s="20" t="inlineStr">
+      <c r="D34" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E34" s="20" t="inlineStr">
+      <c r="E34" s="21" t="inlineStr">
         <is>
           <t>открывается в 09:00 по звонку</t>
         </is>
       </c>
-      <c r="F34" s="17" t="inlineStr">
+      <c r="F34" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G34" s="22" t="n"/>
-      <c r="H34" s="22" t="n"/>
-      <c r="I34" s="22" t="n"/>
-      <c r="J34" s="22" t="n"/>
-      <c r="K34" s="22" t="n"/>
-      <c r="L34" s="22" t="n"/>
-      <c r="M34" s="22" t="n"/>
-      <c r="N34" s="23">
+      <c r="G34" s="23" t="n"/>
+      <c r="H34" s="23" t="n"/>
+      <c r="I34" s="23" t="n"/>
+      <c r="J34" s="23" t="n"/>
+      <c r="K34" s="23" t="n"/>
+      <c r="L34" s="23" t="n"/>
+      <c r="M34" s="23" t="n"/>
+      <c r="N34" s="24">
         <f>COUNTIF(H34:M34,"Г")</f>
         <v/>
       </c>
-      <c r="O34" s="23">
+      <c r="O34" s="24">
         <f>COUNTIF(H34:M34,"Ч")</f>
         <v/>
       </c>
-      <c r="P34" s="24" t="n"/>
-      <c r="Q34" s="25" t="n"/>
+      <c r="P34" s="25" t="n"/>
+      <c r="Q34" s="26" t="n"/>
     </row>
     <row r="35" ht="26" customHeight="1">
-      <c r="A35" s="17" t="n">
+      <c r="A35" s="18" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="18" t="inlineStr">
+      <c r="B35" s="19" t="inlineStr">
         <is>
           <t>Elit Stom (Сейфуллина 102)</t>
         </is>
       </c>
-      <c r="C35" s="19" t="inlineStr">
+      <c r="C35" s="20" t="inlineStr">
         <is>
           <t>+7 747 323 28 34</t>
         </is>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D35" s="21" t="inlineStr">
         <is>
           <t>Турксибский</t>
         </is>
       </c>
-      <c r="E35" s="20" t="inlineStr">
+      <c r="E35" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F35" s="17" t="inlineStr">
+      <c r="F35" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G35" s="22" t="n"/>
-      <c r="H35" s="22" t="n"/>
-      <c r="I35" s="22" t="n"/>
-      <c r="J35" s="22" t="n"/>
-      <c r="K35" s="22" t="n"/>
-      <c r="L35" s="22" t="n"/>
-      <c r="M35" s="22" t="n"/>
-      <c r="N35" s="23">
+      <c r="G35" s="23" t="n"/>
+      <c r="H35" s="23" t="n"/>
+      <c r="I35" s="23" t="n"/>
+      <c r="J35" s="23" t="n"/>
+      <c r="K35" s="23" t="n"/>
+      <c r="L35" s="23" t="n"/>
+      <c r="M35" s="23" t="n"/>
+      <c r="N35" s="24">
         <f>COUNTIF(H35:M35,"Г")</f>
         <v/>
       </c>
-      <c r="O35" s="23">
+      <c r="O35" s="24">
         <f>COUNTIF(H35:M35,"Ч")</f>
         <v/>
       </c>
-      <c r="P35" s="24" t="n"/>
-      <c r="Q35" s="25" t="n"/>
+      <c r="P35" s="25" t="n"/>
+      <c r="Q35" s="26" t="n"/>
     </row>
     <row r="36" ht="26" customHeight="1">
-      <c r="A36" s="17" t="n">
+      <c r="A36" s="18" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="18" t="inlineStr">
+      <c r="B36" s="19" t="inlineStr">
         <is>
           <t>Expert 32 stom</t>
         </is>
       </c>
-      <c r="C36" s="19" t="inlineStr">
+      <c r="C36" s="20" t="inlineStr">
         <is>
           <t>+7 775 846 19 49</t>
         </is>
       </c>
-      <c r="D36" s="20" t="inlineStr">
+      <c r="D36" s="21" t="inlineStr">
         <is>
           <t>Турксибский</t>
         </is>
       </c>
-      <c r="E36" s="20" t="inlineStr">
+      <c r="E36" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F36" s="17" t="inlineStr">
+      <c r="F36" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G36" s="22" t="n"/>
-      <c r="H36" s="22" t="n"/>
-      <c r="I36" s="22" t="n"/>
-      <c r="J36" s="22" t="n"/>
-      <c r="K36" s="22" t="n"/>
-      <c r="L36" s="22" t="n"/>
-      <c r="M36" s="22" t="n"/>
-      <c r="N36" s="23">
+      <c r="G36" s="23" t="n"/>
+      <c r="H36" s="23" t="n"/>
+      <c r="I36" s="23" t="n"/>
+      <c r="J36" s="23" t="n"/>
+      <c r="K36" s="23" t="n"/>
+      <c r="L36" s="23" t="n"/>
+      <c r="M36" s="23" t="n"/>
+      <c r="N36" s="24">
         <f>COUNTIF(H36:M36,"Г")</f>
         <v/>
       </c>
-      <c r="O36" s="23">
+      <c r="O36" s="24">
         <f>COUNTIF(H36:M36,"Ч")</f>
         <v/>
       </c>
-      <c r="P36" s="24" t="n"/>
-      <c r="Q36" s="25" t="n"/>
+      <c r="P36" s="25" t="n"/>
+      <c r="Q36" s="26" t="n"/>
     </row>
     <row r="37" ht="26" customHeight="1">
-      <c r="A37" s="17" t="n">
+      <c r="A37" s="18" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="18" t="inlineStr">
+      <c r="B37" s="19" t="inlineStr">
         <is>
           <t>DentalPRO</t>
         </is>
       </c>
-      <c r="C37" s="19" t="inlineStr">
+      <c r="C37" s="20" t="inlineStr">
         <is>
           <t>+7 771 800 00 67</t>
         </is>
       </c>
-      <c r="D37" s="20" t="inlineStr">
+      <c r="D37" s="21" t="inlineStr">
         <is>
           <t>Турксибский</t>
         </is>
       </c>
-      <c r="E37" s="20" t="inlineStr">
+      <c r="E37" s="21" t="inlineStr">
         <is>
           <t>не указаны</t>
         </is>
       </c>
-      <c r="F37" s="17" t="inlineStr">
+      <c r="F37" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G37" s="22" t="n"/>
-      <c r="H37" s="22" t="n"/>
-      <c r="I37" s="22" t="n"/>
-      <c r="J37" s="22" t="n"/>
-      <c r="K37" s="22" t="n"/>
-      <c r="L37" s="22" t="n"/>
-      <c r="M37" s="22" t="n"/>
-      <c r="N37" s="23">
+      <c r="G37" s="23" t="n"/>
+      <c r="H37" s="23" t="n"/>
+      <c r="I37" s="23" t="n"/>
+      <c r="J37" s="23" t="n"/>
+      <c r="K37" s="23" t="n"/>
+      <c r="L37" s="23" t="n"/>
+      <c r="M37" s="23" t="n"/>
+      <c r="N37" s="24">
         <f>COUNTIF(H37:M37,"Г")</f>
         <v/>
       </c>
-      <c r="O37" s="23">
+      <c r="O37" s="24">
         <f>COUNTIF(H37:M37,"Ч")</f>
         <v/>
       </c>
-      <c r="P37" s="24" t="n"/>
-      <c r="Q37" s="25" t="n"/>
+      <c r="P37" s="25" t="n"/>
+      <c r="Q37" s="26" t="n"/>
     </row>
     <row r="38" ht="26" customHeight="1">
-      <c r="A38" s="17" t="n">
+      <c r="A38" s="18" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="18" t="inlineStr">
+      <c r="B38" s="19" t="inlineStr">
         <is>
           <t>Dr.Omar Dental Clinic</t>
         </is>
       </c>
-      <c r="C38" s="19" t="inlineStr">
+      <c r="C38" s="20" t="inlineStr">
         <is>
           <t>+7 778 143 52 61</t>
         </is>
       </c>
-      <c r="D38" s="20" t="inlineStr">
+      <c r="D38" s="21" t="inlineStr">
         <is>
           <t>Талгарский (Бесагаш)</t>
         </is>
       </c>
-      <c r="E38" s="20" t="inlineStr">
+      <c r="E38" s="21" t="inlineStr">
         <is>
           <t>открывается в 09:00</t>
         </is>
       </c>
-      <c r="F38" s="17" t="inlineStr">
+      <c r="F38" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G38" s="22" t="n"/>
-      <c r="H38" s="22" t="n"/>
-      <c r="I38" s="22" t="n"/>
-      <c r="J38" s="22" t="n"/>
-      <c r="K38" s="22" t="n"/>
-      <c r="L38" s="22" t="n"/>
-      <c r="M38" s="22" t="n"/>
-      <c r="N38" s="23">
+      <c r="G38" s="23" t="n"/>
+      <c r="H38" s="23" t="n"/>
+      <c r="I38" s="23" t="n"/>
+      <c r="J38" s="23" t="n"/>
+      <c r="K38" s="23" t="n"/>
+      <c r="L38" s="23" t="n"/>
+      <c r="M38" s="23" t="n"/>
+      <c r="N38" s="24">
         <f>COUNTIF(H38:M38,"Г")</f>
         <v/>
       </c>
-      <c r="O38" s="23">
+      <c r="O38" s="24">
         <f>COUNTIF(H38:M38,"Ч")</f>
         <v/>
       </c>
-      <c r="P38" s="24" t="n"/>
-      <c r="Q38" s="25" t="n"/>
+      <c r="P38" s="25" t="n"/>
+      <c r="Q38" s="26" t="n"/>
     </row>
     <row r="39" ht="26" customHeight="1">
-      <c r="A39" s="17" t="n">
+      <c r="A39" s="18" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="18" t="inlineStr">
+      <c r="B39" s="19" t="inlineStr">
         <is>
           <t>InClinic</t>
         </is>
       </c>
-      <c r="C39" s="19" t="inlineStr">
+      <c r="C39" s="20" t="inlineStr">
         <is>
           <t>+7 707 333 22 66</t>
         </is>
       </c>
-      <c r="D39" s="20" t="inlineStr">
+      <c r="D39" s="21" t="inlineStr">
         <is>
           <t>Медеуский</t>
         </is>
       </c>
-      <c r="E39" s="20" t="inlineStr">
+      <c r="E39" s="21" t="inlineStr">
         <is>
           <t>открывается в 09:00</t>
         </is>
       </c>
-      <c r="F39" s="17" t="inlineStr">
+      <c r="F39" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G39" s="22" t="n"/>
-      <c r="H39" s="22" t="n"/>
-      <c r="I39" s="22" t="n"/>
-      <c r="J39" s="22" t="n"/>
-      <c r="K39" s="22" t="n"/>
-      <c r="L39" s="22" t="n"/>
-      <c r="M39" s="22" t="n"/>
-      <c r="N39" s="23">
+      <c r="G39" s="23" t="n"/>
+      <c r="H39" s="23" t="n"/>
+      <c r="I39" s="23" t="n"/>
+      <c r="J39" s="23" t="n"/>
+      <c r="K39" s="23" t="n"/>
+      <c r="L39" s="23" t="n"/>
+      <c r="M39" s="23" t="n"/>
+      <c r="N39" s="24">
         <f>COUNTIF(H39:M39,"Г")</f>
         <v/>
       </c>
-      <c r="O39" s="23">
+      <c r="O39" s="24">
         <f>COUNTIF(H39:M39,"Ч")</f>
         <v/>
       </c>
-      <c r="P39" s="24" t="n"/>
-      <c r="Q39" s="25" t="n"/>
+      <c r="P39" s="25" t="n"/>
+      <c r="Q39" s="26" t="n"/>
     </row>
     <row r="40" ht="26" customHeight="1">
-      <c r="A40" s="17" t="n">
+      <c r="A40" s="18" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="18" t="inlineStr">
+      <c r="B40" s="19" t="inlineStr">
         <is>
           <t>DOSTYQ DENTAL CENTER</t>
         </is>
       </c>
-      <c r="C40" s="19" t="inlineStr">
+      <c r="C40" s="20" t="inlineStr">
         <is>
           <t>+7 707 677 71 09</t>
         </is>
       </c>
-      <c r="D40" s="20" t="inlineStr">
+      <c r="D40" s="21" t="inlineStr">
         <is>
           <t>Алмалинский</t>
         </is>
       </c>
-      <c r="E40" s="20" t="inlineStr">
+      <c r="E40" s="21" t="inlineStr">
         <is>
           <t>открывается в 10:00</t>
         </is>
       </c>
-      <c r="F40" s="17" t="inlineStr">
+      <c r="F40" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G40" s="22" t="n"/>
-      <c r="H40" s="22" t="n"/>
-      <c r="I40" s="22" t="n"/>
-      <c r="J40" s="22" t="n"/>
-      <c r="K40" s="22" t="n"/>
-      <c r="L40" s="22" t="n"/>
-      <c r="M40" s="22" t="n"/>
-      <c r="N40" s="23">
+      <c r="G40" s="23" t="n"/>
+      <c r="H40" s="23" t="n"/>
+      <c r="I40" s="23" t="n"/>
+      <c r="J40" s="23" t="n"/>
+      <c r="K40" s="23" t="n"/>
+      <c r="L40" s="23" t="n"/>
+      <c r="M40" s="23" t="n"/>
+      <c r="N40" s="24">
         <f>COUNTIF(H40:M40,"Г")</f>
         <v/>
       </c>
-      <c r="O40" s="23">
+      <c r="O40" s="24">
         <f>COUNTIF(H40:M40,"Ч")</f>
         <v/>
       </c>
-      <c r="P40" s="24" t="n"/>
-      <c r="Q40" s="25" t="n"/>
+      <c r="P40" s="25" t="n"/>
+      <c r="Q40" s="26" t="n"/>
     </row>
     <row r="41" ht="26" customHeight="1">
-      <c r="A41" s="17" t="n">
+      <c r="A41" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="18" t="inlineStr">
+      <c r="B41" s="19" t="inlineStr">
         <is>
           <t>КГМЦ</t>
         </is>
       </c>
-      <c r="C41" s="19" t="inlineStr">
+      <c r="C41" s="20" t="inlineStr">
         <is>
           <t>+7 727 397 37 78</t>
         </is>
       </c>
-      <c r="D41" s="20" t="inlineStr">
+      <c r="D41" s="21" t="inlineStr">
         <is>
           <t>Турксибский</t>
         </is>
       </c>
-      <c r="E41" s="20" t="inlineStr">
+      <c r="E41" s="21" t="inlineStr">
         <is>
           <t>открывается в 09:00 по записи</t>
         </is>
       </c>
-      <c r="F41" s="17" t="inlineStr">
+      <c r="F41" s="18" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G41" s="22" t="n"/>
-      <c r="H41" s="22" t="n"/>
-      <c r="I41" s="22" t="n"/>
-      <c r="J41" s="22" t="n"/>
-      <c r="K41" s="22" t="n"/>
-      <c r="L41" s="22" t="n"/>
-      <c r="M41" s="22" t="n"/>
-      <c r="N41" s="23">
+      <c r="G41" s="23" t="n"/>
+      <c r="H41" s="23" t="n"/>
+      <c r="I41" s="23" t="n"/>
+      <c r="J41" s="23" t="n"/>
+      <c r="K41" s="23" t="n"/>
+      <c r="L41" s="23" t="n"/>
+      <c r="M41" s="23" t="n"/>
+      <c r="N41" s="24">
         <f>COUNTIF(H41:M41,"Г")</f>
         <v/>
       </c>
-      <c r="O41" s="23">
+      <c r="O41" s="24">
         <f>COUNTIF(H41:M41,"Ч")</f>
         <v/>
       </c>
-      <c r="P41" s="24" t="n"/>
-      <c r="Q41" s="25" t="n"/>
+      <c r="P41" s="25" t="n"/>
+      <c r="Q41" s="26" t="n"/>
     </row>
     <row r="42" ht="26" customHeight="1">
-      <c r="A42" s="17" t="n">
+      <c r="A42" s="18" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="18" t="inlineStr">
+      <c r="B42" s="19" t="inlineStr">
         <is>
           <t>Стома Плюс</t>
         </is>
       </c>
-      <c r="C42" s="19" t="inlineStr">
+      <c r="C42" s="20" t="inlineStr">
         <is>
           <t>+7 771 335 30 17</t>
         </is>
       </c>
-      <c r="D42" s="20" t="inlineStr">
+      <c r="D42" s="21" t="inlineStr">
         <is>
           <t>Алатауский</t>
         </is>
       </c>
-      <c r="E42" s="20" t="inlineStr">
+      <c r="E42" s="21" t="inlineStr">
         <is>
           <t>09:00-23:00</t>
         </is>
       </c>
-      <c r="F42" s="17" t="inlineStr">
+      <c r="F42" s="18" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G42" s="22" t="n"/>
-      <c r="H42" s="22" t="n"/>
-      <c r="I42" s="22" t="n"/>
-      <c r="J42" s="22" t="n"/>
-      <c r="K42" s="22" t="n"/>
-      <c r="L42" s="22" t="n"/>
-      <c r="M42" s="22" t="n"/>
-      <c r="N42" s="23">
+      <c r="G42" s="23" t="n"/>
+      <c r="H42" s="23" t="n"/>
+      <c r="I42" s="23" t="n"/>
+      <c r="J42" s="23" t="n"/>
+      <c r="K42" s="23" t="n"/>
+      <c r="L42" s="23" t="n"/>
+      <c r="M42" s="23" t="n"/>
+      <c r="N42" s="24">
         <f>COUNTIF(H42:M42,"Г")</f>
         <v/>
       </c>
-      <c r="O42" s="23">
+      <c r="O42" s="24">
         <f>COUNTIF(H42:M42,"Ч")</f>
         <v/>
       </c>
-      <c r="P42" s="24" t="n"/>
-      <c r="Q42" s="25" t="n"/>
+      <c r="P42" s="25" t="n"/>
+      <c r="Q42" s="26" t="n"/>
     </row>
     <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="17" t="n">
+      <c r="A43" s="18" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="18" t="inlineStr">
+      <c r="B43" s="19" t="inlineStr">
         <is>
           <t>Estet Clinic</t>
         </is>
       </c>
-      <c r="C43" s="19" t="inlineStr">
+      <c r="C43" s="20" t="inlineStr">
         <is>
           <t>+7 707 101 02 33</t>
         </is>
       </c>
-      <c r="D43" s="20" t="inlineStr">
+      <c r="D43" s="21" t="inlineStr">
         <is>
           <t>Ауэзовский</t>
         </is>
       </c>
-      <c r="E43" s="20" t="inlineStr">
+      <c r="E43" s="21" t="inlineStr">
         <is>
           <t>09:00-23:00 ежедневно</t>
         </is>
       </c>
-      <c r="F43" s="17" t="inlineStr">
+      <c r="F43" s="18" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G43" s="22" t="n"/>
-      <c r="H43" s="22" t="n"/>
-      <c r="I43" s="22" t="n"/>
-      <c r="J43" s="22" t="n"/>
-      <c r="K43" s="22" t="n"/>
-      <c r="L43" s="22" t="n"/>
-      <c r="M43" s="22" t="n"/>
-      <c r="N43" s="23">
+      <c r="G43" s="23" t="n"/>
+      <c r="H43" s="23" t="n"/>
+      <c r="I43" s="23" t="n"/>
+      <c r="J43" s="23" t="n"/>
+      <c r="K43" s="23" t="n"/>
+      <c r="L43" s="23" t="n"/>
+      <c r="M43" s="23" t="n"/>
+      <c r="N43" s="24">
         <f>COUNTIF(H43:M43,"Г")</f>
         <v/>
       </c>
-      <c r="O43" s="23">
+      <c r="O43" s="24">
         <f>COUNTIF(H43:M43,"Ч")</f>
         <v/>
       </c>
-      <c r="P43" s="24" t="n"/>
-      <c r="Q43" s="25" t="n"/>
+      <c r="P43" s="25" t="n"/>
+      <c r="Q43" s="26" t="n"/>
     </row>
     <row r="44" ht="26" customHeight="1">
-      <c r="A44" s="17" t="n">
+      <c r="A44" s="18" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="18" t="inlineStr">
+      <c r="B44" s="19" t="inlineStr">
         <is>
           <t>Muslim Dent</t>
         </is>
       </c>
-      <c r="C44" s="19" t="inlineStr">
+      <c r="C44" s="20" t="inlineStr">
         <is>
           <t>+7 771 800 00 65</t>
         </is>
       </c>
-      <c r="D44" s="20" t="inlineStr">
+      <c r="D44" s="21" t="inlineStr">
         <is>
           <t>Алмалинский</t>
         </is>
       </c>
-      <c r="E44" s="20" t="inlineStr">
+      <c r="E44" s="21" t="inlineStr">
         <is>
           <t>10:00-23:45 ежедневно</t>
         </is>
       </c>
-      <c r="F44" s="17" t="inlineStr">
+      <c r="F44" s="18" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G44" s="22" t="n"/>
-      <c r="H44" s="22" t="n"/>
-      <c r="I44" s="22" t="n"/>
-      <c r="J44" s="22" t="n"/>
-      <c r="K44" s="22" t="n"/>
-      <c r="L44" s="22" t="n"/>
-      <c r="M44" s="22" t="n"/>
-      <c r="N44" s="23">
+      <c r="G44" s="23" t="n"/>
+      <c r="H44" s="23" t="n"/>
+      <c r="I44" s="23" t="n"/>
+      <c r="J44" s="23" t="n"/>
+      <c r="K44" s="23" t="n"/>
+      <c r="L44" s="23" t="n"/>
+      <c r="M44" s="23" t="n"/>
+      <c r="N44" s="24">
         <f>COUNTIF(H44:M44,"Г")</f>
         <v/>
       </c>
-      <c r="O44" s="23">
+      <c r="O44" s="24">
         <f>COUNTIF(H44:M44,"Ч")</f>
         <v/>
       </c>
-      <c r="P44" s="24" t="n"/>
-      <c r="Q44" s="25" t="n"/>
+      <c r="P44" s="25" t="n"/>
+      <c r="Q44" s="26" t="n"/>
     </row>
     <row r="45" ht="26" customHeight="1">
-      <c r="A45" s="17" t="n">
+      <c r="A45" s="18" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="18" t="inlineStr">
+      <c r="B45" s="19" t="inlineStr">
         <is>
           <t>Bilal stom</t>
         </is>
       </c>
-      <c r="C45" s="19" t="inlineStr">
+      <c r="C45" s="20" t="inlineStr">
         <is>
           <t>+7 707 666 98 92</t>
         </is>
       </c>
-      <c r="D45" s="20" t="inlineStr">
+      <c r="D45" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E45" s="20" t="inlineStr">
+      <c r="E45" s="21" t="inlineStr">
         <is>
           <t>09:00-24:00 ежедневно</t>
         </is>
       </c>
-      <c r="F45" s="17" t="inlineStr">
+      <c r="F45" s="18" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G45" s="22" t="n"/>
-      <c r="H45" s="22" t="n"/>
-      <c r="I45" s="22" t="n"/>
-      <c r="J45" s="22" t="n"/>
-      <c r="K45" s="22" t="n"/>
-      <c r="L45" s="22" t="n"/>
-      <c r="M45" s="22" t="n"/>
-      <c r="N45" s="23">
+      <c r="G45" s="23" t="n"/>
+      <c r="H45" s="23" t="n"/>
+      <c r="I45" s="23" t="n"/>
+      <c r="J45" s="23" t="n"/>
+      <c r="K45" s="23" t="n"/>
+      <c r="L45" s="23" t="n"/>
+      <c r="M45" s="23" t="n"/>
+      <c r="N45" s="24">
         <f>COUNTIF(H45:M45,"Г")</f>
         <v/>
       </c>
-      <c r="O45" s="23">
+      <c r="O45" s="24">
         <f>COUNTIF(H45:M45,"Ч")</f>
         <v/>
       </c>
-      <c r="P45" s="24" t="n"/>
-      <c r="Q45" s="25" t="n"/>
+      <c r="P45" s="25" t="n"/>
+      <c r="Q45" s="26" t="n"/>
     </row>
     <row r="46" ht="26" customHeight="1">
-      <c r="A46" s="17" t="n">
+      <c r="A46" s="18" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="18" t="inlineStr">
+      <c r="B46" s="19" t="inlineStr">
         <is>
           <t>Dr.SULTANOV ATABEK</t>
         </is>
       </c>
-      <c r="C46" s="19" t="inlineStr">
+      <c r="C46" s="20" t="inlineStr">
         <is>
           <t>+7 775 300 85 05</t>
         </is>
       </c>
-      <c r="D46" s="20" t="inlineStr">
+      <c r="D46" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E46" s="20" t="inlineStr">
+      <c r="E46" s="21" t="inlineStr">
         <is>
           <t>09:00-24:00</t>
         </is>
       </c>
-      <c r="F46" s="17" t="inlineStr">
+      <c r="F46" s="18" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G46" s="22" t="n"/>
-      <c r="H46" s="22" t="n"/>
-      <c r="I46" s="22" t="n"/>
-      <c r="J46" s="22" t="n"/>
-      <c r="K46" s="22" t="n"/>
-      <c r="L46" s="22" t="n"/>
-      <c r="M46" s="22" t="n"/>
-      <c r="N46" s="23">
+      <c r="G46" s="23" t="n"/>
+      <c r="H46" s="23" t="n"/>
+      <c r="I46" s="23" t="n"/>
+      <c r="J46" s="23" t="n"/>
+      <c r="K46" s="23" t="n"/>
+      <c r="L46" s="23" t="n"/>
+      <c r="M46" s="23" t="n"/>
+      <c r="N46" s="24">
         <f>COUNTIF(H46:M46,"Г")</f>
         <v/>
       </c>
-      <c r="O46" s="23">
+      <c r="O46" s="24">
         <f>COUNTIF(H46:M46,"Ч")</f>
         <v/>
       </c>
-      <c r="P46" s="24" t="n"/>
-      <c r="Q46" s="25" t="n"/>
+      <c r="P46" s="25" t="n"/>
+      <c r="Q46" s="26" t="n"/>
     </row>
     <row r="47" ht="26" customHeight="1">
-      <c r="A47" s="17" t="n">
+      <c r="A47" s="18" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="18" t="inlineStr">
+      <c r="B47" s="19" t="inlineStr">
         <is>
           <t>Dr. Beridze</t>
         </is>
       </c>
-      <c r="C47" s="19" t="inlineStr">
+      <c r="C47" s="20" t="inlineStr">
         <is>
           <t>+7 775 522 05 09</t>
         </is>
       </c>
-      <c r="D47" s="20" t="inlineStr">
+      <c r="D47" s="21" t="inlineStr">
         <is>
           <t>Турксибский</t>
         </is>
       </c>
-      <c r="E47" s="20" t="inlineStr">
+      <c r="E47" s="21" t="inlineStr">
         <is>
           <t>09:00-24:00 ежедневно</t>
         </is>
       </c>
-      <c r="F47" s="17" t="inlineStr">
+      <c r="F47" s="18" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G47" s="22" t="n"/>
-      <c r="H47" s="22" t="n"/>
-      <c r="I47" s="22" t="n"/>
-      <c r="J47" s="22" t="n"/>
-      <c r="K47" s="22" t="n"/>
-      <c r="L47" s="22" t="n"/>
-      <c r="M47" s="22" t="n"/>
-      <c r="N47" s="23">
+      <c r="G47" s="23" t="n"/>
+      <c r="H47" s="23" t="n"/>
+      <c r="I47" s="23" t="n"/>
+      <c r="J47" s="23" t="n"/>
+      <c r="K47" s="23" t="n"/>
+      <c r="L47" s="23" t="n"/>
+      <c r="M47" s="23" t="n"/>
+      <c r="N47" s="24">
         <f>COUNTIF(H47:M47,"Г")</f>
         <v/>
       </c>
-      <c r="O47" s="23">
+      <c r="O47" s="24">
         <f>COUNTIF(H47:M47,"Ч")</f>
         <v/>
       </c>
-      <c r="P47" s="24" t="n"/>
-      <c r="Q47" s="25" t="n"/>
+      <c r="P47" s="25" t="n"/>
+      <c r="Q47" s="26" t="n"/>
     </row>
     <row r="48" ht="26" customHeight="1">
-      <c r="A48" s="17" t="n">
+      <c r="A48" s="18" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="18" t="inlineStr">
+      <c r="B48" s="19" t="inlineStr">
         <is>
           <t>Elit Dent</t>
         </is>
       </c>
-      <c r="C48" s="19" t="inlineStr">
+      <c r="C48" s="20" t="inlineStr">
         <is>
           <t>+7 708 269 71 00</t>
         </is>
       </c>
-      <c r="D48" s="20" t="inlineStr">
+      <c r="D48" s="21" t="inlineStr">
         <is>
           <t>Бостандыкский</t>
         </is>
       </c>
-      <c r="E48" s="20" t="inlineStr">
+      <c r="E48" s="21" t="inlineStr">
         <is>
           <t>круглосуточно</t>
         </is>
       </c>
-      <c r="F48" s="17" t="inlineStr">
+      <c r="F48" s="18" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G48" s="22" t="n"/>
-      <c r="H48" s="22" t="n"/>
-      <c r="I48" s="22" t="n"/>
-      <c r="J48" s="22" t="n"/>
-      <c r="K48" s="22" t="n"/>
-      <c r="L48" s="22" t="n"/>
-      <c r="M48" s="22" t="n"/>
-      <c r="N48" s="23">
+      <c r="G48" s="23" t="n"/>
+      <c r="H48" s="23" t="n"/>
+      <c r="I48" s="23" t="n"/>
+      <c r="J48" s="23" t="n"/>
+      <c r="K48" s="23" t="n"/>
+      <c r="L48" s="23" t="n"/>
+      <c r="M48" s="23" t="n"/>
+      <c r="N48" s="24">
         <f>COUNTIF(H48:M48,"Г")</f>
         <v/>
       </c>
-      <c r="O48" s="23">
+      <c r="O48" s="24">
         <f>COUNTIF(H48:M48,"Ч")</f>
         <v/>
       </c>
-      <c r="P48" s="24" t="n"/>
-      <c r="Q48" s="25" t="n"/>
+      <c r="P48" s="25" t="n"/>
+      <c r="Q48" s="26" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q48"/>
@@ -3479,7 +3498,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Итоги обзвона</t>
         </is>
@@ -3493,195 +3512,195 @@
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="27" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>Окно</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Сделано звонков</t>
         </is>
       </c>
-      <c r="C4" s="27" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>Ответил человек</t>
         </is>
       </c>
-      <c r="D4" s="27" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>Гудки без ответа</t>
         </is>
       </c>
-      <c r="E4" s="27" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>Доля гудков</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>Рабочее время</t>
         </is>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="30">
         <f>COUNTA(Обзвон!$G$2:$G$48)</f>
         <v/>
       </c>
-      <c r="C5" s="29">
+      <c r="C5" s="30">
         <f>COUNTIF(Обзвон!$G$2:$G$48,"Ч")</f>
         <v/>
       </c>
-      <c r="D5" s="29">
+      <c r="D5" s="30">
         <f>COUNTIF(Обзвон!$G$2:$G$48,"Г")</f>
         <v/>
       </c>
-      <c r="E5" s="30">
+      <c r="E5" s="31">
         <f>IFERROR(COUNTIF(Обзвон!$G$2:$G$48,"Г")/COUNTA(Обзвон!$G$2:$G$48),"")</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="A6" s="32" t="inlineStr">
         <is>
           <t>Будний вечер</t>
         </is>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="33">
         <f>COUNTA(Обзвон!$H$2:$I$48)</f>
         <v/>
       </c>
-      <c r="C6" s="32">
+      <c r="C6" s="33">
         <f>COUNTIF(Обзвон!$H$2:$I$48,"Ч")</f>
         <v/>
       </c>
-      <c r="D6" s="32">
+      <c r="D6" s="33">
         <f>COUNTIF(Обзвон!$H$2:$I$48,"Г")</f>
         <v/>
       </c>
-      <c r="E6" s="33">
+      <c r="E6" s="34">
         <f>IFERROR(COUNTIF(Обзвон!$H$2:$I$48,"Г")/COUNTA(Обзвон!$H$2:$I$48),"")</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>Суббота</t>
         </is>
       </c>
-      <c r="B7" s="29">
+      <c r="B7" s="30">
         <f>COUNTA(Обзвон!$J$2:$K$48)</f>
         <v/>
       </c>
-      <c r="C7" s="29">
+      <c r="C7" s="30">
         <f>COUNTIF(Обзвон!$J$2:$K$48,"Ч")</f>
         <v/>
       </c>
-      <c r="D7" s="29">
+      <c r="D7" s="30">
         <f>COUNTIF(Обзвон!$J$2:$K$48,"Г")</f>
         <v/>
       </c>
-      <c r="E7" s="30">
+      <c r="E7" s="31">
         <f>IFERROR(COUNTIF(Обзвон!$J$2:$K$48,"Г")/COUNTA(Обзвон!$J$2:$K$48),"")</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="31" t="inlineStr">
+      <c r="A8" s="32" t="inlineStr">
         <is>
           <t>Воскресенье</t>
         </is>
       </c>
-      <c r="B8" s="32">
+      <c r="B8" s="33">
         <f>COUNTA(Обзвон!$L$2:$M$48)</f>
         <v/>
       </c>
-      <c r="C8" s="32">
+      <c r="C8" s="33">
         <f>COUNTIF(Обзвон!$L$2:$M$48,"Ч")</f>
         <v/>
       </c>
-      <c r="D8" s="32">
+      <c r="D8" s="33">
         <f>COUNTIF(Обзвон!$L$2:$M$48,"Г")</f>
         <v/>
       </c>
-      <c r="E8" s="33">
+      <c r="E8" s="34">
         <f>IFERROR(COUNTIF(Обзвон!$L$2:$M$48,"Г")/COUNTA(Обзвон!$L$2:$M$48),"")</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="34" t="inlineStr">
+      <c r="A11" s="35" t="inlineStr">
         <is>
           <t>Что это значит</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="35" t="inlineStr">
+      <c r="A12" s="36" t="inlineStr">
         <is>
           <t>Порог по вечернему окну</t>
         </is>
       </c>
-      <c r="B12" s="36">
+      <c r="B12" s="37">
         <f>IF(E6="","нет данных",IF(E6&gt;0.4,"Продолжаем — гипотеза держится",IF(E6&lt;0.25,"Дверь закрыта — менять нишу или окно","Пограничная зона — смотреть качество ответов")))</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="37" t="inlineStr">
+      <c r="A14" s="38" t="inlineStr">
         <is>
           <t>• Больше 40% гудков вечером — продолжаем.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="37" t="inlineStr">
+      <c r="A15" s="38" t="inlineStr">
         <is>
           <t>• Меньше 25% — клиники закрывают вечер сами, эта дверь не наша.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="37" t="inlineStr">
+      <c r="A16" s="38" t="inlineStr">
         <is>
           <t>• Между 25% и 40% — смотрим заметки: автоответчик без записи и «перезвоните завтра» считаем потерянным звонком.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="34" t="inlineStr">
+      <c r="A19" s="35" t="inlineStr">
         <is>
           <t>Кандидаты на разговор</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="37" t="inlineStr">
+      <c r="A20" s="38" t="inlineStr">
         <is>
           <t>Отсортируйте лист «Обзвон» по колонке «Гудков» по убыванию. Сверху окажутся клиники, которые не ответили ни разу — с них и начинаем.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="38" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>Клиник, не ответивших ни разу (6 из 6)</t>
         </is>
       </c>
-      <c r="B22" s="36">
+      <c r="B22" s="37">
         <f>COUNTIF(Обзвон!$N$2:$N$48,6)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="38" t="inlineStr">
+      <c r="A23" s="39" t="inlineStr">
         <is>
           <t>Клиник, где хотя бы раз ответил человек</t>
         </is>
       </c>
-      <c r="B23" s="39">
+      <c r="B23" s="40">
         <f>COUNTIF(Обзвон!$O$2:$O$48,"&gt;0")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Take the clinic list to a hundred so it survives into the selling
Forty-seven was enough to measure with; the same list has to carry the sales
round afterwards, and a quarter of it will have answered every time. Fifty-four
more clinics, deduplicated by phone rather than by name — chains such as Рахат
publish one number across six branches, and two entries sharing a line would
have been counted as two measurements of the same reception.

Searching by microdistrict rather than by city broke 2GIS out of the promoted
top of the results, which is where the small practices actually live. Medeu,
Nauryzbai and Alatau went from almost nothing to twenty-eight between them.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/obzvon-stomatologii-almaty.xlsx
+++ b/docs/obzvon-stomatologii-almaty.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Итоги" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Обзвон'!$A$1:$Q$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Обзвон'!$A$1:$Q$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1141,7 +1141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q48"/>
+  <dimension ref="A1:Q102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1256,22 +1256,22 @@
       </c>
       <c r="B2" s="19" t="inlineStr">
         <is>
-          <t>Ажар Дент</t>
+          <t>Asyly_dent</t>
         </is>
       </c>
       <c r="C2" s="20" t="inlineStr">
         <is>
-          <t>+7 705 222 99 22</t>
+          <t>+7 700 088 20 21</t>
         </is>
       </c>
       <c r="D2" s="21" t="inlineStr">
         <is>
-          <t>Жетысуский</t>
+          <t>Алатауский</t>
         </is>
       </c>
       <c r="E2" s="21" t="inlineStr">
         <is>
-          <t>09:00-19:00</t>
+          <t>есть обеденный перерыв</t>
         </is>
       </c>
       <c r="F2" s="22" t="inlineStr">
@@ -1303,22 +1303,22 @@
       </c>
       <c r="B3" s="19" t="inlineStr">
         <is>
-          <t>Empire dental clinic</t>
+          <t>Ever Smile</t>
         </is>
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
-          <t>+7 778 114 76 94</t>
+          <t>+7 747 900 30 09</t>
         </is>
       </c>
       <c r="D3" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Алмалинский</t>
         </is>
       </c>
       <c r="E3" s="21" t="inlineStr">
         <is>
-          <t>10:00-20:00</t>
+          <t>10:00-22:00 обед 12:00-14:30</t>
         </is>
       </c>
       <c r="F3" s="22" t="inlineStr">
@@ -1444,17 +1444,17 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Kids Stom</t>
+          <t>Sara clinic</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>+7 707 220 80 00</t>
+          <t>+7 707 675 70 00</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Ауэзовский</t>
         </is>
       </c>
       <c r="E6" s="21" t="inlineStr">
@@ -1491,22 +1491,22 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Sara clinic</t>
+          <t>Dobro Dent</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
-          <t>+7 707 675 70 00</t>
+          <t>+7 775 030 09 99</t>
         </is>
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>Ауэзовский</t>
+          <t>Бостандыкский</t>
         </is>
       </c>
       <c r="E7" s="21" t="inlineStr">
         <is>
-          <t>09:00-21:00 ежедневно</t>
+          <t>09:00-22:00 ежедневно</t>
         </is>
       </c>
       <c r="F7" s="22" t="inlineStr">
@@ -1538,22 +1538,22 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>DS Stomatology</t>
+          <t>Empire dental clinic</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>+7 771 267 61 27</t>
+          <t>+7 778 114 76 94</t>
         </is>
       </c>
       <c r="D8" s="21" t="inlineStr">
         <is>
-          <t>Талгарский</t>
+          <t>Бостандыкский</t>
         </is>
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
-          <t>09:00-21:00 ежедневно</t>
+          <t>10:00-20:00</t>
         </is>
       </c>
       <c r="F8" s="22" t="inlineStr">
@@ -1585,22 +1585,22 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Ever Smile</t>
+          <t>Kids Stom</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>+7 747 900 30 09</t>
+          <t>+7 707 220 80 00</t>
         </is>
       </c>
       <c r="D9" s="21" t="inlineStr">
         <is>
-          <t>Алмалинский</t>
+          <t>Бостандыкский</t>
         </is>
       </c>
       <c r="E9" s="21" t="inlineStr">
         <is>
-          <t>10:00-22:00 обед 12:00-14:30</t>
+          <t>09:00-21:00 ежедневно</t>
         </is>
       </c>
       <c r="F9" s="22" t="inlineStr">
@@ -1679,22 +1679,22 @@
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>Dobro Dent</t>
+          <t>Ажар Дент</t>
         </is>
       </c>
       <c r="C11" s="20" t="inlineStr">
         <is>
-          <t>+7 775 030 09 99</t>
+          <t>+7 705 222 99 22</t>
         </is>
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Жетысуский</t>
         </is>
       </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
-          <t>09:00-22:00 ежедневно</t>
+          <t>09:00-19:00</t>
         </is>
       </c>
       <c r="F11" s="22" t="inlineStr">
@@ -1726,27 +1726,27 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Doctor Dent</t>
+          <t>DS Stomatology</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>+7 705 170 78 59</t>
+          <t>+7 771 267 61 27</t>
         </is>
       </c>
       <c r="D12" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Талгарский</t>
         </is>
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>не указаны</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>B</t>
+          <t>09:00-21:00 ежедневно</t>
+        </is>
+      </c>
+      <c r="F12" s="22" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="G12" s="23" t="n"/>
@@ -1773,17 +1773,17 @@
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>Dr. Baratov</t>
+          <t>Amire Dent</t>
         </is>
       </c>
       <c r="C13" s="20" t="inlineStr">
         <is>
-          <t>+7 707 189 36 45</t>
+          <t>+7 708 929 36 78</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>Алмалинский</t>
+          <t>Алатауский</t>
         </is>
       </c>
       <c r="E13" s="21" t="inlineStr">
@@ -1820,22 +1820,22 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Dr. Park</t>
+          <t>Dara dental clinic (Байтерекова)</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>+7 707 909 78 76</t>
+          <t>+7 707 601 45 50</t>
         </is>
       </c>
       <c r="D14" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Алатауский</t>
         </is>
       </c>
       <c r="E14" s="21" t="inlineStr">
         <is>
-          <t>открывается в 09:00</t>
+          <t>откр. 09:00, по записи</t>
         </is>
       </c>
       <c r="F14" s="18" t="inlineStr">
@@ -1867,22 +1867,22 @@
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>Никамед</t>
+          <t>Emir dental clinic</t>
         </is>
       </c>
       <c r="C15" s="20" t="inlineStr">
         <is>
-          <t>+7 727 973 55 53</t>
+          <t>+7 771 344 73 33</t>
         </is>
       </c>
       <c r="D15" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Алатауский</t>
         </is>
       </c>
       <c r="E15" s="21" t="inlineStr">
         <is>
-          <t>открывается в 08:00</t>
+          <t>откр. 11:00</t>
         </is>
       </c>
       <c r="F15" s="18" t="inlineStr">
@@ -1914,22 +1914,22 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>Diamond Dent</t>
+          <t>Khanstom</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>+7 771 275 39 49</t>
+          <t>+7 700 268 48 82</t>
         </is>
       </c>
       <c r="D16" s="21" t="inlineStr">
         <is>
-          <t>Ауэзовский</t>
+          <t>Алатауский</t>
         </is>
       </c>
       <c r="E16" s="21" t="inlineStr">
         <is>
-          <t>открывается в 09:00</t>
+          <t>откр. 09:00, по записи</t>
         </is>
       </c>
       <c r="F16" s="18" t="inlineStr">
@@ -1961,22 +1961,22 @@
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>Mirai Dental Clinic</t>
+          <t>Light Dental Clinic (Байтерекова)</t>
         </is>
       </c>
       <c r="C17" s="20" t="inlineStr">
         <is>
-          <t>+7 700 302 22 30</t>
+          <t>+7 700 100 00 28</t>
         </is>
       </c>
       <c r="D17" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Алатауский</t>
         </is>
       </c>
       <c r="E17" s="21" t="inlineStr">
         <is>
-          <t>не указаны</t>
+          <t>откр. 09:00</t>
         </is>
       </c>
       <c r="F17" s="18" t="inlineStr">
@@ -2008,22 +2008,22 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Senim Dental Clinic</t>
+          <t>Sapfir Stom</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>+7 701 408 84 44</t>
+          <t>+7 707 029 07 85</t>
         </is>
       </c>
       <c r="D18" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Алатауский</t>
         </is>
       </c>
       <c r="E18" s="21" t="inlineStr">
         <is>
-          <t>не указаны</t>
+          <t>график менялся, уточнить</t>
         </is>
       </c>
       <c r="F18" s="18" t="inlineStr">
@@ -2055,12 +2055,12 @@
       </c>
       <c r="B19" s="19" t="inlineStr">
         <is>
-          <t>Клиника доктора Мирзоева</t>
+          <t>Altyn Dent</t>
         </is>
       </c>
       <c r="C19" s="20" t="inlineStr">
         <is>
-          <t>+7 701 758 55 21</t>
+          <t>+7 747 920 75 71</t>
         </is>
       </c>
       <c r="D19" s="21" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="E19" s="21" t="inlineStr">
         <is>
-          <t>открывается в 10:00 по записи</t>
+          <t>открывается в 09:00</t>
         </is>
       </c>
       <c r="F19" s="18" t="inlineStr">
@@ -2102,12 +2102,12 @@
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t>MC Dent</t>
+          <t>DOSTYQ DENTAL CENTER</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>+7 702 366 59 74</t>
+          <t>+7 707 677 71 09</t>
         </is>
       </c>
       <c r="D20" s="21" t="inlineStr">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="E20" s="21" t="inlineStr">
         <is>
-          <t>не указаны</t>
+          <t>открывается в 10:00</t>
         </is>
       </c>
       <c r="F20" s="18" t="inlineStr">
@@ -2149,22 +2149,22 @@
       </c>
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>Elit Stom (Манаса 19)</t>
+          <t>Dara dental clinic (Толе би)</t>
         </is>
       </c>
       <c r="C21" s="20" t="inlineStr">
         <is>
-          <t>+7 700 818 90 60</t>
+          <t>+7 747 793 73 81</t>
         </is>
       </c>
       <c r="D21" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Алмалинский</t>
         </is>
       </c>
       <c r="E21" s="21" t="inlineStr">
         <is>
-          <t>не указаны</t>
+          <t>откр. 09:00, по записи</t>
         </is>
       </c>
       <c r="F21" s="18" t="inlineStr">
@@ -2196,22 +2196,22 @@
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>Family Dent Dr. Kapanov</t>
+          <t>Dent-Lux</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>+7 771 645 53 96</t>
+          <t>+7 702 075 09 07</t>
         </is>
       </c>
       <c r="D22" s="21" t="inlineStr">
         <is>
-          <t>Ауэзовский</t>
+          <t>Алмалинский</t>
         </is>
       </c>
       <c r="E22" s="21" t="inlineStr">
         <is>
-          <t>не указаны</t>
+          <t>откр. 08:00</t>
         </is>
       </c>
       <c r="F22" s="18" t="inlineStr">
@@ -2243,22 +2243,22 @@
       </c>
       <c r="B23" s="19" t="inlineStr">
         <is>
-          <t>Стоматология Аброра Исмаиловича</t>
+          <t>Dental Planet</t>
         </is>
       </c>
       <c r="C23" s="20" t="inlineStr">
         <is>
-          <t>+7 775 370 12 13</t>
+          <t>+7 705 888 38 15</t>
         </is>
       </c>
       <c r="D23" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Алмалинский</t>
         </is>
       </c>
       <c r="E23" s="21" t="inlineStr">
         <is>
-          <t>не указаны</t>
+          <t>открывается в 08:00</t>
         </is>
       </c>
       <c r="F23" s="18" t="inlineStr">
@@ -2290,12 +2290,12 @@
       </c>
       <c r="B24" s="19" t="inlineStr">
         <is>
-          <t>Smilex Dental Center</t>
+          <t>Dr. Baratov</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>+7 747 897 32 07</t>
+          <t>+7 707 189 36 45</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="E24" s="21" t="inlineStr">
         <is>
-          <t>открывается в 09:30</t>
+          <t>не указаны</t>
         </is>
       </c>
       <c r="F24" s="18" t="inlineStr">
@@ -2337,12 +2337,12 @@
       </c>
       <c r="B25" s="19" t="inlineStr">
         <is>
-          <t>Altyn Dent</t>
+          <t>Dr. Yerzhana Musagalieva</t>
         </is>
       </c>
       <c r="C25" s="20" t="inlineStr">
         <is>
-          <t>+7 747 920 75 71</t>
+          <t>+7 700 710 11 00</t>
         </is>
       </c>
       <c r="D25" s="21" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="E25" s="21" t="inlineStr">
         <is>
-          <t>открывается в 09:00</t>
+          <t>не указаны</t>
         </is>
       </c>
       <c r="F25" s="18" t="inlineStr">
@@ -2384,22 +2384,22 @@
       </c>
       <c r="B26" s="19" t="inlineStr">
         <is>
-          <t>Azu Dental Clinic</t>
+          <t>Hayat dental clinic</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
-          <t>+7 708 002 22 02</t>
+          <t>+7 776 141 20 20</t>
         </is>
       </c>
       <c r="D26" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Алмалинский</t>
         </is>
       </c>
       <c r="E26" s="21" t="inlineStr">
         <is>
-          <t>не указаны</t>
+          <t>откр. 09:00</t>
         </is>
       </c>
       <c r="F26" s="18" t="inlineStr">
@@ -2431,12 +2431,12 @@
       </c>
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t>Dental Planet</t>
+          <t>Izi Clinic</t>
         </is>
       </c>
       <c r="C27" s="20" t="inlineStr">
         <is>
-          <t>+7 705 888 38 15</t>
+          <t>+7 747 094 01 90</t>
         </is>
       </c>
       <c r="D27" s="21" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="E27" s="21" t="inlineStr">
         <is>
-          <t>открывается в 08:00</t>
+          <t>по предварительной записи</t>
         </is>
       </c>
       <c r="F27" s="18" t="inlineStr">
@@ -2478,17 +2478,17 @@
       </c>
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>Estetik Dental Clinic</t>
+          <t>MC Dent</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>+7 707 530 00 54</t>
+          <t>+7 702 366 59 74</t>
         </is>
       </c>
       <c r="D28" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Алмалинский</t>
         </is>
       </c>
       <c r="E28" s="21" t="inlineStr">
@@ -2525,22 +2525,22 @@
       </c>
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>Infinity Dental Clinic</t>
+          <t>Smilex Dental Center</t>
         </is>
       </c>
       <c r="C29" s="20" t="inlineStr">
         <is>
-          <t>+7 707 515 64 85</t>
+          <t>+7 747 897 32 07</t>
         </is>
       </c>
       <c r="D29" s="21" t="inlineStr">
         <is>
-          <t>Ауэзовский</t>
+          <t>Алмалинский</t>
         </is>
       </c>
       <c r="E29" s="21" t="inlineStr">
         <is>
-          <t>не указаны</t>
+          <t>открывается в 09:30</t>
         </is>
       </c>
       <c r="F29" s="18" t="inlineStr">
@@ -2572,12 +2572,12 @@
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>Izi Clinic</t>
+          <t>Клиника доктора Мирзоева</t>
         </is>
       </c>
       <c r="C30" s="20" t="inlineStr">
         <is>
-          <t>+7 747 094 01 90</t>
+          <t>+7 701 758 55 21</t>
         </is>
       </c>
       <c r="D30" s="21" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="E30" s="21" t="inlineStr">
         <is>
-          <t>по предварительной записи</t>
+          <t>открывается в 10:00 по записи</t>
         </is>
       </c>
       <c r="F30" s="18" t="inlineStr">
@@ -2619,12 +2619,12 @@
       </c>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>Like-Clinic</t>
+          <t>AE Dental Clinic</t>
         </is>
       </c>
       <c r="C31" s="20" t="inlineStr">
         <is>
-          <t>+7 775 103 73 23</t>
+          <t>+7 747 557 19 75</t>
         </is>
       </c>
       <c r="D31" s="21" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="E31" s="21" t="inlineStr">
         <is>
-          <t>не указаны</t>
+          <t>откр. 10:00</t>
         </is>
       </c>
       <c r="F31" s="18" t="inlineStr">
@@ -2666,22 +2666,22 @@
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>Dr. Yerzhana Musagalieva</t>
+          <t>AS-Dent</t>
         </is>
       </c>
       <c r="C32" s="20" t="inlineStr">
         <is>
-          <t>+7 700 710 11 00</t>
+          <t>+7 771 447 02 58</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
         <is>
-          <t>Алмалинский</t>
+          <t>Ауэзовский</t>
         </is>
       </c>
       <c r="E32" s="21" t="inlineStr">
         <is>
-          <t>не указаны</t>
+          <t>откр. 09:00</t>
         </is>
       </c>
       <c r="F32" s="18" t="inlineStr">
@@ -2713,22 +2713,22 @@
       </c>
       <c r="B33" s="19" t="inlineStr">
         <is>
-          <t>AQstom</t>
+          <t>Dental city</t>
         </is>
       </c>
       <c r="C33" s="20" t="inlineStr">
         <is>
-          <t>+7 707 000 00 22</t>
+          <t>+7 747 238 25 85</t>
         </is>
       </c>
       <c r="D33" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Ауэзовский</t>
         </is>
       </c>
       <c r="E33" s="21" t="inlineStr">
         <is>
-          <t>не указаны</t>
+          <t>откр. 09:00</t>
         </is>
       </c>
       <c r="F33" s="18" t="inlineStr">
@@ -2760,22 +2760,22 @@
       </c>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>Global Dent</t>
+          <t>Dental студия (Аксай-5)</t>
         </is>
       </c>
       <c r="C34" s="20" t="inlineStr">
         <is>
-          <t>+7 707 470 90 88</t>
+          <t>+7 708 600 51 47</t>
         </is>
       </c>
       <c r="D34" s="21" t="inlineStr">
         <is>
-          <t>Бостандыкский</t>
+          <t>Ауэзовский</t>
         </is>
       </c>
       <c r="E34" s="21" t="inlineStr">
         <is>
-          <t>открывается в 09:00 по звонку</t>
+          <t>откр. 10:00</t>
         </is>
       </c>
       <c r="F34" s="18" t="inlineStr">
@@ -2807,22 +2807,22 @@
       </c>
       <c r="B35" s="19" t="inlineStr">
         <is>
-          <t>Elit Stom (Сейфуллина 102)</t>
+          <t>Diamond Dent</t>
         </is>
       </c>
       <c r="C35" s="20" t="inlineStr">
         <is>
-          <t>+7 747 323 28 34</t>
+          <t>+7 771 275 39 49</t>
         </is>
       </c>
       <c r="D35" s="21" t="inlineStr">
         <is>
-          <t>Турксибский</t>
+          <t>Ауэзовский</t>
         </is>
       </c>
       <c r="E35" s="21" t="inlineStr">
         <is>
-          <t>не указаны</t>
+          <t>открывается в 09:00</t>
         </is>
       </c>
       <c r="F35" s="18" t="inlineStr">
@@ -2854,17 +2854,17 @@
       </c>
       <c r="B36" s="19" t="inlineStr">
         <is>
-          <t>Expert 32 stom</t>
+          <t>Family Dent Dr. Kapanov</t>
         </is>
       </c>
       <c r="C36" s="20" t="inlineStr">
         <is>
-          <t>+7 775 846 19 49</t>
+          <t>+7 771 645 53 96</t>
         </is>
       </c>
       <c r="D36" s="21" t="inlineStr">
         <is>
-          <t>Турксибский</t>
+          <t>Ауэзовский</t>
         </is>
       </c>
       <c r="E36" s="21" t="inlineStr">
@@ -2901,17 +2901,17 @@
       </c>
       <c r="B37" s="19" t="inlineStr">
         <is>
-          <t>DentalPRO</t>
+          <t>Implant_Stom</t>
         </is>
       </c>
       <c r="C37" s="20" t="inlineStr">
         <is>
-          <t>+7 771 800 00 67</t>
+          <t>+7 776 922 12 00</t>
         </is>
       </c>
       <c r="D37" s="21" t="inlineStr">
         <is>
-          <t>Турксибский</t>
+          <t>Ауэзовский</t>
         </is>
       </c>
       <c r="E37" s="21" t="inlineStr">
@@ -2948,22 +2948,22 @@
       </c>
       <c r="B38" s="19" t="inlineStr">
         <is>
-          <t>Dr.Omar Dental Clinic</t>
+          <t>Infinity Dental Clinic</t>
         </is>
       </c>
       <c r="C38" s="20" t="inlineStr">
         <is>
-          <t>+7 778 143 52 61</t>
+          <t>+7 707 515 64 85</t>
         </is>
       </c>
       <c r="D38" s="21" t="inlineStr">
         <is>
-          <t>Талгарский (Бесагаш)</t>
+          <t>Ауэзовский</t>
         </is>
       </c>
       <c r="E38" s="21" t="inlineStr">
         <is>
-          <t>открывается в 09:00</t>
+          <t>не указаны</t>
         </is>
       </c>
       <c r="F38" s="18" t="inlineStr">
@@ -2995,22 +2995,22 @@
       </c>
       <c r="B39" s="19" t="inlineStr">
         <is>
-          <t>InClinic</t>
+          <t>Like-Clinic</t>
         </is>
       </c>
       <c r="C39" s="20" t="inlineStr">
         <is>
-          <t>+7 707 333 22 66</t>
+          <t>+7 775 103 73 23</t>
         </is>
       </c>
       <c r="D39" s="21" t="inlineStr">
         <is>
-          <t>Медеуский</t>
+          <t>Ауэзовский</t>
         </is>
       </c>
       <c r="E39" s="21" t="inlineStr">
         <is>
-          <t>открывается в 09:00</t>
+          <t>не указаны</t>
         </is>
       </c>
       <c r="F39" s="18" t="inlineStr">
@@ -3042,22 +3042,22 @@
       </c>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>DOSTYQ DENTAL CENTER</t>
+          <t>Mamyr Dental Clinic</t>
         </is>
       </c>
       <c r="C40" s="20" t="inlineStr">
         <is>
-          <t>+7 707 677 71 09</t>
+          <t>+7 708 716 22 22</t>
         </is>
       </c>
       <c r="D40" s="21" t="inlineStr">
         <is>
-          <t>Алмалинский</t>
+          <t>Ауэзовский</t>
         </is>
       </c>
       <c r="E40" s="21" t="inlineStr">
         <is>
-          <t>открывается в 10:00</t>
+          <t>откр. 10:00, по записи</t>
         </is>
       </c>
       <c r="F40" s="18" t="inlineStr">
@@ -3089,22 +3089,22 @@
       </c>
       <c r="B41" s="19" t="inlineStr">
         <is>
-          <t>КГМЦ</t>
+          <t>Nurs Stom</t>
         </is>
       </c>
       <c r="C41" s="20" t="inlineStr">
         <is>
-          <t>+7 727 397 37 78</t>
+          <t>+7 777 182 93 84</t>
         </is>
       </c>
       <c r="D41" s="21" t="inlineStr">
         <is>
-          <t>Турксибский</t>
+          <t>Ауэзовский</t>
         </is>
       </c>
       <c r="E41" s="21" t="inlineStr">
         <is>
-          <t>открывается в 09:00 по записи</t>
+          <t>не указаны</t>
         </is>
       </c>
       <c r="F41" s="18" t="inlineStr">
@@ -3136,27 +3136,27 @@
       </c>
       <c r="B42" s="19" t="inlineStr">
         <is>
-          <t>Стома Плюс</t>
+          <t>TS clinic</t>
         </is>
       </c>
       <c r="C42" s="20" t="inlineStr">
         <is>
-          <t>+7 771 335 30 17</t>
+          <t>+7 701 788 70 96</t>
         </is>
       </c>
       <c r="D42" s="21" t="inlineStr">
         <is>
-          <t>Алатауский</t>
+          <t>Ауэзовский</t>
         </is>
       </c>
       <c r="E42" s="21" t="inlineStr">
         <is>
-          <t>09:00-23:00</t>
+          <t>откр. 09:00, по записи</t>
         </is>
       </c>
       <c r="F42" s="18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G42" s="23" t="n"/>
@@ -3183,12 +3183,12 @@
       </c>
       <c r="B43" s="19" t="inlineStr">
         <is>
-          <t>Estet Clinic</t>
+          <t>Агат</t>
         </is>
       </c>
       <c r="C43" s="20" t="inlineStr">
         <is>
-          <t>+7 707 101 02 33</t>
+          <t>+7 747 606 60 30</t>
         </is>
       </c>
       <c r="D43" s="21" t="inlineStr">
@@ -3198,12 +3198,12 @@
       </c>
       <c r="E43" s="21" t="inlineStr">
         <is>
-          <t>09:00-23:00 ежедневно</t>
+          <t>не указаны</t>
         </is>
       </c>
       <c r="F43" s="18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G43" s="23" t="n"/>
@@ -3230,27 +3230,27 @@
       </c>
       <c r="B44" s="19" t="inlineStr">
         <is>
-          <t>Muslim Dent</t>
+          <t>Ом Clinic</t>
         </is>
       </c>
       <c r="C44" s="20" t="inlineStr">
         <is>
-          <t>+7 771 800 00 65</t>
+          <t>+7 707 404 13 54</t>
         </is>
       </c>
       <c r="D44" s="21" t="inlineStr">
         <is>
-          <t>Алмалинский</t>
+          <t>Ауэзовский</t>
         </is>
       </c>
       <c r="E44" s="21" t="inlineStr">
         <is>
-          <t>10:00-23:45 ежедневно</t>
+          <t>откр. 09:00, по записи</t>
         </is>
       </c>
       <c r="F44" s="18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G44" s="23" t="n"/>
@@ -3277,12 +3277,12 @@
       </c>
       <c r="B45" s="19" t="inlineStr">
         <is>
-          <t>Bilal stom</t>
+          <t>AQstom</t>
         </is>
       </c>
       <c r="C45" s="20" t="inlineStr">
         <is>
-          <t>+7 707 666 98 92</t>
+          <t>+7 707 000 00 22</t>
         </is>
       </c>
       <c r="D45" s="21" t="inlineStr">
@@ -3292,12 +3292,12 @@
       </c>
       <c r="E45" s="21" t="inlineStr">
         <is>
-          <t>09:00-24:00 ежедневно</t>
+          <t>не указаны</t>
         </is>
       </c>
       <c r="F45" s="18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G45" s="23" t="n"/>
@@ -3324,12 +3324,12 @@
       </c>
       <c r="B46" s="19" t="inlineStr">
         <is>
-          <t>Dr.SULTANOV ATABEK</t>
+          <t>AV Dental Clinic</t>
         </is>
       </c>
       <c r="C46" s="20" t="inlineStr">
         <is>
-          <t>+7 775 300 85 05</t>
+          <t>+7 778 080 32 32</t>
         </is>
       </c>
       <c r="D46" s="21" t="inlineStr">
@@ -3339,12 +3339,12 @@
       </c>
       <c r="E46" s="21" t="inlineStr">
         <is>
-          <t>09:00-24:00</t>
+          <t>откр. 10:00, по записи</t>
         </is>
       </c>
       <c r="F46" s="18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G46" s="23" t="n"/>
@@ -3371,27 +3371,27 @@
       </c>
       <c r="B47" s="19" t="inlineStr">
         <is>
-          <t>Dr. Beridze</t>
+          <t>Alatau Assistance</t>
         </is>
       </c>
       <c r="C47" s="20" t="inlineStr">
         <is>
-          <t>+7 775 522 05 09</t>
+          <t>+7 727 356 11 77</t>
         </is>
       </c>
       <c r="D47" s="21" t="inlineStr">
         <is>
-          <t>Турксибский</t>
+          <t>Бостандыкский</t>
         </is>
       </c>
       <c r="E47" s="21" t="inlineStr">
         <is>
-          <t>09:00-24:00 ежедневно</t>
+          <t>откр. 08:00</t>
         </is>
       </c>
       <c r="F47" s="18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G47" s="23" t="n"/>
@@ -3418,12 +3418,12 @@
       </c>
       <c r="B48" s="19" t="inlineStr">
         <is>
-          <t>Elit Dent</t>
+          <t>Asia dent</t>
         </is>
       </c>
       <c r="C48" s="20" t="inlineStr">
         <is>
-          <t>+7 708 269 71 00</t>
+          <t>+7 701 617 61 81</t>
         </is>
       </c>
       <c r="D48" s="21" t="inlineStr">
@@ -3433,12 +3433,12 @@
       </c>
       <c r="E48" s="21" t="inlineStr">
         <is>
-          <t>круглосуточно</t>
+          <t>откр. 09:00, по записи</t>
         </is>
       </c>
       <c r="F48" s="18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G48" s="23" t="n"/>
@@ -3459,9 +3459,2547 @@
       <c r="P48" s="25" t="n"/>
       <c r="Q48" s="26" t="n"/>
     </row>
+    <row r="49" ht="26" customHeight="1">
+      <c r="A49" s="18" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="19" t="inlineStr">
+        <is>
+          <t>Azu Dental Clinic</t>
+        </is>
+      </c>
+      <c r="C49" s="20" t="inlineStr">
+        <is>
+          <t>+7 708 002 22 02</t>
+        </is>
+      </c>
+      <c r="D49" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E49" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F49" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G49" s="23" t="n"/>
+      <c r="H49" s="23" t="n"/>
+      <c r="I49" s="23" t="n"/>
+      <c r="J49" s="23" t="n"/>
+      <c r="K49" s="23" t="n"/>
+      <c r="L49" s="23" t="n"/>
+      <c r="M49" s="23" t="n"/>
+      <c r="N49" s="24">
+        <f>COUNTIF(H49:M49,"Г")</f>
+        <v/>
+      </c>
+      <c r="O49" s="24">
+        <f>COUNTIF(H49:M49,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P49" s="25" t="n"/>
+      <c r="Q49" s="26" t="n"/>
+    </row>
+    <row r="50" ht="26" customHeight="1">
+      <c r="A50" s="18" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="19" t="inlineStr">
+        <is>
+          <t>DR.BABUR DENTAL CLINIC</t>
+        </is>
+      </c>
+      <c r="C50" s="20" t="inlineStr">
+        <is>
+          <t>+7 747 093 89 86</t>
+        </is>
+      </c>
+      <c r="D50" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E50" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00, по записи</t>
+        </is>
+      </c>
+      <c r="F50" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G50" s="23" t="n"/>
+      <c r="H50" s="23" t="n"/>
+      <c r="I50" s="23" t="n"/>
+      <c r="J50" s="23" t="n"/>
+      <c r="K50" s="23" t="n"/>
+      <c r="L50" s="23" t="n"/>
+      <c r="M50" s="23" t="n"/>
+      <c r="N50" s="24">
+        <f>COUNTIF(H50:M50,"Г")</f>
+        <v/>
+      </c>
+      <c r="O50" s="24">
+        <f>COUNTIF(H50:M50,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P50" s="25" t="n"/>
+      <c r="Q50" s="26" t="n"/>
+    </row>
+    <row r="51" ht="26" customHeight="1">
+      <c r="A51" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="19" t="inlineStr">
+        <is>
+          <t>Dental студия (Розыбакиева)</t>
+        </is>
+      </c>
+      <c r="C51" s="20" t="inlineStr">
+        <is>
+          <t>+7 708 940 74 12</t>
+        </is>
+      </c>
+      <c r="D51" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E51" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00</t>
+        </is>
+      </c>
+      <c r="F51" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G51" s="23" t="n"/>
+      <c r="H51" s="23" t="n"/>
+      <c r="I51" s="23" t="n"/>
+      <c r="J51" s="23" t="n"/>
+      <c r="K51" s="23" t="n"/>
+      <c r="L51" s="23" t="n"/>
+      <c r="M51" s="23" t="n"/>
+      <c r="N51" s="24">
+        <f>COUNTIF(H51:M51,"Г")</f>
+        <v/>
+      </c>
+      <c r="O51" s="24">
+        <f>COUNTIF(H51:M51,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P51" s="25" t="n"/>
+      <c r="Q51" s="26" t="n"/>
+    </row>
+    <row r="52" ht="26" customHeight="1">
+      <c r="A52" s="18" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="19" t="inlineStr">
+        <is>
+          <t>Doctor Dent</t>
+        </is>
+      </c>
+      <c r="C52" s="20" t="inlineStr">
+        <is>
+          <t>+7 705 170 78 59</t>
+        </is>
+      </c>
+      <c r="D52" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E52" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F52" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G52" s="23" t="n"/>
+      <c r="H52" s="23" t="n"/>
+      <c r="I52" s="23" t="n"/>
+      <c r="J52" s="23" t="n"/>
+      <c r="K52" s="23" t="n"/>
+      <c r="L52" s="23" t="n"/>
+      <c r="M52" s="23" t="n"/>
+      <c r="N52" s="24">
+        <f>COUNTIF(H52:M52,"Г")</f>
+        <v/>
+      </c>
+      <c r="O52" s="24">
+        <f>COUNTIF(H52:M52,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P52" s="25" t="n"/>
+      <c r="Q52" s="26" t="n"/>
+    </row>
+    <row r="53" ht="26" customHeight="1">
+      <c r="A53" s="18" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="19" t="inlineStr">
+        <is>
+          <t>Dr. Park</t>
+        </is>
+      </c>
+      <c r="C53" s="20" t="inlineStr">
+        <is>
+          <t>+7 707 909 78 76</t>
+        </is>
+      </c>
+      <c r="D53" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E53" s="21" t="inlineStr">
+        <is>
+          <t>открывается в 09:00</t>
+        </is>
+      </c>
+      <c r="F53" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G53" s="23" t="n"/>
+      <c r="H53" s="23" t="n"/>
+      <c r="I53" s="23" t="n"/>
+      <c r="J53" s="23" t="n"/>
+      <c r="K53" s="23" t="n"/>
+      <c r="L53" s="23" t="n"/>
+      <c r="M53" s="23" t="n"/>
+      <c r="N53" s="24">
+        <f>COUNTIF(H53:M53,"Г")</f>
+        <v/>
+      </c>
+      <c r="O53" s="24">
+        <f>COUNTIF(H53:M53,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P53" s="25" t="n"/>
+      <c r="Q53" s="26" t="n"/>
+    </row>
+    <row r="54" ht="26" customHeight="1">
+      <c r="A54" s="18" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="19" t="inlineStr">
+        <is>
+          <t>Dr. Poluyev dental clinic</t>
+        </is>
+      </c>
+      <c r="C54" s="20" t="inlineStr">
+        <is>
+          <t>+7 727 311 94 11</t>
+        </is>
+      </c>
+      <c r="D54" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E54" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00</t>
+        </is>
+      </c>
+      <c r="F54" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G54" s="23" t="n"/>
+      <c r="H54" s="23" t="n"/>
+      <c r="I54" s="23" t="n"/>
+      <c r="J54" s="23" t="n"/>
+      <c r="K54" s="23" t="n"/>
+      <c r="L54" s="23" t="n"/>
+      <c r="M54" s="23" t="n"/>
+      <c r="N54" s="24">
+        <f>COUNTIF(H54:M54,"Г")</f>
+        <v/>
+      </c>
+      <c r="O54" s="24">
+        <f>COUNTIF(H54:M54,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P54" s="25" t="n"/>
+      <c r="Q54" s="26" t="n"/>
+    </row>
+    <row r="55" ht="26" customHeight="1">
+      <c r="A55" s="18" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="19" t="inlineStr">
+        <is>
+          <t>Dr.Bond</t>
+        </is>
+      </c>
+      <c r="C55" s="20" t="inlineStr">
+        <is>
+          <t>+7 727 265 39 82</t>
+        </is>
+      </c>
+      <c r="D55" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E55" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00, по записи</t>
+        </is>
+      </c>
+      <c r="F55" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G55" s="23" t="n"/>
+      <c r="H55" s="23" t="n"/>
+      <c r="I55" s="23" t="n"/>
+      <c r="J55" s="23" t="n"/>
+      <c r="K55" s="23" t="n"/>
+      <c r="L55" s="23" t="n"/>
+      <c r="M55" s="23" t="n"/>
+      <c r="N55" s="24">
+        <f>COUNTIF(H55:M55,"Г")</f>
+        <v/>
+      </c>
+      <c r="O55" s="24">
+        <f>COUNTIF(H55:M55,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P55" s="25" t="n"/>
+      <c r="Q55" s="26" t="n"/>
+    </row>
+    <row r="56" ht="26" customHeight="1">
+      <c r="A56" s="18" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="19" t="inlineStr">
+        <is>
+          <t>Elit Stom (Манаса 19)</t>
+        </is>
+      </c>
+      <c r="C56" s="20" t="inlineStr">
+        <is>
+          <t>+7 700 818 90 60</t>
+        </is>
+      </c>
+      <c r="D56" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E56" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F56" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G56" s="23" t="n"/>
+      <c r="H56" s="23" t="n"/>
+      <c r="I56" s="23" t="n"/>
+      <c r="J56" s="23" t="n"/>
+      <c r="K56" s="23" t="n"/>
+      <c r="L56" s="23" t="n"/>
+      <c r="M56" s="23" t="n"/>
+      <c r="N56" s="24">
+        <f>COUNTIF(H56:M56,"Г")</f>
+        <v/>
+      </c>
+      <c r="O56" s="24">
+        <f>COUNTIF(H56:M56,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P56" s="25" t="n"/>
+      <c r="Q56" s="26" t="n"/>
+    </row>
+    <row r="57" ht="26" customHeight="1">
+      <c r="A57" s="18" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="19" t="inlineStr">
+        <is>
+          <t>Estetik Dental Clinic</t>
+        </is>
+      </c>
+      <c r="C57" s="20" t="inlineStr">
+        <is>
+          <t>+7 707 530 00 54</t>
+        </is>
+      </c>
+      <c r="D57" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E57" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F57" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G57" s="23" t="n"/>
+      <c r="H57" s="23" t="n"/>
+      <c r="I57" s="23" t="n"/>
+      <c r="J57" s="23" t="n"/>
+      <c r="K57" s="23" t="n"/>
+      <c r="L57" s="23" t="n"/>
+      <c r="M57" s="23" t="n"/>
+      <c r="N57" s="24">
+        <f>COUNTIF(H57:M57,"Г")</f>
+        <v/>
+      </c>
+      <c r="O57" s="24">
+        <f>COUNTIF(H57:M57,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P57" s="25" t="n"/>
+      <c r="Q57" s="26" t="n"/>
+    </row>
+    <row r="58" ht="26" customHeight="1">
+      <c r="A58" s="18" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="19" t="inlineStr">
+        <is>
+          <t>Global Dent</t>
+        </is>
+      </c>
+      <c r="C58" s="20" t="inlineStr">
+        <is>
+          <t>+7 707 470 90 88</t>
+        </is>
+      </c>
+      <c r="D58" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E58" s="21" t="inlineStr">
+        <is>
+          <t>открывается в 09:00 по звонку</t>
+        </is>
+      </c>
+      <c r="F58" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G58" s="23" t="n"/>
+      <c r="H58" s="23" t="n"/>
+      <c r="I58" s="23" t="n"/>
+      <c r="J58" s="23" t="n"/>
+      <c r="K58" s="23" t="n"/>
+      <c r="L58" s="23" t="n"/>
+      <c r="M58" s="23" t="n"/>
+      <c r="N58" s="24">
+        <f>COUNTIF(H58:M58,"Г")</f>
+        <v/>
+      </c>
+      <c r="O58" s="24">
+        <f>COUNTIF(H58:M58,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P58" s="25" t="n"/>
+      <c r="Q58" s="26" t="n"/>
+    </row>
+    <row r="59" ht="26" customHeight="1">
+      <c r="A59" s="18" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="19" t="inlineStr">
+        <is>
+          <t>Lavi dent</t>
+        </is>
+      </c>
+      <c r="C59" s="20" t="inlineStr">
+        <is>
+          <t>+7 707 971 82 66</t>
+        </is>
+      </c>
+      <c r="D59" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E59" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F59" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G59" s="23" t="n"/>
+      <c r="H59" s="23" t="n"/>
+      <c r="I59" s="23" t="n"/>
+      <c r="J59" s="23" t="n"/>
+      <c r="K59" s="23" t="n"/>
+      <c r="L59" s="23" t="n"/>
+      <c r="M59" s="23" t="n"/>
+      <c r="N59" s="24">
+        <f>COUNTIF(H59:M59,"Г")</f>
+        <v/>
+      </c>
+      <c r="O59" s="24">
+        <f>COUNTIF(H59:M59,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P59" s="25" t="n"/>
+      <c r="Q59" s="26" t="n"/>
+    </row>
+    <row r="60" ht="26" customHeight="1">
+      <c r="A60" s="18" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="19" t="inlineStr">
+        <is>
+          <t>Mirai Dental Clinic</t>
+        </is>
+      </c>
+      <c r="C60" s="20" t="inlineStr">
+        <is>
+          <t>+7 700 302 22 30</t>
+        </is>
+      </c>
+      <c r="D60" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E60" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F60" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G60" s="23" t="n"/>
+      <c r="H60" s="23" t="n"/>
+      <c r="I60" s="23" t="n"/>
+      <c r="J60" s="23" t="n"/>
+      <c r="K60" s="23" t="n"/>
+      <c r="L60" s="23" t="n"/>
+      <c r="M60" s="23" t="n"/>
+      <c r="N60" s="24">
+        <f>COUNTIF(H60:M60,"Г")</f>
+        <v/>
+      </c>
+      <c r="O60" s="24">
+        <f>COUNTIF(H60:M60,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P60" s="25" t="n"/>
+      <c r="Q60" s="26" t="n"/>
+    </row>
+    <row r="61" ht="26" customHeight="1">
+      <c r="A61" s="18" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="19" t="inlineStr">
+        <is>
+          <t>Rabiya Dental Clinic</t>
+        </is>
+      </c>
+      <c r="C61" s="20" t="inlineStr">
+        <is>
+          <t>+7 700 721 39 30</t>
+        </is>
+      </c>
+      <c r="D61" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E61" s="21" t="inlineStr">
+        <is>
+          <t>откр. 10:00, по записи</t>
+        </is>
+      </c>
+      <c r="F61" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G61" s="23" t="n"/>
+      <c r="H61" s="23" t="n"/>
+      <c r="I61" s="23" t="n"/>
+      <c r="J61" s="23" t="n"/>
+      <c r="K61" s="23" t="n"/>
+      <c r="L61" s="23" t="n"/>
+      <c r="M61" s="23" t="n"/>
+      <c r="N61" s="24">
+        <f>COUNTIF(H61:M61,"Г")</f>
+        <v/>
+      </c>
+      <c r="O61" s="24">
+        <f>COUNTIF(H61:M61,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P61" s="25" t="n"/>
+      <c r="Q61" s="26" t="n"/>
+    </row>
+    <row r="62" ht="26" customHeight="1">
+      <c r="A62" s="18" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="19" t="inlineStr">
+        <is>
+          <t>Senim Dental Clinic</t>
+        </is>
+      </c>
+      <c r="C62" s="20" t="inlineStr">
+        <is>
+          <t>+7 701 408 84 44</t>
+        </is>
+      </c>
+      <c r="D62" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E62" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F62" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G62" s="23" t="n"/>
+      <c r="H62" s="23" t="n"/>
+      <c r="I62" s="23" t="n"/>
+      <c r="J62" s="23" t="n"/>
+      <c r="K62" s="23" t="n"/>
+      <c r="L62" s="23" t="n"/>
+      <c r="M62" s="23" t="n"/>
+      <c r="N62" s="24">
+        <f>COUNTIF(H62:M62,"Г")</f>
+        <v/>
+      </c>
+      <c r="O62" s="24">
+        <f>COUNTIF(H62:M62,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P62" s="25" t="n"/>
+      <c r="Q62" s="26" t="n"/>
+    </row>
+    <row r="63" ht="26" customHeight="1">
+      <c r="A63" s="18" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="19" t="inlineStr">
+        <is>
+          <t>StarDent</t>
+        </is>
+      </c>
+      <c r="C63" s="20" t="inlineStr">
+        <is>
+          <t>+7 747 613 48 79</t>
+        </is>
+      </c>
+      <c r="D63" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E63" s="21" t="inlineStr">
+        <is>
+          <t>откр. 10:00</t>
+        </is>
+      </c>
+      <c r="F63" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G63" s="23" t="n"/>
+      <c r="H63" s="23" t="n"/>
+      <c r="I63" s="23" t="n"/>
+      <c r="J63" s="23" t="n"/>
+      <c r="K63" s="23" t="n"/>
+      <c r="L63" s="23" t="n"/>
+      <c r="M63" s="23" t="n"/>
+      <c r="N63" s="24">
+        <f>COUNTIF(H63:M63,"Г")</f>
+        <v/>
+      </c>
+      <c r="O63" s="24">
+        <f>COUNTIF(H63:M63,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P63" s="25" t="n"/>
+      <c r="Q63" s="26" t="n"/>
+    </row>
+    <row r="64" ht="26" customHeight="1">
+      <c r="A64" s="18" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="19" t="inlineStr">
+        <is>
+          <t>Sunna smile</t>
+        </is>
+      </c>
+      <c r="C64" s="20" t="inlineStr">
+        <is>
+          <t>+7 700 308 55 88</t>
+        </is>
+      </c>
+      <c r="D64" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E64" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00, по записи</t>
+        </is>
+      </c>
+      <c r="F64" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G64" s="23" t="n"/>
+      <c r="H64" s="23" t="n"/>
+      <c r="I64" s="23" t="n"/>
+      <c r="J64" s="23" t="n"/>
+      <c r="K64" s="23" t="n"/>
+      <c r="L64" s="23" t="n"/>
+      <c r="M64" s="23" t="n"/>
+      <c r="N64" s="24">
+        <f>COUNTIF(H64:M64,"Г")</f>
+        <v/>
+      </c>
+      <c r="O64" s="24">
+        <f>COUNTIF(H64:M64,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P64" s="25" t="n"/>
+      <c r="Q64" s="26" t="n"/>
+    </row>
+    <row r="65" ht="26" customHeight="1">
+      <c r="A65" s="18" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="19" t="inlineStr">
+        <is>
+          <t>Никамед</t>
+        </is>
+      </c>
+      <c r="C65" s="20" t="inlineStr">
+        <is>
+          <t>+7 727 973 55 53</t>
+        </is>
+      </c>
+      <c r="D65" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E65" s="21" t="inlineStr">
+        <is>
+          <t>открывается в 08:00</t>
+        </is>
+      </c>
+      <c r="F65" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G65" s="23" t="n"/>
+      <c r="H65" s="23" t="n"/>
+      <c r="I65" s="23" t="n"/>
+      <c r="J65" s="23" t="n"/>
+      <c r="K65" s="23" t="n"/>
+      <c r="L65" s="23" t="n"/>
+      <c r="M65" s="23" t="n"/>
+      <c r="N65" s="24">
+        <f>COUNTIF(H65:M65,"Г")</f>
+        <v/>
+      </c>
+      <c r="O65" s="24">
+        <f>COUNTIF(H65:M65,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P65" s="25" t="n"/>
+      <c r="Q65" s="26" t="n"/>
+    </row>
+    <row r="66" ht="26" customHeight="1">
+      <c r="A66" s="18" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="19" t="inlineStr">
+        <is>
+          <t>Рахат</t>
+        </is>
+      </c>
+      <c r="C66" s="20" t="inlineStr">
+        <is>
+          <t>+7 707 900 88 24</t>
+        </is>
+      </c>
+      <c r="D66" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E66" s="21" t="inlineStr">
+        <is>
+          <t>откр. 08:00, сеть 6 филиалов</t>
+        </is>
+      </c>
+      <c r="F66" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G66" s="23" t="n"/>
+      <c r="H66" s="23" t="n"/>
+      <c r="I66" s="23" t="n"/>
+      <c r="J66" s="23" t="n"/>
+      <c r="K66" s="23" t="n"/>
+      <c r="L66" s="23" t="n"/>
+      <c r="M66" s="23" t="n"/>
+      <c r="N66" s="24">
+        <f>COUNTIF(H66:M66,"Г")</f>
+        <v/>
+      </c>
+      <c r="O66" s="24">
+        <f>COUNTIF(H66:M66,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P66" s="25" t="n"/>
+      <c r="Q66" s="26" t="n"/>
+    </row>
+    <row r="67" ht="26" customHeight="1">
+      <c r="A67" s="18" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="19" t="inlineStr">
+        <is>
+          <t>Стоматология Аброра Исмаиловича</t>
+        </is>
+      </c>
+      <c r="C67" s="20" t="inlineStr">
+        <is>
+          <t>+7 775 370 12 13</t>
+        </is>
+      </c>
+      <c r="D67" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E67" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F67" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G67" s="23" t="n"/>
+      <c r="H67" s="23" t="n"/>
+      <c r="I67" s="23" t="n"/>
+      <c r="J67" s="23" t="n"/>
+      <c r="K67" s="23" t="n"/>
+      <c r="L67" s="23" t="n"/>
+      <c r="M67" s="23" t="n"/>
+      <c r="N67" s="24">
+        <f>COUNTIF(H67:M67,"Г")</f>
+        <v/>
+      </c>
+      <c r="O67" s="24">
+        <f>COUNTIF(H67:M67,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P67" s="25" t="n"/>
+      <c r="Q67" s="26" t="n"/>
+    </row>
+    <row r="68" ht="26" customHeight="1">
+      <c r="A68" s="18" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="19" t="inlineStr">
+        <is>
+          <t>Dr. Iskakov clinic</t>
+        </is>
+      </c>
+      <c r="C68" s="20" t="inlineStr">
+        <is>
+          <t>+7 776 060 44 66</t>
+        </is>
+      </c>
+      <c r="D68" s="21" t="inlineStr">
+        <is>
+          <t>Жетысуский</t>
+        </is>
+      </c>
+      <c r="E68" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00</t>
+        </is>
+      </c>
+      <c r="F68" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G68" s="23" t="n"/>
+      <c r="H68" s="23" t="n"/>
+      <c r="I68" s="23" t="n"/>
+      <c r="J68" s="23" t="n"/>
+      <c r="K68" s="23" t="n"/>
+      <c r="L68" s="23" t="n"/>
+      <c r="M68" s="23" t="n"/>
+      <c r="N68" s="24">
+        <f>COUNTIF(H68:M68,"Г")</f>
+        <v/>
+      </c>
+      <c r="O68" s="24">
+        <f>COUNTIF(H68:M68,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P68" s="25" t="n"/>
+      <c r="Q68" s="26" t="n"/>
+    </row>
+    <row r="69" ht="26" customHeight="1">
+      <c r="A69" s="18" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="19" t="inlineStr">
+        <is>
+          <t>Royal Stom</t>
+        </is>
+      </c>
+      <c r="C69" s="20" t="inlineStr">
+        <is>
+          <t>+7 705 413 69 55</t>
+        </is>
+      </c>
+      <c r="D69" s="21" t="inlineStr">
+        <is>
+          <t>Жетысуский</t>
+        </is>
+      </c>
+      <c r="E69" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F69" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G69" s="23" t="n"/>
+      <c r="H69" s="23" t="n"/>
+      <c r="I69" s="23" t="n"/>
+      <c r="J69" s="23" t="n"/>
+      <c r="K69" s="23" t="n"/>
+      <c r="L69" s="23" t="n"/>
+      <c r="M69" s="23" t="n"/>
+      <c r="N69" s="24">
+        <f>COUNTIF(H69:M69,"Г")</f>
+        <v/>
+      </c>
+      <c r="O69" s="24">
+        <f>COUNTIF(H69:M69,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P69" s="25" t="n"/>
+      <c r="Q69" s="26" t="n"/>
+    </row>
+    <row r="70" ht="26" customHeight="1">
+      <c r="A70" s="18" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="19" t="inlineStr">
+        <is>
+          <t>Batyr Dent</t>
+        </is>
+      </c>
+      <c r="C70" s="20" t="inlineStr">
+        <is>
+          <t>+7 747 430 79 82</t>
+        </is>
+      </c>
+      <c r="D70" s="21" t="inlineStr">
+        <is>
+          <t>Медеуский</t>
+        </is>
+      </c>
+      <c r="E70" s="21" t="inlineStr">
+        <is>
+          <t>откр. 10:00, по записи</t>
+        </is>
+      </c>
+      <c r="F70" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G70" s="23" t="n"/>
+      <c r="H70" s="23" t="n"/>
+      <c r="I70" s="23" t="n"/>
+      <c r="J70" s="23" t="n"/>
+      <c r="K70" s="23" t="n"/>
+      <c r="L70" s="23" t="n"/>
+      <c r="M70" s="23" t="n"/>
+      <c r="N70" s="24">
+        <f>COUNTIF(H70:M70,"Г")</f>
+        <v/>
+      </c>
+      <c r="O70" s="24">
+        <f>COUNTIF(H70:M70,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P70" s="25" t="n"/>
+      <c r="Q70" s="26" t="n"/>
+    </row>
+    <row r="71" ht="26" customHeight="1">
+      <c r="A71" s="18" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="19" t="inlineStr">
+        <is>
+          <t>DentalPark</t>
+        </is>
+      </c>
+      <c r="C71" s="20" t="inlineStr">
+        <is>
+          <t>+7 727 220 00 50</t>
+        </is>
+      </c>
+      <c r="D71" s="21" t="inlineStr">
+        <is>
+          <t>Медеуский</t>
+        </is>
+      </c>
+      <c r="E71" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00, по записи</t>
+        </is>
+      </c>
+      <c r="F71" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G71" s="23" t="n"/>
+      <c r="H71" s="23" t="n"/>
+      <c r="I71" s="23" t="n"/>
+      <c r="J71" s="23" t="n"/>
+      <c r="K71" s="23" t="n"/>
+      <c r="L71" s="23" t="n"/>
+      <c r="M71" s="23" t="n"/>
+      <c r="N71" s="24">
+        <f>COUNTIF(H71:M71,"Г")</f>
+        <v/>
+      </c>
+      <c r="O71" s="24">
+        <f>COUNTIF(H71:M71,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P71" s="25" t="n"/>
+      <c r="Q71" s="26" t="n"/>
+    </row>
+    <row r="72" ht="26" customHeight="1">
+      <c r="A72" s="18" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="19" t="inlineStr">
+        <is>
+          <t>Doc doctor onlas clinic</t>
+        </is>
+      </c>
+      <c r="C72" s="20" t="inlineStr">
+        <is>
+          <t>+7 702 247 74 24</t>
+        </is>
+      </c>
+      <c r="D72" s="21" t="inlineStr">
+        <is>
+          <t>Медеуский</t>
+        </is>
+      </c>
+      <c r="E72" s="21" t="inlineStr">
+        <is>
+          <t>откр. 10:00, по записи</t>
+        </is>
+      </c>
+      <c r="F72" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G72" s="23" t="n"/>
+      <c r="H72" s="23" t="n"/>
+      <c r="I72" s="23" t="n"/>
+      <c r="J72" s="23" t="n"/>
+      <c r="K72" s="23" t="n"/>
+      <c r="L72" s="23" t="n"/>
+      <c r="M72" s="23" t="n"/>
+      <c r="N72" s="24">
+        <f>COUNTIF(H72:M72,"Г")</f>
+        <v/>
+      </c>
+      <c r="O72" s="24">
+        <f>COUNTIF(H72:M72,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P72" s="25" t="n"/>
+      <c r="Q72" s="26" t="n"/>
+    </row>
+    <row r="73" ht="26" customHeight="1">
+      <c r="A73" s="18" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="19" t="inlineStr">
+        <is>
+          <t>InClinic</t>
+        </is>
+      </c>
+      <c r="C73" s="20" t="inlineStr">
+        <is>
+          <t>+7 707 333 22 66</t>
+        </is>
+      </c>
+      <c r="D73" s="21" t="inlineStr">
+        <is>
+          <t>Медеуский</t>
+        </is>
+      </c>
+      <c r="E73" s="21" t="inlineStr">
+        <is>
+          <t>открывается в 09:00</t>
+        </is>
+      </c>
+      <c r="F73" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G73" s="23" t="n"/>
+      <c r="H73" s="23" t="n"/>
+      <c r="I73" s="23" t="n"/>
+      <c r="J73" s="23" t="n"/>
+      <c r="K73" s="23" t="n"/>
+      <c r="L73" s="23" t="n"/>
+      <c r="M73" s="23" t="n"/>
+      <c r="N73" s="24">
+        <f>COUNTIF(H73:M73,"Г")</f>
+        <v/>
+      </c>
+      <c r="O73" s="24">
+        <f>COUNTIF(H73:M73,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P73" s="25" t="n"/>
+      <c r="Q73" s="26" t="n"/>
+    </row>
+    <row r="74" ht="26" customHeight="1">
+      <c r="A74" s="18" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="19" t="inlineStr">
+        <is>
+          <t>Like-Clinic (Гоголя)</t>
+        </is>
+      </c>
+      <c r="C74" s="20" t="inlineStr">
+        <is>
+          <t>+7 707 360 60 49</t>
+        </is>
+      </c>
+      <c r="D74" s="21" t="inlineStr">
+        <is>
+          <t>Медеуский</t>
+        </is>
+      </c>
+      <c r="E74" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G74" s="23" t="n"/>
+      <c r="H74" s="23" t="n"/>
+      <c r="I74" s="23" t="n"/>
+      <c r="J74" s="23" t="n"/>
+      <c r="K74" s="23" t="n"/>
+      <c r="L74" s="23" t="n"/>
+      <c r="M74" s="23" t="n"/>
+      <c r="N74" s="24">
+        <f>COUNTIF(H74:M74,"Г")</f>
+        <v/>
+      </c>
+      <c r="O74" s="24">
+        <f>COUNTIF(H74:M74,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P74" s="25" t="n"/>
+      <c r="Q74" s="26" t="n"/>
+    </row>
+    <row r="75" ht="26" customHeight="1">
+      <c r="A75" s="18" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="19" t="inlineStr">
+        <is>
+          <t>MediSa</t>
+        </is>
+      </c>
+      <c r="C75" s="20" t="inlineStr">
+        <is>
+          <t>+7 777 262 99 99</t>
+        </is>
+      </c>
+      <c r="D75" s="21" t="inlineStr">
+        <is>
+          <t>Медеуский</t>
+        </is>
+      </c>
+      <c r="E75" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00, по записи</t>
+        </is>
+      </c>
+      <c r="F75" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G75" s="23" t="n"/>
+      <c r="H75" s="23" t="n"/>
+      <c r="I75" s="23" t="n"/>
+      <c r="J75" s="23" t="n"/>
+      <c r="K75" s="23" t="n"/>
+      <c r="L75" s="23" t="n"/>
+      <c r="M75" s="23" t="n"/>
+      <c r="N75" s="24">
+        <f>COUNTIF(H75:M75,"Г")</f>
+        <v/>
+      </c>
+      <c r="O75" s="24">
+        <f>COUNTIF(H75:M75,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P75" s="25" t="n"/>
+      <c r="Q75" s="26" t="n"/>
+    </row>
+    <row r="76" ht="26" customHeight="1">
+      <c r="A76" s="18" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="19" t="inlineStr">
+        <is>
+          <t>Mydent</t>
+        </is>
+      </c>
+      <c r="C76" s="20" t="inlineStr">
+        <is>
+          <t>+7 771 750 88 88</t>
+        </is>
+      </c>
+      <c r="D76" s="21" t="inlineStr">
+        <is>
+          <t>Медеуский</t>
+        </is>
+      </c>
+      <c r="E76" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00, по записи</t>
+        </is>
+      </c>
+      <c r="F76" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G76" s="23" t="n"/>
+      <c r="H76" s="23" t="n"/>
+      <c r="I76" s="23" t="n"/>
+      <c r="J76" s="23" t="n"/>
+      <c r="K76" s="23" t="n"/>
+      <c r="L76" s="23" t="n"/>
+      <c r="M76" s="23" t="n"/>
+      <c r="N76" s="24">
+        <f>COUNTIF(H76:M76,"Г")</f>
+        <v/>
+      </c>
+      <c r="O76" s="24">
+        <f>COUNTIF(H76:M76,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P76" s="25" t="n"/>
+      <c r="Q76" s="26" t="n"/>
+    </row>
+    <row r="77" ht="26" customHeight="1">
+      <c r="A77" s="18" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="19" t="inlineStr">
+        <is>
+          <t>Nukuyev Clinic</t>
+        </is>
+      </c>
+      <c r="C77" s="20" t="inlineStr">
+        <is>
+          <t>+7 771 202 08 08</t>
+        </is>
+      </c>
+      <c r="D77" s="21" t="inlineStr">
+        <is>
+          <t>Медеуский</t>
+        </is>
+      </c>
+      <c r="E77" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00, по записи</t>
+        </is>
+      </c>
+      <c r="F77" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G77" s="23" t="n"/>
+      <c r="H77" s="23" t="n"/>
+      <c r="I77" s="23" t="n"/>
+      <c r="J77" s="23" t="n"/>
+      <c r="K77" s="23" t="n"/>
+      <c r="L77" s="23" t="n"/>
+      <c r="M77" s="23" t="n"/>
+      <c r="N77" s="24">
+        <f>COUNTIF(H77:M77,"Г")</f>
+        <v/>
+      </c>
+      <c r="O77" s="24">
+        <f>COUNTIF(H77:M77,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P77" s="25" t="n"/>
+      <c r="Q77" s="26" t="n"/>
+    </row>
+    <row r="78" ht="26" customHeight="1">
+      <c r="A78" s="18" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="19" t="inlineStr">
+        <is>
+          <t>Ortho Perio Center</t>
+        </is>
+      </c>
+      <c r="C78" s="20" t="inlineStr">
+        <is>
+          <t>+7 747 460 36 78</t>
+        </is>
+      </c>
+      <c r="D78" s="21" t="inlineStr">
+        <is>
+          <t>Медеуский</t>
+        </is>
+      </c>
+      <c r="E78" s="21" t="inlineStr">
+        <is>
+          <t>откр. 10:00</t>
+        </is>
+      </c>
+      <c r="F78" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G78" s="23" t="n"/>
+      <c r="H78" s="23" t="n"/>
+      <c r="I78" s="23" t="n"/>
+      <c r="J78" s="23" t="n"/>
+      <c r="K78" s="23" t="n"/>
+      <c r="L78" s="23" t="n"/>
+      <c r="M78" s="23" t="n"/>
+      <c r="N78" s="24">
+        <f>COUNTIF(H78:M78,"Г")</f>
+        <v/>
+      </c>
+      <c r="O78" s="24">
+        <f>COUNTIF(H78:M78,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P78" s="25" t="n"/>
+      <c r="Q78" s="26" t="n"/>
+    </row>
+    <row r="79" ht="26" customHeight="1">
+      <c r="A79" s="18" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="19" t="inlineStr">
+        <is>
+          <t>SP Clinic</t>
+        </is>
+      </c>
+      <c r="C79" s="20" t="inlineStr">
+        <is>
+          <t>+7 778 375 88 88</t>
+        </is>
+      </c>
+      <c r="D79" s="21" t="inlineStr">
+        <is>
+          <t>Медеуский</t>
+        </is>
+      </c>
+      <c r="E79" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00</t>
+        </is>
+      </c>
+      <c r="F79" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G79" s="23" t="n"/>
+      <c r="H79" s="23" t="n"/>
+      <c r="I79" s="23" t="n"/>
+      <c r="J79" s="23" t="n"/>
+      <c r="K79" s="23" t="n"/>
+      <c r="L79" s="23" t="n"/>
+      <c r="M79" s="23" t="n"/>
+      <c r="N79" s="24">
+        <f>COUNTIF(H79:M79,"Г")</f>
+        <v/>
+      </c>
+      <c r="O79" s="24">
+        <f>COUNTIF(H79:M79,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P79" s="25" t="n"/>
+      <c r="Q79" s="26" t="n"/>
+    </row>
+    <row r="80" ht="26" customHeight="1">
+      <c r="A80" s="18" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="19" t="inlineStr">
+        <is>
+          <t>abc clinic</t>
+        </is>
+      </c>
+      <c r="C80" s="20" t="inlineStr">
+        <is>
+          <t>+7 727 310 88 85</t>
+        </is>
+      </c>
+      <c r="D80" s="21" t="inlineStr">
+        <is>
+          <t>Медеуский</t>
+        </is>
+      </c>
+      <c r="E80" s="21" t="inlineStr">
+        <is>
+          <t>откр. 10:00</t>
+        </is>
+      </c>
+      <c r="F80" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G80" s="23" t="n"/>
+      <c r="H80" s="23" t="n"/>
+      <c r="I80" s="23" t="n"/>
+      <c r="J80" s="23" t="n"/>
+      <c r="K80" s="23" t="n"/>
+      <c r="L80" s="23" t="n"/>
+      <c r="M80" s="23" t="n"/>
+      <c r="N80" s="24">
+        <f>COUNTIF(H80:M80,"Г")</f>
+        <v/>
+      </c>
+      <c r="O80" s="24">
+        <f>COUNTIF(H80:M80,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P80" s="25" t="n"/>
+      <c r="Q80" s="26" t="n"/>
+    </row>
+    <row r="81" ht="26" customHeight="1">
+      <c r="A81" s="18" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="19" t="inlineStr">
+        <is>
+          <t>ЗамЗам</t>
+        </is>
+      </c>
+      <c r="C81" s="20" t="inlineStr">
+        <is>
+          <t>+7 777 380 36 70</t>
+        </is>
+      </c>
+      <c r="D81" s="21" t="inlineStr">
+        <is>
+          <t>Медеуский</t>
+        </is>
+      </c>
+      <c r="E81" s="21" t="inlineStr">
+        <is>
+          <t>откр. 08:00</t>
+        </is>
+      </c>
+      <c r="F81" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G81" s="23" t="n"/>
+      <c r="H81" s="23" t="n"/>
+      <c r="I81" s="23" t="n"/>
+      <c r="J81" s="23" t="n"/>
+      <c r="K81" s="23" t="n"/>
+      <c r="L81" s="23" t="n"/>
+      <c r="M81" s="23" t="n"/>
+      <c r="N81" s="24">
+        <f>COUNTIF(H81:M81,"Г")</f>
+        <v/>
+      </c>
+      <c r="O81" s="24">
+        <f>COUNTIF(H81:M81,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P81" s="25" t="n"/>
+      <c r="Q81" s="26" t="n"/>
+    </row>
+    <row r="82" ht="26" customHeight="1">
+      <c r="A82" s="18" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="19" t="inlineStr">
+        <is>
+          <t>Clinic Expert</t>
+        </is>
+      </c>
+      <c r="C82" s="20" t="inlineStr">
+        <is>
+          <t>+7 708 088 00 33</t>
+        </is>
+      </c>
+      <c r="D82" s="21" t="inlineStr">
+        <is>
+          <t>Наурызбайский</t>
+        </is>
+      </c>
+      <c r="E82" s="21" t="inlineStr">
+        <is>
+          <t>откр. 08:00</t>
+        </is>
+      </c>
+      <c r="F82" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G82" s="23" t="n"/>
+      <c r="H82" s="23" t="n"/>
+      <c r="I82" s="23" t="n"/>
+      <c r="J82" s="23" t="n"/>
+      <c r="K82" s="23" t="n"/>
+      <c r="L82" s="23" t="n"/>
+      <c r="M82" s="23" t="n"/>
+      <c r="N82" s="24">
+        <f>COUNTIF(H82:M82,"Г")</f>
+        <v/>
+      </c>
+      <c r="O82" s="24">
+        <f>COUNTIF(H82:M82,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P82" s="25" t="n"/>
+      <c r="Q82" s="26" t="n"/>
+    </row>
+    <row r="83" ht="26" customHeight="1">
+      <c r="A83" s="18" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="19" t="inlineStr">
+        <is>
+          <t>DentOs</t>
+        </is>
+      </c>
+      <c r="C83" s="20" t="inlineStr">
+        <is>
+          <t>+7 771 779 68 68</t>
+        </is>
+      </c>
+      <c r="D83" s="21" t="inlineStr">
+        <is>
+          <t>Наурызбайский</t>
+        </is>
+      </c>
+      <c r="E83" s="21" t="inlineStr">
+        <is>
+          <t>откр. 10:00, по записи</t>
+        </is>
+      </c>
+      <c r="F83" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G83" s="23" t="n"/>
+      <c r="H83" s="23" t="n"/>
+      <c r="I83" s="23" t="n"/>
+      <c r="J83" s="23" t="n"/>
+      <c r="K83" s="23" t="n"/>
+      <c r="L83" s="23" t="n"/>
+      <c r="M83" s="23" t="n"/>
+      <c r="N83" s="24">
+        <f>COUNTIF(H83:M83,"Г")</f>
+        <v/>
+      </c>
+      <c r="O83" s="24">
+        <f>COUNTIF(H83:M83,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P83" s="25" t="n"/>
+      <c r="Q83" s="26" t="n"/>
+    </row>
+    <row r="84" ht="26" customHeight="1">
+      <c r="A84" s="18" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="19" t="inlineStr">
+        <is>
+          <t>Lux Dental Clinic</t>
+        </is>
+      </c>
+      <c r="C84" s="20" t="inlineStr">
+        <is>
+          <t>+7 708 085 80 80</t>
+        </is>
+      </c>
+      <c r="D84" s="21" t="inlineStr">
+        <is>
+          <t>Наурызбайский</t>
+        </is>
+      </c>
+      <c r="E84" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00</t>
+        </is>
+      </c>
+      <c r="F84" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G84" s="23" t="n"/>
+      <c r="H84" s="23" t="n"/>
+      <c r="I84" s="23" t="n"/>
+      <c r="J84" s="23" t="n"/>
+      <c r="K84" s="23" t="n"/>
+      <c r="L84" s="23" t="n"/>
+      <c r="M84" s="23" t="n"/>
+      <c r="N84" s="24">
+        <f>COUNTIF(H84:M84,"Г")</f>
+        <v/>
+      </c>
+      <c r="O84" s="24">
+        <f>COUNTIF(H84:M84,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P84" s="25" t="n"/>
+      <c r="Q84" s="26" t="n"/>
+    </row>
+    <row r="85" ht="26" customHeight="1">
+      <c r="A85" s="18" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="19" t="inlineStr">
+        <is>
+          <t>Mivimed</t>
+        </is>
+      </c>
+      <c r="C85" s="20" t="inlineStr">
+        <is>
+          <t>+7 700 315 55 50</t>
+        </is>
+      </c>
+      <c r="D85" s="21" t="inlineStr">
+        <is>
+          <t>Наурызбайский</t>
+        </is>
+      </c>
+      <c r="E85" s="21" t="inlineStr">
+        <is>
+          <t>откр. 08:00</t>
+        </is>
+      </c>
+      <c r="F85" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G85" s="23" t="n"/>
+      <c r="H85" s="23" t="n"/>
+      <c r="I85" s="23" t="n"/>
+      <c r="J85" s="23" t="n"/>
+      <c r="K85" s="23" t="n"/>
+      <c r="L85" s="23" t="n"/>
+      <c r="M85" s="23" t="n"/>
+      <c r="N85" s="24">
+        <f>COUNTIF(H85:M85,"Г")</f>
+        <v/>
+      </c>
+      <c r="O85" s="24">
+        <f>COUNTIF(H85:M85,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P85" s="25" t="n"/>
+      <c r="Q85" s="26" t="n"/>
+    </row>
+    <row r="86" ht="26" customHeight="1">
+      <c r="A86" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="19" t="inlineStr">
+        <is>
+          <t>Rayana Dent</t>
+        </is>
+      </c>
+      <c r="C86" s="20" t="inlineStr">
+        <is>
+          <t>+7 771 192 05 05</t>
+        </is>
+      </c>
+      <c r="D86" s="21" t="inlineStr">
+        <is>
+          <t>Наурызбайский</t>
+        </is>
+      </c>
+      <c r="E86" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00</t>
+        </is>
+      </c>
+      <c r="F86" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G86" s="23" t="n"/>
+      <c r="H86" s="23" t="n"/>
+      <c r="I86" s="23" t="n"/>
+      <c r="J86" s="23" t="n"/>
+      <c r="K86" s="23" t="n"/>
+      <c r="L86" s="23" t="n"/>
+      <c r="M86" s="23" t="n"/>
+      <c r="N86" s="24">
+        <f>COUNTIF(H86:M86,"Г")</f>
+        <v/>
+      </c>
+      <c r="O86" s="24">
+        <f>COUNTIF(H86:M86,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P86" s="25" t="n"/>
+      <c r="Q86" s="26" t="n"/>
+    </row>
+    <row r="87" ht="26" customHeight="1">
+      <c r="A87" s="18" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="19" t="inlineStr">
+        <is>
+          <t>Sinadent</t>
+        </is>
+      </c>
+      <c r="C87" s="20" t="inlineStr">
+        <is>
+          <t>+7 707 138 10 55</t>
+        </is>
+      </c>
+      <c r="D87" s="21" t="inlineStr">
+        <is>
+          <t>Наурызбайский</t>
+        </is>
+      </c>
+      <c r="E87" s="21" t="inlineStr">
+        <is>
+          <t>откр. 10:00</t>
+        </is>
+      </c>
+      <c r="F87" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G87" s="23" t="n"/>
+      <c r="H87" s="23" t="n"/>
+      <c r="I87" s="23" t="n"/>
+      <c r="J87" s="23" t="n"/>
+      <c r="K87" s="23" t="n"/>
+      <c r="L87" s="23" t="n"/>
+      <c r="M87" s="23" t="n"/>
+      <c r="N87" s="24">
+        <f>COUNTIF(H87:M87,"Г")</f>
+        <v/>
+      </c>
+      <c r="O87" s="24">
+        <f>COUNTIF(H87:M87,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P87" s="25" t="n"/>
+      <c r="Q87" s="26" t="n"/>
+    </row>
+    <row r="88" ht="26" customHeight="1">
+      <c r="A88" s="18" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="19" t="inlineStr">
+        <is>
+          <t>Коралл</t>
+        </is>
+      </c>
+      <c r="C88" s="20" t="inlineStr">
+        <is>
+          <t>+7 747 978 56 80</t>
+        </is>
+      </c>
+      <c r="D88" s="21" t="inlineStr">
+        <is>
+          <t>Наурызбайский</t>
+        </is>
+      </c>
+      <c r="E88" s="21" t="inlineStr">
+        <is>
+          <t>откр. 09:00</t>
+        </is>
+      </c>
+      <c r="F88" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G88" s="23" t="n"/>
+      <c r="H88" s="23" t="n"/>
+      <c r="I88" s="23" t="n"/>
+      <c r="J88" s="23" t="n"/>
+      <c r="K88" s="23" t="n"/>
+      <c r="L88" s="23" t="n"/>
+      <c r="M88" s="23" t="n"/>
+      <c r="N88" s="24">
+        <f>COUNTIF(H88:M88,"Г")</f>
+        <v/>
+      </c>
+      <c r="O88" s="24">
+        <f>COUNTIF(H88:M88,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P88" s="25" t="n"/>
+      <c r="Q88" s="26" t="n"/>
+    </row>
+    <row r="89" ht="26" customHeight="1">
+      <c r="A89" s="18" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="19" t="inlineStr">
+        <is>
+          <t>Муслим-стом</t>
+        </is>
+      </c>
+      <c r="C89" s="20" t="inlineStr">
+        <is>
+          <t>+7 707 300 27 47</t>
+        </is>
+      </c>
+      <c r="D89" s="21" t="inlineStr">
+        <is>
+          <t>Наурызбайский</t>
+        </is>
+      </c>
+      <c r="E89" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F89" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G89" s="23" t="n"/>
+      <c r="H89" s="23" t="n"/>
+      <c r="I89" s="23" t="n"/>
+      <c r="J89" s="23" t="n"/>
+      <c r="K89" s="23" t="n"/>
+      <c r="L89" s="23" t="n"/>
+      <c r="M89" s="23" t="n"/>
+      <c r="N89" s="24">
+        <f>COUNTIF(H89:M89,"Г")</f>
+        <v/>
+      </c>
+      <c r="O89" s="24">
+        <f>COUNTIF(H89:M89,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P89" s="25" t="n"/>
+      <c r="Q89" s="26" t="n"/>
+    </row>
+    <row r="90" ht="26" customHeight="1">
+      <c r="A90" s="18" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="19" t="inlineStr">
+        <is>
+          <t>Dr.Omar Dental Clinic</t>
+        </is>
+      </c>
+      <c r="C90" s="20" t="inlineStr">
+        <is>
+          <t>+7 778 143 52 61</t>
+        </is>
+      </c>
+      <c r="D90" s="21" t="inlineStr">
+        <is>
+          <t>Талгарский (Бесагаш)</t>
+        </is>
+      </c>
+      <c r="E90" s="21" t="inlineStr">
+        <is>
+          <t>открывается в 09:00</t>
+        </is>
+      </c>
+      <c r="F90" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G90" s="23" t="n"/>
+      <c r="H90" s="23" t="n"/>
+      <c r="I90" s="23" t="n"/>
+      <c r="J90" s="23" t="n"/>
+      <c r="K90" s="23" t="n"/>
+      <c r="L90" s="23" t="n"/>
+      <c r="M90" s="23" t="n"/>
+      <c r="N90" s="24">
+        <f>COUNTIF(H90:M90,"Г")</f>
+        <v/>
+      </c>
+      <c r="O90" s="24">
+        <f>COUNTIF(H90:M90,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P90" s="25" t="n"/>
+      <c r="Q90" s="26" t="n"/>
+    </row>
+    <row r="91" ht="26" customHeight="1">
+      <c r="A91" s="18" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="19" t="inlineStr">
+        <is>
+          <t>DentalPRO</t>
+        </is>
+      </c>
+      <c r="C91" s="20" t="inlineStr">
+        <is>
+          <t>+7 771 800 00 67</t>
+        </is>
+      </c>
+      <c r="D91" s="21" t="inlineStr">
+        <is>
+          <t>Турксибский</t>
+        </is>
+      </c>
+      <c r="E91" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F91" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G91" s="23" t="n"/>
+      <c r="H91" s="23" t="n"/>
+      <c r="I91" s="23" t="n"/>
+      <c r="J91" s="23" t="n"/>
+      <c r="K91" s="23" t="n"/>
+      <c r="L91" s="23" t="n"/>
+      <c r="M91" s="23" t="n"/>
+      <c r="N91" s="24">
+        <f>COUNTIF(H91:M91,"Г")</f>
+        <v/>
+      </c>
+      <c r="O91" s="24">
+        <f>COUNTIF(H91:M91,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P91" s="25" t="n"/>
+      <c r="Q91" s="26" t="n"/>
+    </row>
+    <row r="92" ht="26" customHeight="1">
+      <c r="A92" s="18" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="19" t="inlineStr">
+        <is>
+          <t>Elit Stom (Сейфуллина 102)</t>
+        </is>
+      </c>
+      <c r="C92" s="20" t="inlineStr">
+        <is>
+          <t>+7 747 323 28 34</t>
+        </is>
+      </c>
+      <c r="D92" s="21" t="inlineStr">
+        <is>
+          <t>Турксибский</t>
+        </is>
+      </c>
+      <c r="E92" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F92" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G92" s="23" t="n"/>
+      <c r="H92" s="23" t="n"/>
+      <c r="I92" s="23" t="n"/>
+      <c r="J92" s="23" t="n"/>
+      <c r="K92" s="23" t="n"/>
+      <c r="L92" s="23" t="n"/>
+      <c r="M92" s="23" t="n"/>
+      <c r="N92" s="24">
+        <f>COUNTIF(H92:M92,"Г")</f>
+        <v/>
+      </c>
+      <c r="O92" s="24">
+        <f>COUNTIF(H92:M92,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P92" s="25" t="n"/>
+      <c r="Q92" s="26" t="n"/>
+    </row>
+    <row r="93" ht="26" customHeight="1">
+      <c r="A93" s="18" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="19" t="inlineStr">
+        <is>
+          <t>Expert 32 stom</t>
+        </is>
+      </c>
+      <c r="C93" s="20" t="inlineStr">
+        <is>
+          <t>+7 775 846 19 49</t>
+        </is>
+      </c>
+      <c r="D93" s="21" t="inlineStr">
+        <is>
+          <t>Турксибский</t>
+        </is>
+      </c>
+      <c r="E93" s="21" t="inlineStr">
+        <is>
+          <t>не указаны</t>
+        </is>
+      </c>
+      <c r="F93" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G93" s="23" t="n"/>
+      <c r="H93" s="23" t="n"/>
+      <c r="I93" s="23" t="n"/>
+      <c r="J93" s="23" t="n"/>
+      <c r="K93" s="23" t="n"/>
+      <c r="L93" s="23" t="n"/>
+      <c r="M93" s="23" t="n"/>
+      <c r="N93" s="24">
+        <f>COUNTIF(H93:M93,"Г")</f>
+        <v/>
+      </c>
+      <c r="O93" s="24">
+        <f>COUNTIF(H93:M93,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P93" s="25" t="n"/>
+      <c r="Q93" s="26" t="n"/>
+    </row>
+    <row r="94" ht="26" customHeight="1">
+      <c r="A94" s="18" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="19" t="inlineStr">
+        <is>
+          <t>КГМЦ</t>
+        </is>
+      </c>
+      <c r="C94" s="20" t="inlineStr">
+        <is>
+          <t>+7 727 397 37 78</t>
+        </is>
+      </c>
+      <c r="D94" s="21" t="inlineStr">
+        <is>
+          <t>Турксибский</t>
+        </is>
+      </c>
+      <c r="E94" s="21" t="inlineStr">
+        <is>
+          <t>открывается в 09:00 по записи</t>
+        </is>
+      </c>
+      <c r="F94" s="18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G94" s="23" t="n"/>
+      <c r="H94" s="23" t="n"/>
+      <c r="I94" s="23" t="n"/>
+      <c r="J94" s="23" t="n"/>
+      <c r="K94" s="23" t="n"/>
+      <c r="L94" s="23" t="n"/>
+      <c r="M94" s="23" t="n"/>
+      <c r="N94" s="24">
+        <f>COUNTIF(H94:M94,"Г")</f>
+        <v/>
+      </c>
+      <c r="O94" s="24">
+        <f>COUNTIF(H94:M94,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P94" s="25" t="n"/>
+      <c r="Q94" s="26" t="n"/>
+    </row>
+    <row r="95" ht="26" customHeight="1">
+      <c r="A95" s="18" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="19" t="inlineStr">
+        <is>
+          <t>Стома Плюс</t>
+        </is>
+      </c>
+      <c r="C95" s="20" t="inlineStr">
+        <is>
+          <t>+7 771 335 30 17</t>
+        </is>
+      </c>
+      <c r="D95" s="21" t="inlineStr">
+        <is>
+          <t>Алатауский</t>
+        </is>
+      </c>
+      <c r="E95" s="21" t="inlineStr">
+        <is>
+          <t>09:00-23:00</t>
+        </is>
+      </c>
+      <c r="F95" s="18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G95" s="23" t="n"/>
+      <c r="H95" s="23" t="n"/>
+      <c r="I95" s="23" t="n"/>
+      <c r="J95" s="23" t="n"/>
+      <c r="K95" s="23" t="n"/>
+      <c r="L95" s="23" t="n"/>
+      <c r="M95" s="23" t="n"/>
+      <c r="N95" s="24">
+        <f>COUNTIF(H95:M95,"Г")</f>
+        <v/>
+      </c>
+      <c r="O95" s="24">
+        <f>COUNTIF(H95:M95,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P95" s="25" t="n"/>
+      <c r="Q95" s="26" t="n"/>
+    </row>
+    <row r="96" ht="26" customHeight="1">
+      <c r="A96" s="18" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="19" t="inlineStr">
+        <is>
+          <t>Muslim Dent</t>
+        </is>
+      </c>
+      <c r="C96" s="20" t="inlineStr">
+        <is>
+          <t>+7 771 800 00 65</t>
+        </is>
+      </c>
+      <c r="D96" s="21" t="inlineStr">
+        <is>
+          <t>Алмалинский</t>
+        </is>
+      </c>
+      <c r="E96" s="21" t="inlineStr">
+        <is>
+          <t>10:00-23:45 ежедневно</t>
+        </is>
+      </c>
+      <c r="F96" s="18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G96" s="23" t="n"/>
+      <c r="H96" s="23" t="n"/>
+      <c r="I96" s="23" t="n"/>
+      <c r="J96" s="23" t="n"/>
+      <c r="K96" s="23" t="n"/>
+      <c r="L96" s="23" t="n"/>
+      <c r="M96" s="23" t="n"/>
+      <c r="N96" s="24">
+        <f>COUNTIF(H96:M96,"Г")</f>
+        <v/>
+      </c>
+      <c r="O96" s="24">
+        <f>COUNTIF(H96:M96,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P96" s="25" t="n"/>
+      <c r="Q96" s="26" t="n"/>
+    </row>
+    <row r="97" ht="26" customHeight="1">
+      <c r="A97" s="18" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="19" t="inlineStr">
+        <is>
+          <t>Estet Clinic</t>
+        </is>
+      </c>
+      <c r="C97" s="20" t="inlineStr">
+        <is>
+          <t>+7 707 101 02 33</t>
+        </is>
+      </c>
+      <c r="D97" s="21" t="inlineStr">
+        <is>
+          <t>Ауэзовский</t>
+        </is>
+      </c>
+      <c r="E97" s="21" t="inlineStr">
+        <is>
+          <t>09:00-23:00 ежедневно</t>
+        </is>
+      </c>
+      <c r="F97" s="18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G97" s="23" t="n"/>
+      <c r="H97" s="23" t="n"/>
+      <c r="I97" s="23" t="n"/>
+      <c r="J97" s="23" t="n"/>
+      <c r="K97" s="23" t="n"/>
+      <c r="L97" s="23" t="n"/>
+      <c r="M97" s="23" t="n"/>
+      <c r="N97" s="24">
+        <f>COUNTIF(H97:M97,"Г")</f>
+        <v/>
+      </c>
+      <c r="O97" s="24">
+        <f>COUNTIF(H97:M97,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P97" s="25" t="n"/>
+      <c r="Q97" s="26" t="n"/>
+    </row>
+    <row r="98" ht="26" customHeight="1">
+      <c r="A98" s="18" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="19" t="inlineStr">
+        <is>
+          <t>Bilal stom</t>
+        </is>
+      </c>
+      <c r="C98" s="20" t="inlineStr">
+        <is>
+          <t>+7 707 666 98 92</t>
+        </is>
+      </c>
+      <c r="D98" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E98" s="21" t="inlineStr">
+        <is>
+          <t>09:00-24:00 ежедневно</t>
+        </is>
+      </c>
+      <c r="F98" s="18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G98" s="23" t="n"/>
+      <c r="H98" s="23" t="n"/>
+      <c r="I98" s="23" t="n"/>
+      <c r="J98" s="23" t="n"/>
+      <c r="K98" s="23" t="n"/>
+      <c r="L98" s="23" t="n"/>
+      <c r="M98" s="23" t="n"/>
+      <c r="N98" s="24">
+        <f>COUNTIF(H98:M98,"Г")</f>
+        <v/>
+      </c>
+      <c r="O98" s="24">
+        <f>COUNTIF(H98:M98,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P98" s="25" t="n"/>
+      <c r="Q98" s="26" t="n"/>
+    </row>
+    <row r="99" ht="26" customHeight="1">
+      <c r="A99" s="18" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="19" t="inlineStr">
+        <is>
+          <t>Dr.SULTANOV ATABEK</t>
+        </is>
+      </c>
+      <c r="C99" s="20" t="inlineStr">
+        <is>
+          <t>+7 775 300 85 05</t>
+        </is>
+      </c>
+      <c r="D99" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E99" s="21" t="inlineStr">
+        <is>
+          <t>09:00-24:00</t>
+        </is>
+      </c>
+      <c r="F99" s="18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G99" s="23" t="n"/>
+      <c r="H99" s="23" t="n"/>
+      <c r="I99" s="23" t="n"/>
+      <c r="J99" s="23" t="n"/>
+      <c r="K99" s="23" t="n"/>
+      <c r="L99" s="23" t="n"/>
+      <c r="M99" s="23" t="n"/>
+      <c r="N99" s="24">
+        <f>COUNTIF(H99:M99,"Г")</f>
+        <v/>
+      </c>
+      <c r="O99" s="24">
+        <f>COUNTIF(H99:M99,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P99" s="25" t="n"/>
+      <c r="Q99" s="26" t="n"/>
+    </row>
+    <row r="100" ht="26" customHeight="1">
+      <c r="A100" s="18" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="19" t="inlineStr">
+        <is>
+          <t>Elit Dent</t>
+        </is>
+      </c>
+      <c r="C100" s="20" t="inlineStr">
+        <is>
+          <t>+7 708 269 71 00</t>
+        </is>
+      </c>
+      <c r="D100" s="21" t="inlineStr">
+        <is>
+          <t>Бостандыкский</t>
+        </is>
+      </c>
+      <c r="E100" s="21" t="inlineStr">
+        <is>
+          <t>круглосуточно</t>
+        </is>
+      </c>
+      <c r="F100" s="18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G100" s="23" t="n"/>
+      <c r="H100" s="23" t="n"/>
+      <c r="I100" s="23" t="n"/>
+      <c r="J100" s="23" t="n"/>
+      <c r="K100" s="23" t="n"/>
+      <c r="L100" s="23" t="n"/>
+      <c r="M100" s="23" t="n"/>
+      <c r="N100" s="24">
+        <f>COUNTIF(H100:M100,"Г")</f>
+        <v/>
+      </c>
+      <c r="O100" s="24">
+        <f>COUNTIF(H100:M100,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P100" s="25" t="n"/>
+      <c r="Q100" s="26" t="n"/>
+    </row>
+    <row r="101" ht="26" customHeight="1">
+      <c r="A101" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="19" t="inlineStr">
+        <is>
+          <t>Smart dental clinic</t>
+        </is>
+      </c>
+      <c r="C101" s="20" t="inlineStr">
+        <is>
+          <t>+7 707 708 88 15</t>
+        </is>
+      </c>
+      <c r="D101" s="21" t="inlineStr">
+        <is>
+          <t>Карасайский (за городом)</t>
+        </is>
+      </c>
+      <c r="E101" s="21" t="inlineStr">
+        <is>
+          <t>откр. 10:00</t>
+        </is>
+      </c>
+      <c r="F101" s="18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G101" s="23" t="n"/>
+      <c r="H101" s="23" t="n"/>
+      <c r="I101" s="23" t="n"/>
+      <c r="J101" s="23" t="n"/>
+      <c r="K101" s="23" t="n"/>
+      <c r="L101" s="23" t="n"/>
+      <c r="M101" s="23" t="n"/>
+      <c r="N101" s="24">
+        <f>COUNTIF(H101:M101,"Г")</f>
+        <v/>
+      </c>
+      <c r="O101" s="24">
+        <f>COUNTIF(H101:M101,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P101" s="25" t="n"/>
+      <c r="Q101" s="26" t="n"/>
+    </row>
+    <row r="102" ht="26" customHeight="1">
+      <c r="A102" s="18" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="19" t="inlineStr">
+        <is>
+          <t>Dr. Beridze</t>
+        </is>
+      </c>
+      <c r="C102" s="20" t="inlineStr">
+        <is>
+          <t>+7 775 522 05 09</t>
+        </is>
+      </c>
+      <c r="D102" s="21" t="inlineStr">
+        <is>
+          <t>Турксибский</t>
+        </is>
+      </c>
+      <c r="E102" s="21" t="inlineStr">
+        <is>
+          <t>09:00-24:00 ежедневно</t>
+        </is>
+      </c>
+      <c r="F102" s="18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G102" s="23" t="n"/>
+      <c r="H102" s="23" t="n"/>
+      <c r="I102" s="23" t="n"/>
+      <c r="J102" s="23" t="n"/>
+      <c r="K102" s="23" t="n"/>
+      <c r="L102" s="23" t="n"/>
+      <c r="M102" s="23" t="n"/>
+      <c r="N102" s="24">
+        <f>COUNTIF(H102:M102,"Г")</f>
+        <v/>
+      </c>
+      <c r="O102" s="24">
+        <f>COUNTIF(H102:M102,"Ч")</f>
+        <v/>
+      </c>
+      <c r="P102" s="25" t="n"/>
+      <c r="Q102" s="26" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q48"/>
-  <conditionalFormatting sqref="G2:M48">
+  <autoFilter ref="A1:Q102"/>
+  <conditionalFormatting sqref="G2:M102">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Г"</formula>
     </cfRule>
@@ -3473,7 +6011,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G2:M48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Неизвестный код" error="Только: Ч, А, Г, З, Н, С" promptTitle="Итог звонка" prompt="Ч — ответил человек&#10;А — автоответчик&#10;Г — гудки&#10;З — занято&#10;Н — недоступен&#10;С — сбросили" type="list">
+    <dataValidation sqref="G2:M102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Неизвестный код" error="Только: Ч, А, Г, З, Н, С" promptTitle="Итог звонка" prompt="Ч — ответил человек&#10;А — автоответчик&#10;Г — гудки&#10;З — занято&#10;Н — недоступен&#10;С — сбросили" type="list">
       <formula1>"Ч,А,Г,З,Н,С"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3545,19 +6083,19 @@
         </is>
       </c>
       <c r="B5" s="30">
-        <f>COUNTA(Обзвон!$G$2:$G$48)</f>
+        <f>COUNTA(Обзвон!$G$2:$G$102)</f>
         <v/>
       </c>
       <c r="C5" s="30">
-        <f>COUNTIF(Обзвон!$G$2:$G$48,"Ч")</f>
+        <f>COUNTIF(Обзвон!$G$2:$G$102,"Ч")</f>
         <v/>
       </c>
       <c r="D5" s="30">
-        <f>COUNTIF(Обзвон!$G$2:$G$48,"Г")</f>
+        <f>COUNTIF(Обзвон!$G$2:$G$102,"Г")</f>
         <v/>
       </c>
       <c r="E5" s="31">
-        <f>IFERROR(COUNTIF(Обзвон!$G$2:$G$48,"Г")/COUNTA(Обзвон!$G$2:$G$48),"")</f>
+        <f>IFERROR(COUNTIF(Обзвон!$G$2:$G$102,"Г")/COUNTA(Обзвон!$G$2:$G$102),"")</f>
         <v/>
       </c>
     </row>
@@ -3568,19 +6106,19 @@
         </is>
       </c>
       <c r="B6" s="33">
-        <f>COUNTA(Обзвон!$H$2:$I$48)</f>
+        <f>COUNTA(Обзвон!$H$2:$I$102)</f>
         <v/>
       </c>
       <c r="C6" s="33">
-        <f>COUNTIF(Обзвон!$H$2:$I$48,"Ч")</f>
+        <f>COUNTIF(Обзвон!$H$2:$I$102,"Ч")</f>
         <v/>
       </c>
       <c r="D6" s="33">
-        <f>COUNTIF(Обзвон!$H$2:$I$48,"Г")</f>
+        <f>COUNTIF(Обзвон!$H$2:$I$102,"Г")</f>
         <v/>
       </c>
       <c r="E6" s="34">
-        <f>IFERROR(COUNTIF(Обзвон!$H$2:$I$48,"Г")/COUNTA(Обзвон!$H$2:$I$48),"")</f>
+        <f>IFERROR(COUNTIF(Обзвон!$H$2:$I$102,"Г")/COUNTA(Обзвон!$H$2:$I$102),"")</f>
         <v/>
       </c>
     </row>
@@ -3591,19 +6129,19 @@
         </is>
       </c>
       <c r="B7" s="30">
-        <f>COUNTA(Обзвон!$J$2:$K$48)</f>
+        <f>COUNTA(Обзвон!$J$2:$K$102)</f>
         <v/>
       </c>
       <c r="C7" s="30">
-        <f>COUNTIF(Обзвон!$J$2:$K$48,"Ч")</f>
+        <f>COUNTIF(Обзвон!$J$2:$K$102,"Ч")</f>
         <v/>
       </c>
       <c r="D7" s="30">
-        <f>COUNTIF(Обзвон!$J$2:$K$48,"Г")</f>
+        <f>COUNTIF(Обзвон!$J$2:$K$102,"Г")</f>
         <v/>
       </c>
       <c r="E7" s="31">
-        <f>IFERROR(COUNTIF(Обзвон!$J$2:$K$48,"Г")/COUNTA(Обзвон!$J$2:$K$48),"")</f>
+        <f>IFERROR(COUNTIF(Обзвон!$J$2:$K$102,"Г")/COUNTA(Обзвон!$J$2:$K$102),"")</f>
         <v/>
       </c>
     </row>
@@ -3614,19 +6152,19 @@
         </is>
       </c>
       <c r="B8" s="33">
-        <f>COUNTA(Обзвон!$L$2:$M$48)</f>
+        <f>COUNTA(Обзвон!$L$2:$M$102)</f>
         <v/>
       </c>
       <c r="C8" s="33">
-        <f>COUNTIF(Обзвон!$L$2:$M$48,"Ч")</f>
+        <f>COUNTIF(Обзвон!$L$2:$M$102,"Ч")</f>
         <v/>
       </c>
       <c r="D8" s="33">
-        <f>COUNTIF(Обзвон!$L$2:$M$48,"Г")</f>
+        <f>COUNTIF(Обзвон!$L$2:$M$102,"Г")</f>
         <v/>
       </c>
       <c r="E8" s="34">
-        <f>IFERROR(COUNTIF(Обзвон!$L$2:$M$48,"Г")/COUNTA(Обзвон!$L$2:$M$48),"")</f>
+        <f>IFERROR(COUNTIF(Обзвон!$L$2:$M$102,"Г")/COUNTA(Обзвон!$L$2:$M$102),"")</f>
         <v/>
       </c>
     </row>
@@ -3690,7 +6228,7 @@
         </is>
       </c>
       <c r="B22" s="37">
-        <f>COUNTIF(Обзвон!$N$2:$N$48,6)</f>
+        <f>COUNTIF(Обзвон!$N$2:$N$102,6)</f>
         <v/>
       </c>
     </row>
@@ -3701,7 +6239,7 @@
         </is>
       </c>
       <c r="B23" s="40">
-        <f>COUNTIF(Обзвон!$O$2:$O$48,"&gt;0")</f>
+        <f>COUNTIF(Обзвон!$O$2:$O$102,"&gt;0")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Say that the middle priority group is unmeasured, not mediocre
A, B and C read as good, average and poor, which is the wrong axis entirely —
the letter records how many hours a clinic's phone goes unanswered, and B means
2GIS only ever showed us an opening time because the clinic was shut when we
looked. Those eighty-two will split between A and C once the daytime call
establishes when they close.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/obzvon-stomatologii-almaty.xlsx
+++ b/docs/obzvon-stomatologii-almaty.xlsx
@@ -713,7 +713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -821,307 +821,351 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="5" t="inlineStr"/>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Порядок: сначала приоритет A, потом B. Группа C — если останется время, у них вечернего окна почти нет.</t>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>ЧТО ЗНАЧИТ ПРИОРИТЕТ</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="3" t="inlineStr"/>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>КОДЫ</t>
+      <c r="A14" s="5" t="inlineStr"/>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Это размер окна, когда телефон молчит, а не оценка клиники.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Закрываются в 19:00–22:00 или есть обед. Окно широкое, до 14 часов в сутки. Звонить первыми.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Часы в 2ГИС не указаны — окно НЕИЗВЕСТНО. Это не «средние», это «пока не знаем». Выяснится на дневном звонке, и группа разойдётся по A и C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Работают до 23:00–24:00 или круглосуточно. Вечернего окна почти нет. В последнюю очередь и только если останется время.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>КОДЫ</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
           <t>Ч</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>ответил живой человек</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>А</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>автоответчик или голосовое сообщение</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Г</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>гудки, никто не взял трубку</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>З</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>занято</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Н</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>номер недоступен или не существует</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>С</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>сбросили звонок</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="5" t="inlineStr"/>
-      <c r="B21" s="6" t="inlineStr">
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="5" t="inlineStr"/>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Клетка подсвечивается сама: зелёным если ответили, красным если гудки.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="3" t="inlineStr"/>
-      <c r="B23" s="4" t="inlineStr">
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>ПРИМЕР ЗАПОЛНЕНИЯ</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>Клиника</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Раб.</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Веч.1</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D30" s="8" t="inlineStr">
         <is>
           <t>Веч.2</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
         <is>
           <t>Сб.1</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="F30" s="8" t="inlineStr">
         <is>
           <t>Сб.2</t>
         </is>
       </c>
-      <c r="G24" s="8" t="inlineStr">
+      <c r="G30" s="8" t="inlineStr">
         <is>
           <t>Вс.1</t>
         </is>
       </c>
-      <c r="H24" s="8" t="inlineStr">
+      <c r="H30" s="8" t="inlineStr">
         <is>
           <t>Вс.2</t>
         </is>
       </c>
-      <c r="I24" s="8" t="inlineStr">
+      <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Заметки</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="46" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+    <row r="31" ht="46" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>Ажар Дент</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>Ч</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>Г</t>
         </is>
       </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="D31" s="10" t="inlineStr">
         <is>
           <t>Г</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E31" s="10" t="inlineStr">
         <is>
           <t>Г</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="F31" s="10" t="inlineStr">
         <is>
           <t>А</t>
         </is>
       </c>
-      <c r="G25" s="10" t="inlineStr">
+      <c r="G31" s="10" t="inlineStr">
         <is>
           <t>Г</t>
         </is>
       </c>
-      <c r="H25" s="10" t="inlineStr">
+      <c r="H31" s="10" t="inlineStr">
         <is>
           <t>Г</t>
         </is>
       </c>
-      <c r="I25" s="9" t="inlineStr">
+      <c r="I31" s="9" t="inlineStr">
         <is>
           <t>Днём ответил администратор. Сказала, что вечером никого нет. Автоответчик в субботу: «клиника работает с 9 до 19». Перезвонили в пн 09:14.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="3" t="inlineStr"/>
-      <c r="B28" s="4" t="inlineStr">
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="3" t="inlineStr"/>
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>ЕСЛИ СНЯЛИ ТРУБКУ</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="5" t="inlineStr"/>
-      <c r="B29" s="6" t="inlineStr">
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="5" t="inlineStr"/>
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Представиться и сказать правду, без легенд: «Здравствуйте. Я провожу небольшое исследование по клиникам Алматы, буквально два вопроса, если у вас есть полминуты».</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>У вас можно записаться по телефону вечером, после закрытия?</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>Кто отвечает на звонки в выходные — администратор или кто-то дежурит?</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="5" t="inlineStr">
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>Сколько примерно записавшихся до вас не доходит? — самый ценный вопрос, ответ записывать целиком и своими словами.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="11" t="inlineStr"/>
-      <c r="B34" s="12" t="inlineStr">
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="11" t="inlineStr"/>
+      <c r="B40" s="12" t="inlineStr">
         <is>
           <t>ЧЕГО ДЕЛАТЬ НЕЛЬЗЯ</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="13" t="inlineStr"/>
-      <c r="B35" s="14" t="inlineStr">
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="13" t="inlineStr"/>
+      <c r="B41" s="14" t="inlineStr">
         <is>
           <t>Не притворяться пациентом. Ни при каких условиях.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="13" t="inlineStr"/>
-      <c r="B36" s="14" t="inlineStr">
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="13" t="inlineStr"/>
+      <c r="B42" s="14" t="inlineStr">
         <is>
           <t>Не молчать в трубку. Ответили — сразу говорим.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="13" t="inlineStr"/>
-      <c r="B37" s="14" t="inlineStr">
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="13" t="inlineStr"/>
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>Ничего не предлагать и не продавать. Сейчас мы только считаем.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="13" t="inlineStr"/>
-      <c r="B38" s="14" t="inlineStr">
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="13" t="inlineStr"/>
+      <c r="B44" s="14" t="inlineStr">
         <is>
           <t>Не спорить и не уговаривать. Отказались — спасибо, до свидания.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="28" customHeight="1">
-      <c r="A40" s="5" t="inlineStr"/>
-      <c r="B40" s="6" t="inlineStr">
+    <row r="46" ht="28" customHeight="1">
+      <c r="A46" s="5" t="inlineStr"/>
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>Звонить с одного номера все дни, и с того, на который готовы ответить утром. Часть клиник перезвонит на пропущенный — записывайте дату и время в колонку «Перезвонили».</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="28" customHeight="1">
-      <c r="A42" s="15" t="inlineStr"/>
-      <c r="B42" s="16" t="inlineStr">
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="15" t="inlineStr"/>
+      <c r="B48" s="16" t="inlineStr">
         <is>
           <t>Телефоны, часы и районы взяты из 2ГИС 22 августа 2026 года. Если клиника называет другой график — впишите в заметки.</t>
         </is>

</xml_diff>

<commit_message>
Point the conversation at no-shows and stop it from pitching
The daytime call is worth more as an interview than as a measurement, and the
question worth asking is what the clinic already does about patients who book
and never arrive — what they have built or paid for already is the only honest
signal that the problem costs them something.

So the script asks for last week's count rather than whether it "happens", asks
what they do before we say what we would do, and forbids naming our own service
during the call: a person who hears the remedy starts agreeing with the
diagnosis to be polite. Two columns capture the answers instead of burying them
in free text.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/obzvon-stomatologii-almaty.xlsx
+++ b/docs/obzvon-stomatologii-almaty.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Итоги" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Обзвон'!$A$1:$Q$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Обзвон'!$A$1:$S$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -713,7 +713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1067,105 +1067,173 @@
       <c r="A34" s="3" t="inlineStr"/>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>ЕСЛИ СНЯЛИ ТРУБКУ</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="28" customHeight="1">
+          <t>ЕСЛИ СНЯЛИ ТРУБКУ — СКРИПТ</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
       <c r="A35" s="5" t="inlineStr"/>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Представиться и сказать правду, без легенд: «Здравствуйте. Я провожу небольшое исследование по клиникам Алматы, буквально два вопроса, если у вас есть полминуты».</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="16" customHeight="1">
+          <t>Главное в этом звонке — узнать про неявки. Всё остальное второстепенно.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>1.</t>
+          <t>Начало</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>У вас можно записаться по телефону вечером, после закрытия?</t>
+          <t>«Здравствуйте! Меня зовут ___. Я не пациент — я делаю сервис для стоматологий и сейчас изучаю, как у клиник устроена запись. Три вопроса, если найдётся минута.»</t>
         </is>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>2.</t>
+          <t>1.</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Кто отвечает на звонки в выходные — администратор или кто-то дежурит?</t>
+          <t>«Скажите, у вас бывает так, что пациент записался, а потом не пришёл?»</t>
         </is>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>«А примерно сколько таких было на прошлой неделе?» — нужно число, а не «часто» или «бывает». Записать в колонку «Неявки: сколько».</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>Сколько примерно записавшихся до вас не доходит? — самый ценный вопрос, ответ записывать целиком и своими словами.</t>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>«И что вы с этим сейчас делаете?» — САМЫЙ ВАЖНЫЙ ВОПРОС. Дать договорить, не подсказывать варианты. Записать в «Что делают сейчас».</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="11" t="inlineStr"/>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>ЧЕГО ДЕЛАТЬ НЕЛЬЗЯ</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="13" t="inlineStr"/>
-      <c r="B41" s="14" t="inlineStr">
-        <is>
-          <t>Не притворяться пациентом. Ни при каких условиях.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="13" t="inlineStr"/>
-      <c r="B42" s="14" t="inlineStr">
-        <is>
-          <t>Не молчать в трубку. Ответили — сразу говорим.</t>
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>если напоминают</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>«А кто напоминает и за сколько до приёма? Помогает, стало меньше?»</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Закрытие</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>«И последнее: если человек звонит вечером после закрытия — он может к вам записаться?» Потом: «Спасибо большое, вы очень помогли.»</t>
         </is>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="13" t="inlineStr"/>
-      <c r="B43" s="14" t="inlineStr">
-        <is>
-          <t>Ничего не предлагать и не продавать. Сейчас мы только считаем.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="16" customHeight="1">
+      <c r="A43" s="11" t="inlineStr"/>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>ЧЕГО НЕ ДЕЛАТЬ В ЭТОМ РАЗГОВОРЕ</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="42" customHeight="1">
       <c r="A44" s="13" t="inlineStr"/>
       <c r="B44" s="14" t="inlineStr">
         <is>
+          <t>Не рассказывать, что мы делаем сервис против неявок. Как только человек услышит про решение, он начнёт вежливо соглашаться, и ответ обесценится. Сначала узнаём, рассказываем потом и не в этом звонке.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="13" t="inlineStr"/>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>Не спрашивать «а вам было бы интересно...». Мнения о будущем ничего не стоят, нужны факты про прошлую неделю.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="13" t="inlineStr"/>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>Не советовать и не спорить, даже если решение кажется очевидным.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="A48" s="11" t="inlineStr"/>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>ЧЕГО ДЕЛАТЬ НЕЛЬЗЯ ВООБЩЕ</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="13" t="inlineStr"/>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>Не притворяться пациентом. Ни при каких условиях.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="16" customHeight="1">
+      <c r="A50" s="13" t="inlineStr"/>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>Не молчать в трубку. Ответили — сразу говорим.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="16" customHeight="1">
+      <c r="A51" s="13" t="inlineStr"/>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>Ничего не предлагать и не продавать. Сейчас мы только считаем.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="13" t="inlineStr"/>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
           <t>Не спорить и не уговаривать. Отказались — спасибо, до свидания.</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="28" customHeight="1">
-      <c r="A46" s="5" t="inlineStr"/>
-      <c r="B46" s="6" t="inlineStr">
+    <row r="54" ht="28" customHeight="1">
+      <c r="A54" s="5" t="inlineStr"/>
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>Звонить с одного номера все дни, и с того, на который готовы ответить утром. Часть клиник перезвонит на пропущенный — записывайте дату и время в колонку «Перезвонили».</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="28" customHeight="1">
-      <c r="A48" s="15" t="inlineStr"/>
-      <c r="B48" s="16" t="inlineStr">
+    <row r="56" ht="28" customHeight="1">
+      <c r="A56" s="15" t="inlineStr"/>
+      <c r="B56" s="16" t="inlineStr">
         <is>
           <t>Телефоны, часы и районы взяты из 2ГИС 22 августа 2026 года. Если клиника называет другой график — впишите в заметки.</t>
         </is>
@@ -1185,7 +1253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q102"/>
+  <dimension ref="A1:S102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1203,8 +1271,10 @@
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="9" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="52" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="42" customWidth="1" min="18" max="18"/>
+    <col width="42" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1289,6 +1359,16 @@
         </is>
       </c>
       <c r="Q1" s="17" t="inlineStr">
+        <is>
+          <t>Неявки: сколько</t>
+        </is>
+      </c>
+      <c r="R1" s="17" t="inlineStr">
+        <is>
+          <t>Что делают сейчас</t>
+        </is>
+      </c>
+      <c r="S1" s="17" t="inlineStr">
         <is>
           <t>Заметки</t>
         </is>
@@ -1340,6 +1420,8 @@
       </c>
       <c r="P2" s="25" t="n"/>
       <c r="Q2" s="26" t="n"/>
+      <c r="R2" s="26" t="n"/>
+      <c r="S2" s="26" t="n"/>
     </row>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="18" t="n">
@@ -1387,6 +1469,8 @@
       </c>
       <c r="P3" s="25" t="n"/>
       <c r="Q3" s="26" t="n"/>
+      <c r="R3" s="26" t="n"/>
+      <c r="S3" s="26" t="n"/>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="18" t="n">
@@ -1434,6 +1518,8 @@
       </c>
       <c r="P4" s="25" t="n"/>
       <c r="Q4" s="26" t="n"/>
+      <c r="R4" s="26" t="n"/>
+      <c r="S4" s="26" t="n"/>
     </row>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="18" t="n">
@@ -1481,6 +1567,8 @@
       </c>
       <c r="P5" s="25" t="n"/>
       <c r="Q5" s="26" t="n"/>
+      <c r="R5" s="26" t="n"/>
+      <c r="S5" s="26" t="n"/>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="18" t="n">
@@ -1528,6 +1616,8 @@
       </c>
       <c r="P6" s="25" t="n"/>
       <c r="Q6" s="26" t="n"/>
+      <c r="R6" s="26" t="n"/>
+      <c r="S6" s="26" t="n"/>
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="18" t="n">
@@ -1575,6 +1665,8 @@
       </c>
       <c r="P7" s="25" t="n"/>
       <c r="Q7" s="26" t="n"/>
+      <c r="R7" s="26" t="n"/>
+      <c r="S7" s="26" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="18" t="n">
@@ -1622,6 +1714,8 @@
       </c>
       <c r="P8" s="25" t="n"/>
       <c r="Q8" s="26" t="n"/>
+      <c r="R8" s="26" t="n"/>
+      <c r="S8" s="26" t="n"/>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="18" t="n">
@@ -1669,6 +1763,8 @@
       </c>
       <c r="P9" s="25" t="n"/>
       <c r="Q9" s="26" t="n"/>
+      <c r="R9" s="26" t="n"/>
+      <c r="S9" s="26" t="n"/>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="18" t="n">
@@ -1716,6 +1812,8 @@
       </c>
       <c r="P10" s="25" t="n"/>
       <c r="Q10" s="26" t="n"/>
+      <c r="R10" s="26" t="n"/>
+      <c r="S10" s="26" t="n"/>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="18" t="n">
@@ -1763,6 +1861,8 @@
       </c>
       <c r="P11" s="25" t="n"/>
       <c r="Q11" s="26" t="n"/>
+      <c r="R11" s="26" t="n"/>
+      <c r="S11" s="26" t="n"/>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="18" t="n">
@@ -1810,6 +1910,8 @@
       </c>
       <c r="P12" s="25" t="n"/>
       <c r="Q12" s="26" t="n"/>
+      <c r="R12" s="26" t="n"/>
+      <c r="S12" s="26" t="n"/>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="18" t="n">
@@ -1857,6 +1959,8 @@
       </c>
       <c r="P13" s="25" t="n"/>
       <c r="Q13" s="26" t="n"/>
+      <c r="R13" s="26" t="n"/>
+      <c r="S13" s="26" t="n"/>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="18" t="n">
@@ -1904,6 +2008,8 @@
       </c>
       <c r="P14" s="25" t="n"/>
       <c r="Q14" s="26" t="n"/>
+      <c r="R14" s="26" t="n"/>
+      <c r="S14" s="26" t="n"/>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="18" t="n">
@@ -1951,6 +2057,8 @@
       </c>
       <c r="P15" s="25" t="n"/>
       <c r="Q15" s="26" t="n"/>
+      <c r="R15" s="26" t="n"/>
+      <c r="S15" s="26" t="n"/>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="18" t="n">
@@ -1998,6 +2106,8 @@
       </c>
       <c r="P16" s="25" t="n"/>
       <c r="Q16" s="26" t="n"/>
+      <c r="R16" s="26" t="n"/>
+      <c r="S16" s="26" t="n"/>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="18" t="n">
@@ -2045,6 +2155,8 @@
       </c>
       <c r="P17" s="25" t="n"/>
       <c r="Q17" s="26" t="n"/>
+      <c r="R17" s="26" t="n"/>
+      <c r="S17" s="26" t="n"/>
     </row>
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="18" t="n">
@@ -2092,6 +2204,8 @@
       </c>
       <c r="P18" s="25" t="n"/>
       <c r="Q18" s="26" t="n"/>
+      <c r="R18" s="26" t="n"/>
+      <c r="S18" s="26" t="n"/>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="18" t="n">
@@ -2139,6 +2253,8 @@
       </c>
       <c r="P19" s="25" t="n"/>
       <c r="Q19" s="26" t="n"/>
+      <c r="R19" s="26" t="n"/>
+      <c r="S19" s="26" t="n"/>
     </row>
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="18" t="n">
@@ -2186,6 +2302,8 @@
       </c>
       <c r="P20" s="25" t="n"/>
       <c r="Q20" s="26" t="n"/>
+      <c r="R20" s="26" t="n"/>
+      <c r="S20" s="26" t="n"/>
     </row>
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="18" t="n">
@@ -2233,6 +2351,8 @@
       </c>
       <c r="P21" s="25" t="n"/>
       <c r="Q21" s="26" t="n"/>
+      <c r="R21" s="26" t="n"/>
+      <c r="S21" s="26" t="n"/>
     </row>
     <row r="22" ht="26" customHeight="1">
       <c r="A22" s="18" t="n">
@@ -2280,6 +2400,8 @@
       </c>
       <c r="P22" s="25" t="n"/>
       <c r="Q22" s="26" t="n"/>
+      <c r="R22" s="26" t="n"/>
+      <c r="S22" s="26" t="n"/>
     </row>
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="18" t="n">
@@ -2327,6 +2449,8 @@
       </c>
       <c r="P23" s="25" t="n"/>
       <c r="Q23" s="26" t="n"/>
+      <c r="R23" s="26" t="n"/>
+      <c r="S23" s="26" t="n"/>
     </row>
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="18" t="n">
@@ -2374,6 +2498,8 @@
       </c>
       <c r="P24" s="25" t="n"/>
       <c r="Q24" s="26" t="n"/>
+      <c r="R24" s="26" t="n"/>
+      <c r="S24" s="26" t="n"/>
     </row>
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="18" t="n">
@@ -2421,6 +2547,8 @@
       </c>
       <c r="P25" s="25" t="n"/>
       <c r="Q25" s="26" t="n"/>
+      <c r="R25" s="26" t="n"/>
+      <c r="S25" s="26" t="n"/>
     </row>
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="18" t="n">
@@ -2468,6 +2596,8 @@
       </c>
       <c r="P26" s="25" t="n"/>
       <c r="Q26" s="26" t="n"/>
+      <c r="R26" s="26" t="n"/>
+      <c r="S26" s="26" t="n"/>
     </row>
     <row r="27" ht="26" customHeight="1">
       <c r="A27" s="18" t="n">
@@ -2515,6 +2645,8 @@
       </c>
       <c r="P27" s="25" t="n"/>
       <c r="Q27" s="26" t="n"/>
+      <c r="R27" s="26" t="n"/>
+      <c r="S27" s="26" t="n"/>
     </row>
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="18" t="n">
@@ -2562,6 +2694,8 @@
       </c>
       <c r="P28" s="25" t="n"/>
       <c r="Q28" s="26" t="n"/>
+      <c r="R28" s="26" t="n"/>
+      <c r="S28" s="26" t="n"/>
     </row>
     <row r="29" ht="26" customHeight="1">
       <c r="A29" s="18" t="n">
@@ -2609,6 +2743,8 @@
       </c>
       <c r="P29" s="25" t="n"/>
       <c r="Q29" s="26" t="n"/>
+      <c r="R29" s="26" t="n"/>
+      <c r="S29" s="26" t="n"/>
     </row>
     <row r="30" ht="26" customHeight="1">
       <c r="A30" s="18" t="n">
@@ -2656,6 +2792,8 @@
       </c>
       <c r="P30" s="25" t="n"/>
       <c r="Q30" s="26" t="n"/>
+      <c r="R30" s="26" t="n"/>
+      <c r="S30" s="26" t="n"/>
     </row>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="18" t="n">
@@ -2703,6 +2841,8 @@
       </c>
       <c r="P31" s="25" t="n"/>
       <c r="Q31" s="26" t="n"/>
+      <c r="R31" s="26" t="n"/>
+      <c r="S31" s="26" t="n"/>
     </row>
     <row r="32" ht="26" customHeight="1">
       <c r="A32" s="18" t="n">
@@ -2750,6 +2890,8 @@
       </c>
       <c r="P32" s="25" t="n"/>
       <c r="Q32" s="26" t="n"/>
+      <c r="R32" s="26" t="n"/>
+      <c r="S32" s="26" t="n"/>
     </row>
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="18" t="n">
@@ -2797,6 +2939,8 @@
       </c>
       <c r="P33" s="25" t="n"/>
       <c r="Q33" s="26" t="n"/>
+      <c r="R33" s="26" t="n"/>
+      <c r="S33" s="26" t="n"/>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="18" t="n">
@@ -2844,6 +2988,8 @@
       </c>
       <c r="P34" s="25" t="n"/>
       <c r="Q34" s="26" t="n"/>
+      <c r="R34" s="26" t="n"/>
+      <c r="S34" s="26" t="n"/>
     </row>
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="18" t="n">
@@ -2891,6 +3037,8 @@
       </c>
       <c r="P35" s="25" t="n"/>
       <c r="Q35" s="26" t="n"/>
+      <c r="R35" s="26" t="n"/>
+      <c r="S35" s="26" t="n"/>
     </row>
     <row r="36" ht="26" customHeight="1">
       <c r="A36" s="18" t="n">
@@ -2938,6 +3086,8 @@
       </c>
       <c r="P36" s="25" t="n"/>
       <c r="Q36" s="26" t="n"/>
+      <c r="R36" s="26" t="n"/>
+      <c r="S36" s="26" t="n"/>
     </row>
     <row r="37" ht="26" customHeight="1">
       <c r="A37" s="18" t="n">
@@ -2985,6 +3135,8 @@
       </c>
       <c r="P37" s="25" t="n"/>
       <c r="Q37" s="26" t="n"/>
+      <c r="R37" s="26" t="n"/>
+      <c r="S37" s="26" t="n"/>
     </row>
     <row r="38" ht="26" customHeight="1">
       <c r="A38" s="18" t="n">
@@ -3032,6 +3184,8 @@
       </c>
       <c r="P38" s="25" t="n"/>
       <c r="Q38" s="26" t="n"/>
+      <c r="R38" s="26" t="n"/>
+      <c r="S38" s="26" t="n"/>
     </row>
     <row r="39" ht="26" customHeight="1">
       <c r="A39" s="18" t="n">
@@ -3079,6 +3233,8 @@
       </c>
       <c r="P39" s="25" t="n"/>
       <c r="Q39" s="26" t="n"/>
+      <c r="R39" s="26" t="n"/>
+      <c r="S39" s="26" t="n"/>
     </row>
     <row r="40" ht="26" customHeight="1">
       <c r="A40" s="18" t="n">
@@ -3126,6 +3282,8 @@
       </c>
       <c r="P40" s="25" t="n"/>
       <c r="Q40" s="26" t="n"/>
+      <c r="R40" s="26" t="n"/>
+      <c r="S40" s="26" t="n"/>
     </row>
     <row r="41" ht="26" customHeight="1">
       <c r="A41" s="18" t="n">
@@ -3173,6 +3331,8 @@
       </c>
       <c r="P41" s="25" t="n"/>
       <c r="Q41" s="26" t="n"/>
+      <c r="R41" s="26" t="n"/>
+      <c r="S41" s="26" t="n"/>
     </row>
     <row r="42" ht="26" customHeight="1">
       <c r="A42" s="18" t="n">
@@ -3220,6 +3380,8 @@
       </c>
       <c r="P42" s="25" t="n"/>
       <c r="Q42" s="26" t="n"/>
+      <c r="R42" s="26" t="n"/>
+      <c r="S42" s="26" t="n"/>
     </row>
     <row r="43" ht="26" customHeight="1">
       <c r="A43" s="18" t="n">
@@ -3267,6 +3429,8 @@
       </c>
       <c r="P43" s="25" t="n"/>
       <c r="Q43" s="26" t="n"/>
+      <c r="R43" s="26" t="n"/>
+      <c r="S43" s="26" t="n"/>
     </row>
     <row r="44" ht="26" customHeight="1">
       <c r="A44" s="18" t="n">
@@ -3314,6 +3478,8 @@
       </c>
       <c r="P44" s="25" t="n"/>
       <c r="Q44" s="26" t="n"/>
+      <c r="R44" s="26" t="n"/>
+      <c r="S44" s="26" t="n"/>
     </row>
     <row r="45" ht="26" customHeight="1">
       <c r="A45" s="18" t="n">
@@ -3361,6 +3527,8 @@
       </c>
       <c r="P45" s="25" t="n"/>
       <c r="Q45" s="26" t="n"/>
+      <c r="R45" s="26" t="n"/>
+      <c r="S45" s="26" t="n"/>
     </row>
     <row r="46" ht="26" customHeight="1">
       <c r="A46" s="18" t="n">
@@ -3408,6 +3576,8 @@
       </c>
       <c r="P46" s="25" t="n"/>
       <c r="Q46" s="26" t="n"/>
+      <c r="R46" s="26" t="n"/>
+      <c r="S46" s="26" t="n"/>
     </row>
     <row r="47" ht="26" customHeight="1">
       <c r="A47" s="18" t="n">
@@ -3455,6 +3625,8 @@
       </c>
       <c r="P47" s="25" t="n"/>
       <c r="Q47" s="26" t="n"/>
+      <c r="R47" s="26" t="n"/>
+      <c r="S47" s="26" t="n"/>
     </row>
     <row r="48" ht="26" customHeight="1">
       <c r="A48" s="18" t="n">
@@ -3502,6 +3674,8 @@
       </c>
       <c r="P48" s="25" t="n"/>
       <c r="Q48" s="26" t="n"/>
+      <c r="R48" s="26" t="n"/>
+      <c r="S48" s="26" t="n"/>
     </row>
     <row r="49" ht="26" customHeight="1">
       <c r="A49" s="18" t="n">
@@ -3549,6 +3723,8 @@
       </c>
       <c r="P49" s="25" t="n"/>
       <c r="Q49" s="26" t="n"/>
+      <c r="R49" s="26" t="n"/>
+      <c r="S49" s="26" t="n"/>
     </row>
     <row r="50" ht="26" customHeight="1">
       <c r="A50" s="18" t="n">
@@ -3596,6 +3772,8 @@
       </c>
       <c r="P50" s="25" t="n"/>
       <c r="Q50" s="26" t="n"/>
+      <c r="R50" s="26" t="n"/>
+      <c r="S50" s="26" t="n"/>
     </row>
     <row r="51" ht="26" customHeight="1">
       <c r="A51" s="18" t="n">
@@ -3643,6 +3821,8 @@
       </c>
       <c r="P51" s="25" t="n"/>
       <c r="Q51" s="26" t="n"/>
+      <c r="R51" s="26" t="n"/>
+      <c r="S51" s="26" t="n"/>
     </row>
     <row r="52" ht="26" customHeight="1">
       <c r="A52" s="18" t="n">
@@ -3690,6 +3870,8 @@
       </c>
       <c r="P52" s="25" t="n"/>
       <c r="Q52" s="26" t="n"/>
+      <c r="R52" s="26" t="n"/>
+      <c r="S52" s="26" t="n"/>
     </row>
     <row r="53" ht="26" customHeight="1">
       <c r="A53" s="18" t="n">
@@ -3737,6 +3919,8 @@
       </c>
       <c r="P53" s="25" t="n"/>
       <c r="Q53" s="26" t="n"/>
+      <c r="R53" s="26" t="n"/>
+      <c r="S53" s="26" t="n"/>
     </row>
     <row r="54" ht="26" customHeight="1">
       <c r="A54" s="18" t="n">
@@ -3784,6 +3968,8 @@
       </c>
       <c r="P54" s="25" t="n"/>
       <c r="Q54" s="26" t="n"/>
+      <c r="R54" s="26" t="n"/>
+      <c r="S54" s="26" t="n"/>
     </row>
     <row r="55" ht="26" customHeight="1">
       <c r="A55" s="18" t="n">
@@ -3831,6 +4017,8 @@
       </c>
       <c r="P55" s="25" t="n"/>
       <c r="Q55" s="26" t="n"/>
+      <c r="R55" s="26" t="n"/>
+      <c r="S55" s="26" t="n"/>
     </row>
     <row r="56" ht="26" customHeight="1">
       <c r="A56" s="18" t="n">
@@ -3878,6 +4066,8 @@
       </c>
       <c r="P56" s="25" t="n"/>
       <c r="Q56" s="26" t="n"/>
+      <c r="R56" s="26" t="n"/>
+      <c r="S56" s="26" t="n"/>
     </row>
     <row r="57" ht="26" customHeight="1">
       <c r="A57" s="18" t="n">
@@ -3925,6 +4115,8 @@
       </c>
       <c r="P57" s="25" t="n"/>
       <c r="Q57" s="26" t="n"/>
+      <c r="R57" s="26" t="n"/>
+      <c r="S57" s="26" t="n"/>
     </row>
     <row r="58" ht="26" customHeight="1">
       <c r="A58" s="18" t="n">
@@ -3972,6 +4164,8 @@
       </c>
       <c r="P58" s="25" t="n"/>
       <c r="Q58" s="26" t="n"/>
+      <c r="R58" s="26" t="n"/>
+      <c r="S58" s="26" t="n"/>
     </row>
     <row r="59" ht="26" customHeight="1">
       <c r="A59" s="18" t="n">
@@ -4019,6 +4213,8 @@
       </c>
       <c r="P59" s="25" t="n"/>
       <c r="Q59" s="26" t="n"/>
+      <c r="R59" s="26" t="n"/>
+      <c r="S59" s="26" t="n"/>
     </row>
     <row r="60" ht="26" customHeight="1">
       <c r="A60" s="18" t="n">
@@ -4066,6 +4262,8 @@
       </c>
       <c r="P60" s="25" t="n"/>
       <c r="Q60" s="26" t="n"/>
+      <c r="R60" s="26" t="n"/>
+      <c r="S60" s="26" t="n"/>
     </row>
     <row r="61" ht="26" customHeight="1">
       <c r="A61" s="18" t="n">
@@ -4113,6 +4311,8 @@
       </c>
       <c r="P61" s="25" t="n"/>
       <c r="Q61" s="26" t="n"/>
+      <c r="R61" s="26" t="n"/>
+      <c r="S61" s="26" t="n"/>
     </row>
     <row r="62" ht="26" customHeight="1">
       <c r="A62" s="18" t="n">
@@ -4160,6 +4360,8 @@
       </c>
       <c r="P62" s="25" t="n"/>
       <c r="Q62" s="26" t="n"/>
+      <c r="R62" s="26" t="n"/>
+      <c r="S62" s="26" t="n"/>
     </row>
     <row r="63" ht="26" customHeight="1">
       <c r="A63" s="18" t="n">
@@ -4207,6 +4409,8 @@
       </c>
       <c r="P63" s="25" t="n"/>
       <c r="Q63" s="26" t="n"/>
+      <c r="R63" s="26" t="n"/>
+      <c r="S63" s="26" t="n"/>
     </row>
     <row r="64" ht="26" customHeight="1">
       <c r="A64" s="18" t="n">
@@ -4254,6 +4458,8 @@
       </c>
       <c r="P64" s="25" t="n"/>
       <c r="Q64" s="26" t="n"/>
+      <c r="R64" s="26" t="n"/>
+      <c r="S64" s="26" t="n"/>
     </row>
     <row r="65" ht="26" customHeight="1">
       <c r="A65" s="18" t="n">
@@ -4301,6 +4507,8 @@
       </c>
       <c r="P65" s="25" t="n"/>
       <c r="Q65" s="26" t="n"/>
+      <c r="R65" s="26" t="n"/>
+      <c r="S65" s="26" t="n"/>
     </row>
     <row r="66" ht="26" customHeight="1">
       <c r="A66" s="18" t="n">
@@ -4348,6 +4556,8 @@
       </c>
       <c r="P66" s="25" t="n"/>
       <c r="Q66" s="26" t="n"/>
+      <c r="R66" s="26" t="n"/>
+      <c r="S66" s="26" t="n"/>
     </row>
     <row r="67" ht="26" customHeight="1">
       <c r="A67" s="18" t="n">
@@ -4395,6 +4605,8 @@
       </c>
       <c r="P67" s="25" t="n"/>
       <c r="Q67" s="26" t="n"/>
+      <c r="R67" s="26" t="n"/>
+      <c r="S67" s="26" t="n"/>
     </row>
     <row r="68" ht="26" customHeight="1">
       <c r="A68" s="18" t="n">
@@ -4442,6 +4654,8 @@
       </c>
       <c r="P68" s="25" t="n"/>
       <c r="Q68" s="26" t="n"/>
+      <c r="R68" s="26" t="n"/>
+      <c r="S68" s="26" t="n"/>
     </row>
     <row r="69" ht="26" customHeight="1">
       <c r="A69" s="18" t="n">
@@ -4489,6 +4703,8 @@
       </c>
       <c r="P69" s="25" t="n"/>
       <c r="Q69" s="26" t="n"/>
+      <c r="R69" s="26" t="n"/>
+      <c r="S69" s="26" t="n"/>
     </row>
     <row r="70" ht="26" customHeight="1">
       <c r="A70" s="18" t="n">
@@ -4536,6 +4752,8 @@
       </c>
       <c r="P70" s="25" t="n"/>
       <c r="Q70" s="26" t="n"/>
+      <c r="R70" s="26" t="n"/>
+      <c r="S70" s="26" t="n"/>
     </row>
     <row r="71" ht="26" customHeight="1">
       <c r="A71" s="18" t="n">
@@ -4583,6 +4801,8 @@
       </c>
       <c r="P71" s="25" t="n"/>
       <c r="Q71" s="26" t="n"/>
+      <c r="R71" s="26" t="n"/>
+      <c r="S71" s="26" t="n"/>
     </row>
     <row r="72" ht="26" customHeight="1">
       <c r="A72" s="18" t="n">
@@ -4630,6 +4850,8 @@
       </c>
       <c r="P72" s="25" t="n"/>
       <c r="Q72" s="26" t="n"/>
+      <c r="R72" s="26" t="n"/>
+      <c r="S72" s="26" t="n"/>
     </row>
     <row r="73" ht="26" customHeight="1">
       <c r="A73" s="18" t="n">
@@ -4677,6 +4899,8 @@
       </c>
       <c r="P73" s="25" t="n"/>
       <c r="Q73" s="26" t="n"/>
+      <c r="R73" s="26" t="n"/>
+      <c r="S73" s="26" t="n"/>
     </row>
     <row r="74" ht="26" customHeight="1">
       <c r="A74" s="18" t="n">
@@ -4724,6 +4948,8 @@
       </c>
       <c r="P74" s="25" t="n"/>
       <c r="Q74" s="26" t="n"/>
+      <c r="R74" s="26" t="n"/>
+      <c r="S74" s="26" t="n"/>
     </row>
     <row r="75" ht="26" customHeight="1">
       <c r="A75" s="18" t="n">
@@ -4771,6 +4997,8 @@
       </c>
       <c r="P75" s="25" t="n"/>
       <c r="Q75" s="26" t="n"/>
+      <c r="R75" s="26" t="n"/>
+      <c r="S75" s="26" t="n"/>
     </row>
     <row r="76" ht="26" customHeight="1">
       <c r="A76" s="18" t="n">
@@ -4818,6 +5046,8 @@
       </c>
       <c r="P76" s="25" t="n"/>
       <c r="Q76" s="26" t="n"/>
+      <c r="R76" s="26" t="n"/>
+      <c r="S76" s="26" t="n"/>
     </row>
     <row r="77" ht="26" customHeight="1">
       <c r="A77" s="18" t="n">
@@ -4865,6 +5095,8 @@
       </c>
       <c r="P77" s="25" t="n"/>
       <c r="Q77" s="26" t="n"/>
+      <c r="R77" s="26" t="n"/>
+      <c r="S77" s="26" t="n"/>
     </row>
     <row r="78" ht="26" customHeight="1">
       <c r="A78" s="18" t="n">
@@ -4912,6 +5144,8 @@
       </c>
       <c r="P78" s="25" t="n"/>
       <c r="Q78" s="26" t="n"/>
+      <c r="R78" s="26" t="n"/>
+      <c r="S78" s="26" t="n"/>
     </row>
     <row r="79" ht="26" customHeight="1">
       <c r="A79" s="18" t="n">
@@ -4959,6 +5193,8 @@
       </c>
       <c r="P79" s="25" t="n"/>
       <c r="Q79" s="26" t="n"/>
+      <c r="R79" s="26" t="n"/>
+      <c r="S79" s="26" t="n"/>
     </row>
     <row r="80" ht="26" customHeight="1">
       <c r="A80" s="18" t="n">
@@ -5006,6 +5242,8 @@
       </c>
       <c r="P80" s="25" t="n"/>
       <c r="Q80" s="26" t="n"/>
+      <c r="R80" s="26" t="n"/>
+      <c r="S80" s="26" t="n"/>
     </row>
     <row r="81" ht="26" customHeight="1">
       <c r="A81" s="18" t="n">
@@ -5053,6 +5291,8 @@
       </c>
       <c r="P81" s="25" t="n"/>
       <c r="Q81" s="26" t="n"/>
+      <c r="R81" s="26" t="n"/>
+      <c r="S81" s="26" t="n"/>
     </row>
     <row r="82" ht="26" customHeight="1">
       <c r="A82" s="18" t="n">
@@ -5100,6 +5340,8 @@
       </c>
       <c r="P82" s="25" t="n"/>
       <c r="Q82" s="26" t="n"/>
+      <c r="R82" s="26" t="n"/>
+      <c r="S82" s="26" t="n"/>
     </row>
     <row r="83" ht="26" customHeight="1">
       <c r="A83" s="18" t="n">
@@ -5147,6 +5389,8 @@
       </c>
       <c r="P83" s="25" t="n"/>
       <c r="Q83" s="26" t="n"/>
+      <c r="R83" s="26" t="n"/>
+      <c r="S83" s="26" t="n"/>
     </row>
     <row r="84" ht="26" customHeight="1">
       <c r="A84" s="18" t="n">
@@ -5194,6 +5438,8 @@
       </c>
       <c r="P84" s="25" t="n"/>
       <c r="Q84" s="26" t="n"/>
+      <c r="R84" s="26" t="n"/>
+      <c r="S84" s="26" t="n"/>
     </row>
     <row r="85" ht="26" customHeight="1">
       <c r="A85" s="18" t="n">
@@ -5241,6 +5487,8 @@
       </c>
       <c r="P85" s="25" t="n"/>
       <c r="Q85" s="26" t="n"/>
+      <c r="R85" s="26" t="n"/>
+      <c r="S85" s="26" t="n"/>
     </row>
     <row r="86" ht="26" customHeight="1">
       <c r="A86" s="18" t="n">
@@ -5288,6 +5536,8 @@
       </c>
       <c r="P86" s="25" t="n"/>
       <c r="Q86" s="26" t="n"/>
+      <c r="R86" s="26" t="n"/>
+      <c r="S86" s="26" t="n"/>
     </row>
     <row r="87" ht="26" customHeight="1">
       <c r="A87" s="18" t="n">
@@ -5335,6 +5585,8 @@
       </c>
       <c r="P87" s="25" t="n"/>
       <c r="Q87" s="26" t="n"/>
+      <c r="R87" s="26" t="n"/>
+      <c r="S87" s="26" t="n"/>
     </row>
     <row r="88" ht="26" customHeight="1">
       <c r="A88" s="18" t="n">
@@ -5382,6 +5634,8 @@
       </c>
       <c r="P88" s="25" t="n"/>
       <c r="Q88" s="26" t="n"/>
+      <c r="R88" s="26" t="n"/>
+      <c r="S88" s="26" t="n"/>
     </row>
     <row r="89" ht="26" customHeight="1">
       <c r="A89" s="18" t="n">
@@ -5429,6 +5683,8 @@
       </c>
       <c r="P89" s="25" t="n"/>
       <c r="Q89" s="26" t="n"/>
+      <c r="R89" s="26" t="n"/>
+      <c r="S89" s="26" t="n"/>
     </row>
     <row r="90" ht="26" customHeight="1">
       <c r="A90" s="18" t="n">
@@ -5476,6 +5732,8 @@
       </c>
       <c r="P90" s="25" t="n"/>
       <c r="Q90" s="26" t="n"/>
+      <c r="R90" s="26" t="n"/>
+      <c r="S90" s="26" t="n"/>
     </row>
     <row r="91" ht="26" customHeight="1">
       <c r="A91" s="18" t="n">
@@ -5523,6 +5781,8 @@
       </c>
       <c r="P91" s="25" t="n"/>
       <c r="Q91" s="26" t="n"/>
+      <c r="R91" s="26" t="n"/>
+      <c r="S91" s="26" t="n"/>
     </row>
     <row r="92" ht="26" customHeight="1">
       <c r="A92" s="18" t="n">
@@ -5570,6 +5830,8 @@
       </c>
       <c r="P92" s="25" t="n"/>
       <c r="Q92" s="26" t="n"/>
+      <c r="R92" s="26" t="n"/>
+      <c r="S92" s="26" t="n"/>
     </row>
     <row r="93" ht="26" customHeight="1">
       <c r="A93" s="18" t="n">
@@ -5617,6 +5879,8 @@
       </c>
       <c r="P93" s="25" t="n"/>
       <c r="Q93" s="26" t="n"/>
+      <c r="R93" s="26" t="n"/>
+      <c r="S93" s="26" t="n"/>
     </row>
     <row r="94" ht="26" customHeight="1">
       <c r="A94" s="18" t="n">
@@ -5664,6 +5928,8 @@
       </c>
       <c r="P94" s="25" t="n"/>
       <c r="Q94" s="26" t="n"/>
+      <c r="R94" s="26" t="n"/>
+      <c r="S94" s="26" t="n"/>
     </row>
     <row r="95" ht="26" customHeight="1">
       <c r="A95" s="18" t="n">
@@ -5711,6 +5977,8 @@
       </c>
       <c r="P95" s="25" t="n"/>
       <c r="Q95" s="26" t="n"/>
+      <c r="R95" s="26" t="n"/>
+      <c r="S95" s="26" t="n"/>
     </row>
     <row r="96" ht="26" customHeight="1">
       <c r="A96" s="18" t="n">
@@ -5758,6 +6026,8 @@
       </c>
       <c r="P96" s="25" t="n"/>
       <c r="Q96" s="26" t="n"/>
+      <c r="R96" s="26" t="n"/>
+      <c r="S96" s="26" t="n"/>
     </row>
     <row r="97" ht="26" customHeight="1">
       <c r="A97" s="18" t="n">
@@ -5805,6 +6075,8 @@
       </c>
       <c r="P97" s="25" t="n"/>
       <c r="Q97" s="26" t="n"/>
+      <c r="R97" s="26" t="n"/>
+      <c r="S97" s="26" t="n"/>
     </row>
     <row r="98" ht="26" customHeight="1">
       <c r="A98" s="18" t="n">
@@ -5852,6 +6124,8 @@
       </c>
       <c r="P98" s="25" t="n"/>
       <c r="Q98" s="26" t="n"/>
+      <c r="R98" s="26" t="n"/>
+      <c r="S98" s="26" t="n"/>
     </row>
     <row r="99" ht="26" customHeight="1">
       <c r="A99" s="18" t="n">
@@ -5899,6 +6173,8 @@
       </c>
       <c r="P99" s="25" t="n"/>
       <c r="Q99" s="26" t="n"/>
+      <c r="R99" s="26" t="n"/>
+      <c r="S99" s="26" t="n"/>
     </row>
     <row r="100" ht="26" customHeight="1">
       <c r="A100" s="18" t="n">
@@ -5946,6 +6222,8 @@
       </c>
       <c r="P100" s="25" t="n"/>
       <c r="Q100" s="26" t="n"/>
+      <c r="R100" s="26" t="n"/>
+      <c r="S100" s="26" t="n"/>
     </row>
     <row r="101" ht="26" customHeight="1">
       <c r="A101" s="18" t="n">
@@ -5993,6 +6271,8 @@
       </c>
       <c r="P101" s="25" t="n"/>
       <c r="Q101" s="26" t="n"/>
+      <c r="R101" s="26" t="n"/>
+      <c r="S101" s="26" t="n"/>
     </row>
     <row r="102" ht="26" customHeight="1">
       <c r="A102" s="18" t="n">
@@ -6040,9 +6320,11 @@
       </c>
       <c r="P102" s="25" t="n"/>
       <c r="Q102" s="26" t="n"/>
+      <c r="R102" s="26" t="n"/>
+      <c r="S102" s="26" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q102"/>
+  <autoFilter ref="A1:S102"/>
   <conditionalFormatting sqref="G2:M102">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Г"</formula>

</xml_diff>